<commit_message>
Remove rate calculator; shorten About into a quick overview
</commit_message>
<xml_diff>
--- a/docs/downloads/warranty-atlas.xlsx
+++ b/docs/downloads/warranty-atlas.xlsx
@@ -56,7 +56,7 @@
     <t xml:space="preserve">Audit fields: claim deadlines, chargeback windows, rate submission, manufacturer response and challenge, penalties, with quotes.</t>
   </si>
   <si>
-    <t xml:space="preserve">Rate sample rules: what the rate calculator applies for each state.</t>
+    <t xml:space="preserve">Rate sample rules: each state's retail-rate sample, RO age limit and exclusions.</t>
   </si>
   <si>
     <t xml:space="preserve">Law dates: last amendment, amending act, original enactment, next scheduled change.</t>
@@ -5543,7 +5543,7 @@
     <t xml:space="preserve">Resubmission frequency</t>
   </si>
   <si>
-    <t xml:space="preserve">Calculator note</t>
+    <t xml:space="preserve">Note</t>
   </si>
   <si>
     <t xml:space="preserve">no statutory labor sample</t>

</xml_diff>

<commit_message>
Redesign: States home table and state overview pages; matrix moved to Research detail
</commit_message>
<xml_diff>
--- a/docs/downloads/warranty-atlas.xlsx
+++ b/docs/downloads/warranty-atlas.xlsx
@@ -5645,7 +5645,7 @@
     <t xml:space="preserve">DISCOUNT; OTHER; MAINT; RECON; ACCESS; BODY; INSURANCE; INSPECT; GOODWILL; GOVT; TIRES; ALIGN; INTERNAL</t>
   </si>
   <si>
-    <t xml:space="preserve">New Jersey also allows an optional average retail labor-time multiplier (customer-billed hours ÷ OEM hours). Supply OEM hours to see it.</t>
+    <t xml:space="preserve">New Jersey also allows an optional labor-time multiplier: customer-billed hours ÷ OEM hours for the same sampled repairs, applied to OEM warranty times.</t>
   </si>
   <si>
     <t xml:space="preserve">OTHER; TIRES; MAINT; RECON</t>
@@ -5690,7 +5690,7 @@
     <t xml:space="preserve">MAINT; WARRANTY</t>
   </si>
   <si>
-    <t xml:space="preserve">Wisconsin divides customer labor charges by the hours the manufacturer's warranty time allowances would allow for the same repairs. Supply OEM hours for each RO.</t>
+    <t xml:space="preserve">Wisconsin divides customer labor charges by the hours the manufacturer's warranty time allowances would allow for the same repairs, so each sampled RO needs its OEM hours.</t>
   </si>
   <si>
     <t xml:space="preserve">DISCOUNT; INTERNAL; MAINT; ACCESS; RECON; INSPECT; BODY; WARRANTY; OTHER</t>

</xml_diff>

<commit_message>
News: law and industry-commentary streams with a published source list; Update log summary for 2026-09-28
</commit_message>
<xml_diff>
--- a/docs/downloads/warranty-atlas.xlsx
+++ b/docs/downloads/warranty-atlas.xlsx
@@ -25,7 +25,7 @@
     <definedName function="false" hidden="true" localSheetId="8" name="_xlnm._FilterDatabase" vbProcedure="false">'Audit procedures'!$A$1:$X$51</definedName>
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Coverage!$A$1:$L$201</definedName>
     <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">'Law dates'!$A$1:$M$51</definedName>
-    <definedName function="false" hidden="true" localSheetId="7" name="_xlnm._FilterDatabase" vbProcedure="false">News!$A$1:$I$4</definedName>
+    <definedName function="false" hidden="true" localSheetId="7" name="_xlnm._FilterDatabase" vbProcedure="false">News!$A$1:$J$6</definedName>
     <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">'Rate sample rules'!$A$1:$L$51</definedName>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Summary!$A$1:$R$51</definedName>
     <definedName function="false" hidden="true" localSheetId="6" name="_xlnm._FilterDatabase" vbProcedure="false">'Weekly log'!$A$1:$J$17</definedName>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6631" uniqueCount="2482">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6654" uniqueCount="2496">
   <si>
     <t xml:space="preserve">Warranty Atlas · workpaper export</t>
   </si>
@@ -6504,6 +6504,9 @@
     <t xml:space="preserve">Week of</t>
   </si>
   <si>
+    <t xml:space="preserve">Type</t>
+  </si>
+  <si>
     <t xml:space="preserve">Date</t>
   </si>
   <si>
@@ -6525,9 +6528,54 @@
     <t xml:space="preserve">URL</t>
   </si>
   <si>
+    <t xml:space="preserve">Industry commentary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mid-Year U.S. Auto Warranty Expenses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Warranty Week</t>
+  </si>
+  <si>
+    <t xml:space="preserve">independent industry newsletter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">neutral</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Industry cost context for warranty audit planning: the report ties rising claims to higher parts and labor costs (including retail-rate reimbursement), complex electronics and large recalls, and calls elevated warranty costs "the new normal". Useful benchmark when explaining warranty expense trends.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.warrantyweek.com/archive/ww20260908.html</t>
+  </si>
+  <si>
     <t xml:space="preserve">2026-09-21</t>
   </si>
   <si>
+    <t xml:space="preserve">Why Every Dealership Acquisition Should Begin with a Retail Warranty Reimbursement Review</t>
+  </si>
+  <si>
+    <t xml:space="preserve">California New Car Dealer Quarterly (CNCDA); author: Jordan Jankowski, COO, Armatus Dealer Uplift</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dealer association magazine (vendor author)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dealer-side</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Signals where dealer-side vendors are steering buyers: expect retail-rate submissions soon after buy-sells. Rate submissions tied to ownership changes may deserve a closer look against the state's RO-sample rules.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://california-new-car-dealer.thenewslinkgroup.org/why-every-dealership-acquisition-should-begin-with-a-retail-warranty-reimbursement-review/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Law or ruling</t>
+  </si>
+  <si>
     <t xml:space="preserve">2026-09-18</t>
   </si>
   <si>
@@ -6540,9 +6588,6 @@
     <t xml:space="preserve">government</t>
   </si>
   <si>
-    <t xml:space="preserve">neutral</t>
-  </si>
-  <si>
     <t xml:space="preserve">From 10/1/2026 Subaru's recall and warranty claim systems must accept and pay Connecticut used-inventory stop-sale claims on the 30-day/1-year-audit timetable, and may not claw these payments back through chargebacks or incentive programs unless the action applies uniformly to every same-line-make dealer in the state.</t>
   </si>
   <si>
@@ -6559,9 +6604,6 @@
   </si>
   <si>
     <t xml:space="preserve">dealer association</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dealer-side</t>
   </si>
   <si>
     <t xml:space="preserve">This is the first board ruling that recovering statutory warranty uplift through per-vehicle or parts-account debits is an illegal surcharge. Subaru should confirm that nothing in its Illinois pricing or charge structure is tied to warranty reimbursement, and should watch for the same argument under other anti-cost-recovery statutes, such as RI § 31-5.1-6(g).</t>
@@ -8091,58 +8133,58 @@
         <v>19</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>2439</v>
+        <v>2453</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>2440</v>
+        <v>2454</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>2441</v>
+        <v>2455</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>2442</v>
+        <v>2456</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>2443</v>
+        <v>2457</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>2444</v>
+        <v>2458</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>2445</v>
+        <v>2459</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>2446</v>
+        <v>2460</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>2447</v>
+        <v>2461</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>2448</v>
+        <v>2462</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>2449</v>
+        <v>2463</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>2450</v>
+        <v>2464</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>2451</v>
+        <v>2465</v>
       </c>
       <c r="P1" s="4" t="s">
-        <v>2452</v>
+        <v>2466</v>
       </c>
       <c r="Q1" s="4" t="s">
-        <v>2453</v>
+        <v>2467</v>
       </c>
       <c r="R1" s="4" t="s">
-        <v>2454</v>
+        <v>2468</v>
       </c>
       <c r="S1" s="4" t="s">
-        <v>2455</v>
+        <v>2469</v>
       </c>
       <c r="T1" s="4" t="s">
-        <v>2456</v>
+        <v>2470</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8156,7 +8198,7 @@
         <v>10</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>2457</v>
+        <v>2471</v>
       </c>
       <c r="E2" s="6" t="n">
         <v>44</v>
@@ -8216,7 +8258,7 @@
         <v>25</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>2458</v>
+        <v>2472</v>
       </c>
       <c r="E3" s="6" t="n">
         <v>31</v>
@@ -8276,7 +8318,7 @@
         <v>30</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>2459</v>
+        <v>2473</v>
       </c>
       <c r="E4" s="6" t="n">
         <v>22</v>
@@ -8336,7 +8378,7 @@
         <v>30</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>2459</v>
+        <v>2473</v>
       </c>
       <c r="E5" s="6" t="n">
         <v>23</v>
@@ -8396,7 +8438,7 @@
         <v>75</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>2460</v>
+        <v>2474</v>
       </c>
       <c r="E6" s="6" t="n">
         <v>1</v>
@@ -8456,7 +8498,7 @@
         <v>35</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>2459</v>
+        <v>2473</v>
       </c>
       <c r="E7" s="6" t="n">
         <v>13</v>
@@ -8516,7 +8558,7 @@
         <v>20</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>2458</v>
+        <v>2472</v>
       </c>
       <c r="E8" s="6" t="n">
         <v>38</v>
@@ -8564,7 +8606,7 @@
         <v>0</v>
       </c>
       <c r="T8" s="6" t="s">
-        <v>2461</v>
+        <v>2475</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8578,7 +8620,7 @@
         <v>30</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>2459</v>
+        <v>2473</v>
       </c>
       <c r="E9" s="6" t="n">
         <v>24</v>
@@ -8638,7 +8680,7 @@
         <v>70</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>2460</v>
+        <v>2474</v>
       </c>
       <c r="E10" s="6" t="n">
         <v>2</v>
@@ -8698,7 +8740,7 @@
         <v>40</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>2462</v>
+        <v>2476</v>
       </c>
       <c r="E11" s="6" t="n">
         <v>7</v>
@@ -8758,7 +8800,7 @@
         <v>35</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>2459</v>
+        <v>2473</v>
       </c>
       <c r="E12" s="6" t="n">
         <v>14</v>
@@ -8806,7 +8848,7 @@
         <v>0</v>
       </c>
       <c r="T12" s="6" t="s">
-        <v>2463</v>
+        <v>2477</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8820,7 +8862,7 @@
         <v>25</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>2458</v>
+        <v>2472</v>
       </c>
       <c r="E13" s="6" t="n">
         <v>32</v>
@@ -8880,7 +8922,7 @@
         <v>25</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>2458</v>
+        <v>2472</v>
       </c>
       <c r="E14" s="6" t="n">
         <v>33</v>
@@ -8940,7 +8982,7 @@
         <v>25</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>2458</v>
+        <v>2472</v>
       </c>
       <c r="E15" s="6" t="n">
         <v>34</v>
@@ -9000,7 +9042,7 @@
         <v>35</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>2459</v>
+        <v>2473</v>
       </c>
       <c r="E16" s="6" t="n">
         <v>15</v>
@@ -9060,7 +9102,7 @@
         <v>40</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>2462</v>
+        <v>2476</v>
       </c>
       <c r="E17" s="6" t="n">
         <v>8</v>
@@ -9120,7 +9162,7 @@
         <v>30</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>2459</v>
+        <v>2473</v>
       </c>
       <c r="E18" s="6" t="n">
         <v>25</v>
@@ -9180,7 +9222,7 @@
         <v>30</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>2459</v>
+        <v>2473</v>
       </c>
       <c r="E19" s="6" t="n">
         <v>26</v>
@@ -9240,7 +9282,7 @@
         <v>40</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>2462</v>
+        <v>2476</v>
       </c>
       <c r="E20" s="6" t="n">
         <v>9</v>
@@ -9288,7 +9330,7 @@
         <v>5</v>
       </c>
       <c r="T20" s="6" t="s">
-        <v>2461</v>
+        <v>2475</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9302,7 +9344,7 @@
         <v>30</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>2459</v>
+        <v>2473</v>
       </c>
       <c r="E21" s="6" t="n">
         <v>27</v>
@@ -9362,7 +9404,7 @@
         <v>15</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>2457</v>
+        <v>2471</v>
       </c>
       <c r="E22" s="6" t="n">
         <v>43</v>
@@ -9410,7 +9452,7 @@
         <v>0</v>
       </c>
       <c r="T22" s="6" t="s">
-        <v>2461</v>
+        <v>2475</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9424,7 +9466,7 @@
         <v>35</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>2459</v>
+        <v>2473</v>
       </c>
       <c r="E23" s="6" t="n">
         <v>16</v>
@@ -9484,7 +9526,7 @@
         <v>20</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>2458</v>
+        <v>2472</v>
       </c>
       <c r="E24" s="6" t="n">
         <v>39</v>
@@ -9544,7 +9586,7 @@
         <v>35</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>2459</v>
+        <v>2473</v>
       </c>
       <c r="E25" s="6" t="n">
         <v>17</v>
@@ -9604,7 +9646,7 @@
         <v>20</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>2458</v>
+        <v>2472</v>
       </c>
       <c r="E26" s="6" t="n">
         <v>40</v>
@@ -9664,7 +9706,7 @@
         <v>30</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>2459</v>
+        <v>2473</v>
       </c>
       <c r="E27" s="6" t="n">
         <v>28</v>
@@ -9724,7 +9766,7 @@
         <v>55</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>2460</v>
+        <v>2474</v>
       </c>
       <c r="E28" s="6" t="n">
         <v>4</v>
@@ -9784,7 +9826,7 @@
         <v>10</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>2457</v>
+        <v>2471</v>
       </c>
       <c r="E29" s="6" t="n">
         <v>45</v>
@@ -9844,7 +9886,7 @@
         <v>35</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>2459</v>
+        <v>2473</v>
       </c>
       <c r="E30" s="6" t="n">
         <v>18</v>
@@ -9904,7 +9946,7 @@
         <v>40</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>2462</v>
+        <v>2476</v>
       </c>
       <c r="E31" s="6" t="n">
         <v>10</v>
@@ -9952,7 +9994,7 @@
         <v>0</v>
       </c>
       <c r="T31" s="6" t="s">
-        <v>2461</v>
+        <v>2475</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9966,7 +10008,7 @@
         <v>50</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>2460</v>
+        <v>2474</v>
       </c>
       <c r="E32" s="6" t="n">
         <v>5</v>
@@ -10014,7 +10056,7 @@
         <v>0</v>
       </c>
       <c r="T32" s="6" t="s">
-        <v>2464</v>
+        <v>2478</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10028,7 +10070,7 @@
         <v>35</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>2459</v>
+        <v>2473</v>
       </c>
       <c r="E33" s="6" t="n">
         <v>19</v>
@@ -10088,7 +10130,7 @@
         <v>35</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>2459</v>
+        <v>2473</v>
       </c>
       <c r="E34" s="6" t="n">
         <v>20</v>
@@ -10148,7 +10190,7 @@
         <v>40</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>2462</v>
+        <v>2476</v>
       </c>
       <c r="E35" s="6" t="n">
         <v>11</v>
@@ -10196,7 +10238,7 @@
         <v>0</v>
       </c>
       <c r="T35" s="6" t="s">
-        <v>2465</v>
+        <v>2479</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10210,7 +10252,7 @@
         <v>40</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>2462</v>
+        <v>2476</v>
       </c>
       <c r="E36" s="6" t="n">
         <v>12</v>
@@ -10270,7 +10312,7 @@
         <v>30</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>2459</v>
+        <v>2473</v>
       </c>
       <c r="E37" s="6" t="n">
         <v>29</v>
@@ -10330,7 +10372,7 @@
         <v>25</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>2458</v>
+        <v>2472</v>
       </c>
       <c r="E38" s="6" t="n">
         <v>35</v>
@@ -10390,7 +10432,7 @@
         <v>35</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>2459</v>
+        <v>2473</v>
       </c>
       <c r="E39" s="6" t="n">
         <v>21</v>
@@ -10450,7 +10492,7 @@
         <v>20</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>2458</v>
+        <v>2472</v>
       </c>
       <c r="E40" s="6" t="n">
         <v>41</v>
@@ -10498,7 +10540,7 @@
         <v>0</v>
       </c>
       <c r="T40" s="6" t="s">
-        <v>2461</v>
+        <v>2475</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10512,7 +10554,7 @@
         <v>25</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>2458</v>
+        <v>2472</v>
       </c>
       <c r="E41" s="6" t="n">
         <v>36</v>
@@ -10572,7 +10614,7 @@
         <v>20</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>2458</v>
+        <v>2472</v>
       </c>
       <c r="E42" s="6" t="n">
         <v>42</v>
@@ -10632,7 +10674,7 @@
         <v>0</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>2457</v>
+        <v>2471</v>
       </c>
       <c r="E43" s="6" t="n">
         <v>50</v>
@@ -10692,7 +10734,7 @@
         <v>10</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>2457</v>
+        <v>2471</v>
       </c>
       <c r="E44" s="6" t="n">
         <v>46</v>
@@ -10752,7 +10794,7 @@
         <v>65</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>2460</v>
+        <v>2474</v>
       </c>
       <c r="E45" s="6" t="n">
         <v>3</v>
@@ -10812,7 +10854,7 @@
         <v>45</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>2462</v>
+        <v>2476</v>
       </c>
       <c r="E46" s="6" t="n">
         <v>6</v>
@@ -10872,7 +10914,7 @@
         <v>25</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>2458</v>
+        <v>2472</v>
       </c>
       <c r="E47" s="6" t="n">
         <v>37</v>
@@ -10920,7 +10962,7 @@
         <v>0</v>
       </c>
       <c r="T47" s="6" t="s">
-        <v>2461</v>
+        <v>2475</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10934,7 +10976,7 @@
         <v>10</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>2457</v>
+        <v>2471</v>
       </c>
       <c r="E48" s="6" t="n">
         <v>47</v>
@@ -10994,7 +11036,7 @@
         <v>5</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>2457</v>
+        <v>2471</v>
       </c>
       <c r="E49" s="6" t="n">
         <v>48</v>
@@ -11054,7 +11096,7 @@
         <v>30</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>2459</v>
+        <v>2473</v>
       </c>
       <c r="E50" s="6" t="n">
         <v>30</v>
@@ -11114,7 +11156,7 @@
         <v>5</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>2457</v>
+        <v>2471</v>
       </c>
       <c r="E51" s="6" t="n">
         <v>49</v>
@@ -11165,82 +11207,82 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="5" t="s">
-        <v>2466</v>
+        <v>2480</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="s">
-        <v>2467</v>
+        <v>2481</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="s">
-        <v>2468</v>
+        <v>2482</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="s">
-        <v>2469</v>
+        <v>2483</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="s">
-        <v>2470</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="s">
-        <v>2471</v>
+        <v>2485</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="7" t="s">
-        <v>2472</v>
+        <v>2486</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="7" t="s">
-        <v>2473</v>
+        <v>2487</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="7" t="s">
-        <v>2474</v>
+        <v>2488</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="7" t="s">
-        <v>2475</v>
+        <v>2489</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="7" t="s">
-        <v>2476</v>
+        <v>2490</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="s">
-        <v>2477</v>
+        <v>2491</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="7" t="s">
-        <v>2478</v>
+        <v>2492</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="7" t="s">
-        <v>2479</v>
+        <v>2493</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="7" t="s">
-        <v>2480</v>
+        <v>2494</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="7" t="s">
-        <v>2481</v>
+        <v>2495</v>
       </c>
     </row>
   </sheetData>
@@ -31075,16 +31117,18 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="60"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="40"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -31101,10 +31145,10 @@
         <v>2156</v>
       </c>
       <c r="E1" s="4" t="s">
+        <v>2157</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>262</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>2157</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>2158</v>
@@ -31115,10 +31159,13 @@
       <c r="I1" s="4" t="s">
         <v>2160</v>
       </c>
+      <c r="J1" s="4" t="s">
+        <v>2161</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>2161</v>
+        <v>2085</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>2162</v>
@@ -31136,21 +31183,22 @@
         <v>2166</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="H2" s="6" t="s">
         <v>2167</v>
       </c>
+      <c r="H2" s="6"/>
       <c r="I2" s="6" t="s">
         <v>2168</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J2" s="6" t="s">
+        <v>2169</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>2161</v>
+        <v>2085</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>2169</v>
+        <v>2162</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>2170</v>
@@ -31165,46 +31213,116 @@
         <v>2173</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>113</v>
+        <v>2174</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>2174</v>
+        <v>68</v>
       </c>
       <c r="I3" s="6" t="s">
         <v>2175</v>
       </c>
+      <c r="J3" s="6" t="s">
+        <v>2176</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>2161</v>
+        <v>2170</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>2176</v>
+        <v>2177</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>2177</v>
+        <v>2178</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>2178</v>
+        <v>2179</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>2179</v>
+        <v>2180</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>2180</v>
+        <v>2181</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>209</v>
+        <v>2167</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>2181</v>
+        <v>79</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>2182</v>
       </c>
+      <c r="J4" s="6" t="s">
+        <v>2183</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
+        <v>2170</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>2177</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>2184</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>2185</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>2186</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>2187</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>2174</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>2188</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>2189</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
+        <v>2170</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>2177</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>2190</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>2191</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>2192</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>2193</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>2194</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>2195</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>2196</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I4"/>
+  <autoFilter ref="A1:J6"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -31256,67 +31374,67 @@
         <v>19</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>2183</v>
+        <v>2197</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>2184</v>
+        <v>2198</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>2185</v>
+        <v>2199</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>2186</v>
+        <v>2200</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>2187</v>
+        <v>2201</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>2188</v>
+        <v>2202</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>2189</v>
+        <v>2203</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>2190</v>
+        <v>2204</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>2191</v>
+        <v>2205</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>2192</v>
+        <v>2206</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>2193</v>
+        <v>2207</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>2194</v>
+        <v>2208</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>2195</v>
+        <v>2209</v>
       </c>
       <c r="P1" s="4" t="s">
-        <v>2196</v>
+        <v>2210</v>
       </c>
       <c r="Q1" s="4" t="s">
-        <v>2197</v>
+        <v>2211</v>
       </c>
       <c r="R1" s="4" t="s">
-        <v>2198</v>
+        <v>2212</v>
       </c>
       <c r="S1" s="4" t="s">
-        <v>2199</v>
+        <v>2213</v>
       </c>
       <c r="T1" s="4" t="s">
-        <v>2200</v>
+        <v>2214</v>
       </c>
       <c r="U1" s="4" t="s">
-        <v>2201</v>
+        <v>2215</v>
       </c>
       <c r="V1" s="4" t="s">
         <v>35</v>
       </c>
       <c r="W1" s="4" t="s">
-        <v>2202</v>
+        <v>2216</v>
       </c>
       <c r="X1" s="4" t="s">
         <v>715</v>
@@ -31330,42 +31448,42 @@
         <v>38</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D2" s="6"/>
       <c r="E2" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>2204</v>
+        <v>2218</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>2205</v>
+        <v>2219</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I2" s="6"/>
       <c r="J2" s="6" t="s">
-        <v>2206</v>
+        <v>2220</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="M2" s="6" t="s">
-        <v>2204</v>
+        <v>2218</v>
       </c>
       <c r="N2" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O2" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="P2" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="Q2" s="6" t="s">
         <v>42</v>
@@ -31374,10 +31492,10 @@
         <v>42</v>
       </c>
       <c r="S2" s="6" t="s">
-        <v>2208</v>
+        <v>2222</v>
       </c>
       <c r="T2" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U2" s="6"/>
       <c r="V2" s="6" t="s">
@@ -31387,7 +31505,7 @@
         <v>740</v>
       </c>
       <c r="X2" s="6" t="s">
-        <v>2210</v>
+        <v>2224</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31398,34 +31516,34 @@
         <v>50</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>2204</v>
+        <v>2218</v>
       </c>
       <c r="G3" s="6"/>
       <c r="H3" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I3" s="6"/>
       <c r="J3" s="6" t="s">
-        <v>2211</v>
+        <v>2225</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L3" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="M3" s="6" t="s">
-        <v>2204</v>
+        <v>2218</v>
       </c>
       <c r="N3" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O3" s="6" t="s">
         <v>42</v>
@@ -31440,20 +31558,20 @@
         <v>42</v>
       </c>
       <c r="S3" s="6" t="s">
-        <v>2212</v>
+        <v>2226</v>
       </c>
       <c r="T3" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U3" s="6"/>
       <c r="V3" s="6" t="s">
         <v>47</v>
       </c>
       <c r="W3" s="6" t="s">
-        <v>2213</v>
+        <v>2227</v>
       </c>
       <c r="X3" s="6" t="s">
-        <v>2214</v>
+        <v>2228</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="236.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31464,40 +31582,40 @@
         <v>58</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>2204</v>
+        <v>2218</v>
       </c>
       <c r="G4" s="6"/>
       <c r="H4" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I4" s="6"/>
       <c r="J4" s="6" t="s">
-        <v>2215</v>
+        <v>2229</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L4" s="6" t="s">
         <v>42</v>
       </c>
       <c r="M4" s="6" t="s">
-        <v>2216</v>
+        <v>2230</v>
       </c>
       <c r="N4" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O4" s="6" t="s">
         <v>42</v>
       </c>
       <c r="P4" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="Q4" s="6" t="s">
         <v>42</v>
@@ -31506,22 +31624,22 @@
         <v>42</v>
       </c>
       <c r="S4" s="6" t="s">
-        <v>2217</v>
+        <v>2231</v>
       </c>
       <c r="T4" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U4" s="6" t="s">
-        <v>2218</v>
+        <v>2232</v>
       </c>
       <c r="V4" s="6" t="s">
         <v>61</v>
       </c>
       <c r="W4" s="6" t="s">
-        <v>2219</v>
+        <v>2233</v>
       </c>
       <c r="X4" s="6" t="s">
-        <v>2220</v>
+        <v>2234</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31532,40 +31650,40 @@
         <v>64</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D5" s="6"/>
       <c r="E5" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>2204</v>
+        <v>2218</v>
       </c>
       <c r="G5" s="6"/>
       <c r="H5" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I5" s="6"/>
       <c r="J5" s="6" t="s">
-        <v>2221</v>
+        <v>2235</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L5" s="6" t="s">
         <v>42</v>
       </c>
       <c r="M5" s="6" t="s">
-        <v>2222</v>
+        <v>2236</v>
       </c>
       <c r="N5" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O5" s="6" t="s">
         <v>42</v>
       </c>
       <c r="P5" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="Q5" s="6" t="s">
         <v>42</v>
@@ -31574,10 +31692,10 @@
         <v>42</v>
       </c>
       <c r="S5" s="6" t="s">
+        <v>2237</v>
+      </c>
+      <c r="T5" s="6" t="s">
         <v>2223</v>
-      </c>
-      <c r="T5" s="6" t="s">
-        <v>2209</v>
       </c>
       <c r="U5" s="6"/>
       <c r="V5" s="6" t="s">
@@ -31587,7 +31705,7 @@
         <v>299</v>
       </c>
       <c r="X5" s="6" t="s">
-        <v>2224</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="169.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31605,10 +31723,10 @@
         <v>42</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>2225</v>
+        <v>2239</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>2226</v>
+        <v>2240</v>
       </c>
       <c r="H6" s="6" t="s">
         <v>42</v>
@@ -31617,7 +31735,7 @@
         <v>30</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>2227</v>
+        <v>2241</v>
       </c>
       <c r="K6" s="6" t="s">
         <v>42</v>
@@ -31626,10 +31744,10 @@
         <v>42</v>
       </c>
       <c r="M6" s="6" t="s">
-        <v>2228</v>
+        <v>2242</v>
       </c>
       <c r="N6" s="6" t="s">
-        <v>2229</v>
+        <v>2243</v>
       </c>
       <c r="O6" s="6" t="s">
         <v>42</v>
@@ -31644,22 +31762,22 @@
         <v>42</v>
       </c>
       <c r="S6" s="6" t="s">
-        <v>2230</v>
+        <v>2244</v>
       </c>
       <c r="T6" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U6" s="6" t="s">
-        <v>2231</v>
+        <v>2245</v>
       </c>
       <c r="V6" s="6" t="s">
         <v>47</v>
       </c>
       <c r="W6" s="6" t="s">
-        <v>2232</v>
+        <v>2246</v>
       </c>
       <c r="X6" s="6" t="s">
-        <v>2233</v>
+        <v>2247</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31670,37 +31788,37 @@
         <v>74</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D7" s="6"/>
       <c r="E7" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>2204</v>
+        <v>2218</v>
       </c>
       <c r="G7" s="6"/>
       <c r="H7" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I7" s="6"/>
       <c r="J7" s="6" t="s">
-        <v>2234</v>
+        <v>2248</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L7" s="6" t="s">
         <v>42</v>
       </c>
       <c r="M7" s="6" t="s">
-        <v>2235</v>
+        <v>2249</v>
       </c>
       <c r="N7" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O7" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="P7" s="6" t="s">
         <v>42</v>
@@ -31712,22 +31830,22 @@
         <v>42</v>
       </c>
       <c r="S7" s="6" t="s">
-        <v>2236</v>
+        <v>2250</v>
       </c>
       <c r="T7" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U7" s="6" t="s">
-        <v>2237</v>
+        <v>2251</v>
       </c>
       <c r="V7" s="6" t="s">
         <v>47</v>
       </c>
       <c r="W7" s="6" t="s">
-        <v>2238</v>
+        <v>2252</v>
       </c>
       <c r="X7" s="6" t="s">
-        <v>2239</v>
+        <v>2253</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31738,42 +31856,42 @@
         <v>80</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D8" s="6"/>
       <c r="E8" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>2204</v>
+        <v>2218</v>
       </c>
       <c r="G8" s="6"/>
       <c r="H8" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I8" s="6" t="n">
         <v>30</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>2240</v>
+        <v>2254</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L8" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="M8" s="6" t="s">
-        <v>2204</v>
+        <v>2218</v>
       </c>
       <c r="N8" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O8" s="6" t="s">
         <v>42</v>
       </c>
       <c r="P8" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="Q8" s="6" t="s">
         <v>42</v>
@@ -31782,20 +31900,20 @@
         <v>42</v>
       </c>
       <c r="S8" s="6" t="s">
-        <v>2241</v>
+        <v>2255</v>
       </c>
       <c r="T8" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U8" s="6"/>
       <c r="V8" s="6" t="s">
         <v>47</v>
       </c>
       <c r="W8" s="6" t="s">
-        <v>2242</v>
+        <v>2256</v>
       </c>
       <c r="X8" s="6" t="s">
-        <v>2243</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31806,34 +31924,34 @@
         <v>87</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D9" s="6"/>
       <c r="E9" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>2204</v>
+        <v>2218</v>
       </c>
       <c r="G9" s="6"/>
       <c r="H9" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I9" s="6"/>
       <c r="J9" s="6" t="s">
-        <v>2204</v>
+        <v>2218</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L9" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="M9" s="6" t="s">
-        <v>2204</v>
+        <v>2218</v>
       </c>
       <c r="N9" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O9" s="6" t="s">
         <v>42</v>
@@ -31848,10 +31966,10 @@
         <v>42</v>
       </c>
       <c r="S9" s="6" t="s">
-        <v>2244</v>
+        <v>2258</v>
       </c>
       <c r="T9" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U9" s="6"/>
       <c r="V9" s="6" t="s">
@@ -31861,7 +31979,7 @@
         <v>907</v>
       </c>
       <c r="X9" s="6" t="s">
-        <v>2245</v>
+        <v>2259</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31872,17 +31990,17 @@
         <v>92</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D10" s="6"/>
       <c r="E10" s="6" t="s">
         <v>42</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>2246</v>
+        <v>2260</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>2247</v>
+        <v>2261</v>
       </c>
       <c r="H10" s="6" t="s">
         <v>42</v>
@@ -31891,19 +32009,19 @@
         <v>45</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>2248</v>
+        <v>2262</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L10" s="6" t="s">
         <v>42</v>
       </c>
       <c r="M10" s="6" t="s">
-        <v>2249</v>
+        <v>2263</v>
       </c>
       <c r="N10" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O10" s="6" t="s">
         <v>42</v>
@@ -31918,22 +32036,22 @@
         <v>42</v>
       </c>
       <c r="S10" s="6" t="s">
-        <v>2250</v>
+        <v>2264</v>
       </c>
       <c r="T10" s="6" t="s">
-        <v>2251</v>
+        <v>2265</v>
       </c>
       <c r="U10" s="6" t="s">
-        <v>2252</v>
+        <v>2266</v>
       </c>
       <c r="V10" s="6" t="s">
         <v>47</v>
       </c>
       <c r="W10" s="6" t="s">
-        <v>2253</v>
+        <v>2267</v>
       </c>
       <c r="X10" s="6" t="s">
-        <v>2254</v>
+        <v>2268</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31944,36 +32062,36 @@
         <v>97</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D11" s="6"/>
       <c r="E11" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>2204</v>
+        <v>2218</v>
       </c>
       <c r="G11" s="6"/>
       <c r="H11" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I11" s="6" t="n">
         <v>30</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>2255</v>
+        <v>2269</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L11" s="6" t="s">
         <v>42</v>
       </c>
       <c r="M11" s="6" t="s">
-        <v>2256</v>
+        <v>2270</v>
       </c>
       <c r="N11" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O11" s="6" t="s">
         <v>42</v>
@@ -31988,22 +32106,22 @@
         <v>42</v>
       </c>
       <c r="S11" s="6" t="s">
-        <v>2257</v>
+        <v>2271</v>
       </c>
       <c r="T11" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U11" s="6" t="s">
-        <v>2258</v>
+        <v>2272</v>
       </c>
       <c r="V11" s="6" t="s">
         <v>47</v>
       </c>
       <c r="W11" s="6" t="s">
-        <v>2259</v>
+        <v>2273</v>
       </c>
       <c r="X11" s="6" t="s">
-        <v>2260</v>
+        <v>2274</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32014,14 +32132,14 @@
         <v>102</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>2204</v>
+        <v>2218</v>
       </c>
       <c r="G12" s="6"/>
       <c r="H12" s="6" t="s">
@@ -32031,22 +32149,22 @@
         <v>30</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>2261</v>
+        <v>2275</v>
       </c>
       <c r="K12" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L12" s="6" t="s">
         <v>42</v>
       </c>
       <c r="M12" s="6" t="s">
-        <v>2262</v>
+        <v>2276</v>
       </c>
       <c r="N12" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O12" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="P12" s="6" t="s">
         <v>42</v>
@@ -32058,22 +32176,22 @@
         <v>42</v>
       </c>
       <c r="S12" s="6" t="s">
-        <v>2263</v>
+        <v>2277</v>
       </c>
       <c r="T12" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U12" s="6" t="s">
-        <v>2264</v>
+        <v>2278</v>
       </c>
       <c r="V12" s="6" t="s">
         <v>47</v>
       </c>
       <c r="W12" s="6" t="s">
-        <v>2265</v>
+        <v>2279</v>
       </c>
       <c r="X12" s="6" t="s">
-        <v>2266</v>
+        <v>2280</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32084,30 +32202,30 @@
         <v>106</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D13" s="6"/>
       <c r="E13" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F13" s="6"/>
       <c r="G13" s="6"/>
       <c r="H13" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I13" s="6"/>
       <c r="J13" s="6" t="s">
-        <v>2267</v>
+        <v>2281</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L13" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="M13" s="6"/>
       <c r="N13" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O13" s="6" t="s">
         <v>42</v>
@@ -32122,22 +32240,22 @@
         <v>42</v>
       </c>
       <c r="S13" s="6" t="s">
-        <v>2268</v>
+        <v>2282</v>
       </c>
       <c r="T13" s="6" t="s">
-        <v>2251</v>
+        <v>2265</v>
       </c>
       <c r="U13" s="6" t="s">
-        <v>2269</v>
+        <v>2283</v>
       </c>
       <c r="V13" s="6" t="s">
         <v>47</v>
       </c>
       <c r="W13" s="6" t="s">
-        <v>2270</v>
+        <v>2284</v>
       </c>
       <c r="X13" s="6" t="s">
-        <v>2271</v>
+        <v>2285</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32148,36 +32266,36 @@
         <v>110</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>2204</v>
+        <v>2218</v>
       </c>
       <c r="G14" s="6"/>
       <c r="H14" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I14" s="6" t="n">
         <v>30</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>2272</v>
+        <v>2286</v>
       </c>
       <c r="K14" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L14" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="M14" s="6" t="s">
-        <v>2273</v>
+        <v>2287</v>
       </c>
       <c r="N14" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O14" s="6" t="s">
         <v>42</v>
@@ -32192,20 +32310,20 @@
         <v>42</v>
       </c>
       <c r="S14" s="6" t="s">
-        <v>2274</v>
+        <v>2288</v>
       </c>
       <c r="T14" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U14" s="6"/>
       <c r="V14" s="6" t="s">
         <v>47</v>
       </c>
       <c r="W14" s="6" t="s">
-        <v>2275</v>
+        <v>2289</v>
       </c>
       <c r="X14" s="6" t="s">
-        <v>2276</v>
+        <v>2290</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32216,30 +32334,30 @@
         <v>114</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D15" s="6"/>
       <c r="E15" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F15" s="6"/>
       <c r="G15" s="6"/>
       <c r="H15" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I15" s="6"/>
       <c r="J15" s="6" t="s">
-        <v>2277</v>
+        <v>2291</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L15" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="M15" s="6"/>
       <c r="N15" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O15" s="6" t="s">
         <v>42</v>
@@ -32254,20 +32372,20 @@
         <v>42</v>
       </c>
       <c r="S15" s="6" t="s">
-        <v>2278</v>
+        <v>2292</v>
       </c>
       <c r="T15" s="6" t="s">
-        <v>2251</v>
+        <v>2265</v>
       </c>
       <c r="U15" s="6"/>
       <c r="V15" s="6" t="s">
         <v>61</v>
       </c>
       <c r="W15" s="6" t="s">
-        <v>2279</v>
+        <v>2293</v>
       </c>
       <c r="X15" s="6" t="s">
-        <v>2280</v>
+        <v>2294</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="236.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32278,11 +32396,11 @@
         <v>120</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D16" s="6"/>
       <c r="E16" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F16" s="6"/>
       <c r="G16" s="6"/>
@@ -32293,19 +32411,19 @@
         <v>30</v>
       </c>
       <c r="J16" s="6" t="s">
-        <v>2281</v>
+        <v>2295</v>
       </c>
       <c r="K16" s="6" t="s">
         <v>42</v>
       </c>
       <c r="L16" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="M16" s="6" t="s">
-        <v>2282</v>
+        <v>2296</v>
       </c>
       <c r="N16" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O16" s="6" t="s">
         <v>42</v>
@@ -32320,20 +32438,20 @@
         <v>42</v>
       </c>
       <c r="S16" s="6" t="s">
-        <v>2283</v>
+        <v>2297</v>
       </c>
       <c r="T16" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U16" s="6"/>
       <c r="V16" s="6" t="s">
         <v>47</v>
       </c>
       <c r="W16" s="6" t="s">
-        <v>2284</v>
+        <v>2298</v>
       </c>
       <c r="X16" s="6" t="s">
-        <v>2285</v>
+        <v>2299</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32344,30 +32462,30 @@
         <v>124</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D17" s="6"/>
       <c r="E17" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F17" s="6"/>
       <c r="G17" s="6"/>
       <c r="H17" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I17" s="6"/>
       <c r="J17" s="6"/>
       <c r="K17" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L17" s="6" t="s">
         <v>42</v>
       </c>
       <c r="M17" s="6" t="s">
-        <v>2286</v>
+        <v>2300</v>
       </c>
       <c r="N17" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O17" s="6" t="s">
         <v>42</v>
@@ -32382,13 +32500,13 @@
         <v>42</v>
       </c>
       <c r="S17" s="6" t="s">
-        <v>2287</v>
+        <v>2301</v>
       </c>
       <c r="T17" s="6" t="s">
-        <v>2251</v>
+        <v>2265</v>
       </c>
       <c r="U17" s="6" t="s">
-        <v>2288</v>
+        <v>2302</v>
       </c>
       <c r="V17" s="6" t="s">
         <v>47</v>
@@ -32397,7 +32515,7 @@
         <v>398</v>
       </c>
       <c r="X17" s="6" t="s">
-        <v>2289</v>
+        <v>2303</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32408,11 +32526,11 @@
         <v>127</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D18" s="6"/>
       <c r="E18" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F18" s="6"/>
       <c r="G18" s="6"/>
@@ -32423,17 +32541,17 @@
         <v>5</v>
       </c>
       <c r="J18" s="6" t="s">
-        <v>2290</v>
+        <v>2304</v>
       </c>
       <c r="K18" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L18" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="M18" s="6"/>
       <c r="N18" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O18" s="6" t="s">
         <v>42</v>
@@ -32445,23 +32563,23 @@
         <v>42</v>
       </c>
       <c r="R18" s="6" t="s">
-        <v>2291</v>
+        <v>2305</v>
       </c>
       <c r="S18" s="6" t="s">
-        <v>2292</v>
+        <v>2306</v>
       </c>
       <c r="T18" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U18" s="6"/>
       <c r="V18" s="6" t="s">
         <v>47</v>
       </c>
       <c r="W18" s="6" t="s">
-        <v>2293</v>
+        <v>2307</v>
       </c>
       <c r="X18" s="6" t="s">
-        <v>2294</v>
+        <v>2308</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32472,32 +32590,32 @@
         <v>130</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D19" s="6"/>
       <c r="E19" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F19" s="6"/>
       <c r="G19" s="6" t="s">
-        <v>2295</v>
+        <v>2309</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I19" s="6"/>
       <c r="J19" s="6" t="s">
-        <v>2296</v>
+        <v>2310</v>
       </c>
       <c r="K19" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L19" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="M19" s="6"/>
       <c r="N19" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O19" s="6" t="s">
         <v>42</v>
@@ -32512,13 +32630,13 @@
         <v>42</v>
       </c>
       <c r="S19" s="6" t="s">
-        <v>2297</v>
+        <v>2311</v>
       </c>
       <c r="T19" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U19" s="6" t="s">
-        <v>2298</v>
+        <v>2312</v>
       </c>
       <c r="V19" s="6" t="s">
         <v>47</v>
@@ -32527,7 +32645,7 @@
         <v>1136</v>
       </c>
       <c r="X19" s="6" t="s">
-        <v>2299</v>
+        <v>2313</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32538,14 +32656,14 @@
         <v>134</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D20" s="6"/>
       <c r="E20" s="6" t="s">
         <v>42</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>2300</v>
+        <v>2314</v>
       </c>
       <c r="G20" s="6"/>
       <c r="H20" s="6" t="s">
@@ -32555,22 +32673,22 @@
         <v>30</v>
       </c>
       <c r="J20" s="6" t="s">
-        <v>2301</v>
+        <v>2315</v>
       </c>
       <c r="K20" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L20" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="M20" s="6" t="s">
-        <v>2302</v>
+        <v>2316</v>
       </c>
       <c r="N20" s="6" t="s">
-        <v>2229</v>
+        <v>2243</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="P20" s="6" t="s">
         <v>42</v>
@@ -32582,22 +32700,22 @@
         <v>42</v>
       </c>
       <c r="S20" s="6" t="s">
-        <v>2303</v>
+        <v>2317</v>
       </c>
       <c r="T20" s="6" t="s">
-        <v>2251</v>
+        <v>2265</v>
       </c>
       <c r="U20" s="6" t="s">
-        <v>2304</v>
+        <v>2318</v>
       </c>
       <c r="V20" s="6" t="s">
         <v>47</v>
       </c>
       <c r="W20" s="6" t="s">
-        <v>2305</v>
+        <v>2319</v>
       </c>
       <c r="X20" s="6" t="s">
-        <v>2306</v>
+        <v>2320</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32608,28 +32726,28 @@
         <v>139</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D21" s="6"/>
       <c r="E21" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F21" s="6"/>
       <c r="G21" s="6"/>
       <c r="H21" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I21" s="6"/>
       <c r="J21" s="6"/>
       <c r="K21" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L21" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="M21" s="6"/>
       <c r="N21" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O21" s="6" t="s">
         <v>42</v>
@@ -32644,22 +32762,22 @@
         <v>42</v>
       </c>
       <c r="S21" s="6" t="s">
-        <v>2307</v>
+        <v>2321</v>
       </c>
       <c r="T21" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U21" s="6" t="s">
-        <v>2308</v>
+        <v>2322</v>
       </c>
       <c r="V21" s="6" t="s">
         <v>47</v>
       </c>
       <c r="W21" s="6" t="s">
-        <v>2309</v>
+        <v>2323</v>
       </c>
       <c r="X21" s="6" t="s">
-        <v>2310</v>
+        <v>2324</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32670,56 +32788,56 @@
         <v>143</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D22" s="6"/>
       <c r="E22" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F22" s="6"/>
       <c r="G22" s="6"/>
       <c r="H22" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I22" s="6"/>
       <c r="J22" s="6"/>
       <c r="K22" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L22" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="M22" s="6"/>
       <c r="N22" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O22" s="6" t="s">
         <v>42</v>
       </c>
       <c r="P22" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="Q22" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="R22" s="6" t="s">
         <v>42</v>
       </c>
       <c r="S22" s="6" t="s">
-        <v>2311</v>
+        <v>2325</v>
       </c>
       <c r="T22" s="6" t="s">
-        <v>2251</v>
+        <v>2265</v>
       </c>
       <c r="U22" s="6"/>
       <c r="V22" s="6" t="s">
         <v>47</v>
       </c>
       <c r="W22" s="6" t="s">
-        <v>2312</v>
+        <v>2326</v>
       </c>
       <c r="X22" s="6" t="s">
-        <v>2313</v>
+        <v>2327</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32730,14 +32848,14 @@
         <v>146</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D23" s="6"/>
       <c r="E23" s="6" t="s">
         <v>42</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>2314</v>
+        <v>2328</v>
       </c>
       <c r="G23" s="6"/>
       <c r="H23" s="6" t="s">
@@ -32747,25 +32865,25 @@
         <v>45</v>
       </c>
       <c r="J23" s="6" t="s">
-        <v>2315</v>
+        <v>2329</v>
       </c>
       <c r="K23" s="6" t="s">
         <v>42</v>
       </c>
       <c r="L23" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="M23" s="6" t="s">
-        <v>2316</v>
+        <v>2330</v>
       </c>
       <c r="N23" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O23" s="6" t="s">
         <v>42</v>
       </c>
       <c r="P23" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="Q23" s="6" t="s">
         <v>42</v>
@@ -32774,20 +32892,20 @@
         <v>42</v>
       </c>
       <c r="S23" s="6" t="s">
-        <v>2317</v>
+        <v>2331</v>
       </c>
       <c r="T23" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U23" s="6"/>
       <c r="V23" s="6" t="s">
         <v>47</v>
       </c>
       <c r="W23" s="6" t="s">
-        <v>2318</v>
+        <v>2332</v>
       </c>
       <c r="X23" s="6" t="s">
-        <v>2319</v>
+        <v>2333</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32798,60 +32916,60 @@
         <v>149</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D24" s="6"/>
       <c r="E24" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F24" s="6"/>
       <c r="G24" s="6"/>
       <c r="H24" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I24" s="6" t="n">
         <v>30</v>
       </c>
       <c r="J24" s="6" t="s">
-        <v>2320</v>
+        <v>2334</v>
       </c>
       <c r="K24" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L24" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="M24" s="6"/>
       <c r="N24" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O24" s="6" t="s">
         <v>42</v>
       </c>
       <c r="P24" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="Q24" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="R24" s="6" t="s">
         <v>42</v>
       </c>
       <c r="S24" s="6" t="s">
-        <v>2321</v>
+        <v>2335</v>
       </c>
       <c r="T24" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U24" s="6"/>
       <c r="V24" s="6" t="s">
         <v>47</v>
       </c>
       <c r="W24" s="6" t="s">
-        <v>2322</v>
+        <v>2336</v>
       </c>
       <c r="X24" s="6" t="s">
-        <v>2323</v>
+        <v>2337</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32862,11 +32980,11 @@
         <v>153</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D25" s="6"/>
       <c r="E25" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F25" s="6"/>
       <c r="G25" s="6"/>
@@ -32876,19 +32994,19 @@
       <c r="I25" s="6"/>
       <c r="J25" s="6"/>
       <c r="K25" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L25" s="6" t="s">
         <v>42</v>
       </c>
       <c r="M25" s="6" t="s">
-        <v>2324</v>
+        <v>2338</v>
       </c>
       <c r="N25" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O25" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="P25" s="6" t="s">
         <v>42</v>
@@ -32897,16 +33015,16 @@
         <v>42</v>
       </c>
       <c r="R25" s="6" t="s">
-        <v>2291</v>
+        <v>2305</v>
       </c>
       <c r="S25" s="6" t="s">
-        <v>2325</v>
+        <v>2339</v>
       </c>
       <c r="T25" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U25" s="6" t="s">
-        <v>2326</v>
+        <v>2340</v>
       </c>
       <c r="V25" s="6" t="s">
         <v>47</v>
@@ -32915,7 +33033,7 @@
         <v>464</v>
       </c>
       <c r="X25" s="6" t="s">
-        <v>2327</v>
+        <v>2341</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="314.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32926,30 +33044,30 @@
         <v>157</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D26" s="6"/>
       <c r="E26" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F26" s="6"/>
       <c r="G26" s="6"/>
       <c r="H26" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I26" s="6"/>
       <c r="J26" s="6" t="s">
-        <v>2328</v>
+        <v>2342</v>
       </c>
       <c r="K26" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L26" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="M26" s="6"/>
       <c r="N26" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O26" s="6" t="s">
         <v>42</v>
@@ -32964,20 +33082,20 @@
         <v>42</v>
       </c>
       <c r="S26" s="6" t="s">
-        <v>2329</v>
+        <v>2343</v>
       </c>
       <c r="T26" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U26" s="6"/>
       <c r="V26" s="6" t="s">
         <v>61</v>
       </c>
       <c r="W26" s="6" t="s">
-        <v>2330</v>
+        <v>2344</v>
       </c>
       <c r="X26" s="6" t="s">
-        <v>2331</v>
+        <v>2345</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32988,32 +33106,32 @@
         <v>161</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D27" s="6"/>
       <c r="E27" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F27" s="6"/>
       <c r="G27" s="6"/>
       <c r="H27" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I27" s="6" t="n">
         <v>60</v>
       </c>
       <c r="J27" s="6" t="s">
-        <v>2332</v>
+        <v>2346</v>
       </c>
       <c r="K27" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L27" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="M27" s="6"/>
       <c r="N27" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O27" s="6" t="s">
         <v>42</v>
@@ -33028,20 +33146,20 @@
         <v>42</v>
       </c>
       <c r="S27" s="6" t="s">
-        <v>2333</v>
+        <v>2347</v>
       </c>
       <c r="T27" s="6" t="s">
-        <v>2251</v>
+        <v>2265</v>
       </c>
       <c r="U27" s="6"/>
       <c r="V27" s="6" t="s">
         <v>47</v>
       </c>
       <c r="W27" s="6" t="s">
-        <v>2334</v>
+        <v>2348</v>
       </c>
       <c r="X27" s="6" t="s">
-        <v>2335</v>
+        <v>2349</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33059,29 +33177,29 @@
         <v>42</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>2336</v>
+        <v>2350</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>2337</v>
+        <v>2351</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I28" s="6"/>
       <c r="J28" s="6" t="s">
-        <v>2338</v>
+        <v>2352</v>
       </c>
       <c r="K28" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L28" s="6" t="s">
         <v>42</v>
       </c>
       <c r="M28" s="6" t="s">
-        <v>2339</v>
+        <v>2353</v>
       </c>
       <c r="N28" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O28" s="6" t="s">
         <v>42</v>
@@ -33096,20 +33214,20 @@
         <v>42</v>
       </c>
       <c r="S28" s="6" t="s">
-        <v>2340</v>
+        <v>2354</v>
       </c>
       <c r="T28" s="6" t="s">
-        <v>2251</v>
+        <v>2265</v>
       </c>
       <c r="U28" s="6"/>
       <c r="V28" s="6" t="s">
         <v>47</v>
       </c>
       <c r="W28" s="6" t="s">
-        <v>2341</v>
+        <v>2355</v>
       </c>
       <c r="X28" s="6" t="s">
-        <v>2342</v>
+        <v>2356</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33120,31 +33238,31 @@
         <v>167</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D29" s="6"/>
       <c r="E29" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F29" s="6"/>
       <c r="G29" s="6"/>
       <c r="H29" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I29" s="6"/>
       <c r="J29" s="6"/>
       <c r="K29" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L29" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="M29" s="6"/>
       <c r="N29" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O29" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="P29" s="6" t="s">
         <v>42</v>
@@ -33156,10 +33274,10 @@
         <v>42</v>
       </c>
       <c r="S29" s="6" t="s">
-        <v>2343</v>
+        <v>2357</v>
       </c>
       <c r="T29" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U29" s="6"/>
       <c r="V29" s="6" t="s">
@@ -33169,7 +33287,7 @@
         <v>494</v>
       </c>
       <c r="X29" s="6" t="s">
-        <v>2344</v>
+        <v>2358</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="202.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33180,32 +33298,32 @@
         <v>171</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D30" s="6"/>
       <c r="E30" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F30" s="6"/>
       <c r="G30" s="6"/>
       <c r="H30" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I30" s="6"/>
       <c r="J30" s="6" t="s">
-        <v>2345</v>
+        <v>2359</v>
       </c>
       <c r="K30" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L30" s="6" t="s">
         <v>42</v>
       </c>
       <c r="M30" s="6" t="s">
-        <v>2346</v>
+        <v>2360</v>
       </c>
       <c r="N30" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O30" s="6" t="s">
         <v>42</v>
@@ -33220,20 +33338,20 @@
         <v>42</v>
       </c>
       <c r="S30" s="6" t="s">
-        <v>2347</v>
+        <v>2361</v>
       </c>
       <c r="T30" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U30" s="6"/>
       <c r="V30" s="6" t="s">
         <v>47</v>
       </c>
       <c r="W30" s="6" t="s">
-        <v>2348</v>
+        <v>2362</v>
       </c>
       <c r="X30" s="6" t="s">
-        <v>2349</v>
+        <v>2363</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33244,30 +33362,30 @@
         <v>175</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D31" s="6"/>
       <c r="E31" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F31" s="6"/>
       <c r="G31" s="6"/>
       <c r="H31" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I31" s="6"/>
       <c r="J31" s="6"/>
       <c r="K31" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L31" s="6" t="s">
         <v>42</v>
       </c>
       <c r="M31" s="6" t="s">
-        <v>2350</v>
+        <v>2364</v>
       </c>
       <c r="N31" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O31" s="6" t="s">
         <v>42</v>
@@ -33282,10 +33400,10 @@
         <v>42</v>
       </c>
       <c r="S31" s="6" t="s">
-        <v>2351</v>
+        <v>2365</v>
       </c>
       <c r="T31" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U31" s="6"/>
       <c r="V31" s="6" t="s">
@@ -33295,7 +33413,7 @@
         <v>511</v>
       </c>
       <c r="X31" s="6" t="s">
-        <v>2352</v>
+        <v>2366</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33306,14 +33424,14 @@
         <v>179</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D32" s="6"/>
       <c r="E32" s="6" t="s">
         <v>42</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>2353</v>
+        <v>2367</v>
       </c>
       <c r="G32" s="6"/>
       <c r="H32" s="6" t="s">
@@ -33322,16 +33440,16 @@
       <c r="I32" s="6"/>
       <c r="J32" s="6"/>
       <c r="K32" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L32" s="6" t="s">
         <v>42</v>
       </c>
       <c r="M32" s="6" t="s">
-        <v>2354</v>
+        <v>2368</v>
       </c>
       <c r="N32" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O32" s="6" t="s">
         <v>42</v>
@@ -33346,10 +33464,10 @@
         <v>42</v>
       </c>
       <c r="S32" s="6" t="s">
-        <v>2355</v>
+        <v>2369</v>
       </c>
       <c r="T32" s="6" t="s">
-        <v>2251</v>
+        <v>2265</v>
       </c>
       <c r="U32" s="6"/>
       <c r="V32" s="6" t="s">
@@ -33359,7 +33477,7 @@
         <v>1423</v>
       </c>
       <c r="X32" s="6" t="s">
-        <v>2356</v>
+        <v>2370</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="169.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33370,32 +33488,32 @@
         <v>183</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D33" s="6"/>
       <c r="E33" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F33" s="6"/>
       <c r="G33" s="6"/>
       <c r="H33" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I33" s="6" t="n">
         <v>90</v>
       </c>
       <c r="J33" s="6" t="s">
-        <v>2357</v>
+        <v>2371</v>
       </c>
       <c r="K33" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L33" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="M33" s="6"/>
       <c r="N33" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O33" s="6" t="s">
         <v>42</v>
@@ -33410,20 +33528,20 @@
         <v>42</v>
       </c>
       <c r="S33" s="6" t="s">
-        <v>2358</v>
+        <v>2372</v>
       </c>
       <c r="T33" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U33" s="6"/>
       <c r="V33" s="6" t="s">
         <v>47</v>
       </c>
       <c r="W33" s="6" t="s">
-        <v>2359</v>
+        <v>2373</v>
       </c>
       <c r="X33" s="6" t="s">
-        <v>2360</v>
+        <v>2374</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33434,32 +33552,32 @@
         <v>187</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D34" s="6"/>
       <c r="E34" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F34" s="6"/>
       <c r="G34" s="6"/>
       <c r="H34" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I34" s="6" t="n">
         <v>60</v>
       </c>
       <c r="J34" s="6" t="s">
-        <v>2361</v>
+        <v>2375</v>
       </c>
       <c r="K34" s="6" t="s">
         <v>42</v>
       </c>
       <c r="L34" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="M34" s="6"/>
       <c r="N34" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O34" s="6" t="s">
         <v>42</v>
@@ -33468,14 +33586,14 @@
         <v>42</v>
       </c>
       <c r="Q34" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="R34" s="6" t="s">
-        <v>2291</v>
+        <v>2305</v>
       </c>
       <c r="S34" s="6"/>
       <c r="T34" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U34" s="6"/>
       <c r="V34" s="6" t="s">
@@ -33485,7 +33603,7 @@
         <v>537</v>
       </c>
       <c r="X34" s="6" t="s">
-        <v>2362</v>
+        <v>2376</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33496,34 +33614,34 @@
         <v>190</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D35" s="6"/>
       <c r="E35" s="6" t="s">
         <v>42</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>2363</v>
+        <v>2377</v>
       </c>
       <c r="G35" s="6"/>
       <c r="H35" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I35" s="6"/>
       <c r="J35" s="6" t="s">
-        <v>2364</v>
+        <v>2378</v>
       </c>
       <c r="K35" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L35" s="6" t="s">
         <v>42</v>
       </c>
       <c r="M35" s="6" t="s">
-        <v>2365</v>
+        <v>2379</v>
       </c>
       <c r="N35" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O35" s="6" t="s">
         <v>42</v>
@@ -33538,20 +33656,20 @@
         <v>42</v>
       </c>
       <c r="S35" s="6" t="s">
-        <v>2366</v>
+        <v>2380</v>
       </c>
       <c r="T35" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U35" s="6"/>
       <c r="V35" s="6" t="s">
         <v>61</v>
       </c>
       <c r="W35" s="6" t="s">
-        <v>2367</v>
+        <v>2381</v>
       </c>
       <c r="X35" s="6" t="s">
-        <v>2368</v>
+        <v>2382</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33562,30 +33680,30 @@
         <v>194</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D36" s="6"/>
       <c r="E36" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F36" s="6"/>
       <c r="G36" s="6"/>
       <c r="H36" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I36" s="6"/>
       <c r="J36" s="6"/>
       <c r="K36" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L36" s="6" t="s">
         <v>42</v>
       </c>
       <c r="M36" s="6" t="s">
-        <v>2369</v>
+        <v>2383</v>
       </c>
       <c r="N36" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O36" s="6" t="s">
         <v>42</v>
@@ -33600,22 +33718,22 @@
         <v>42</v>
       </c>
       <c r="S36" s="6" t="s">
-        <v>2370</v>
+        <v>2384</v>
       </c>
       <c r="T36" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U36" s="6" t="s">
-        <v>2371</v>
+        <v>2385</v>
       </c>
       <c r="V36" s="6" t="s">
         <v>47</v>
       </c>
       <c r="W36" s="6" t="s">
-        <v>2372</v>
+        <v>2386</v>
       </c>
       <c r="X36" s="6" t="s">
-        <v>2373</v>
+        <v>2387</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33626,11 +33744,11 @@
         <v>198</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D37" s="6"/>
       <c r="E37" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F37" s="6"/>
       <c r="G37" s="6"/>
@@ -33639,22 +33757,22 @@
       </c>
       <c r="I37" s="6"/>
       <c r="J37" s="6" t="s">
-        <v>2374</v>
+        <v>2388</v>
       </c>
       <c r="K37" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L37" s="6" t="s">
         <v>42</v>
       </c>
       <c r="M37" s="6" t="s">
-        <v>2375</v>
+        <v>2389</v>
       </c>
       <c r="N37" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O37" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="P37" s="6" t="s">
         <v>42</v>
@@ -33666,20 +33784,20 @@
         <v>42</v>
       </c>
       <c r="S37" s="6" t="s">
-        <v>2376</v>
+        <v>2390</v>
       </c>
       <c r="T37" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U37" s="6"/>
       <c r="V37" s="6" t="s">
         <v>61</v>
       </c>
       <c r="W37" s="6" t="s">
-        <v>2377</v>
+        <v>2391</v>
       </c>
       <c r="X37" s="6" t="s">
-        <v>2378</v>
+        <v>2392</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="281.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33690,32 +33808,32 @@
         <v>202</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D38" s="6"/>
       <c r="E38" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F38" s="6"/>
       <c r="G38" s="6"/>
       <c r="H38" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I38" s="6" t="n">
         <v>45</v>
       </c>
       <c r="J38" s="6" t="s">
-        <v>2379</v>
+        <v>2393</v>
       </c>
       <c r="K38" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L38" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="M38" s="6"/>
       <c r="N38" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O38" s="6" t="s">
         <v>42</v>
@@ -33730,20 +33848,20 @@
         <v>42</v>
       </c>
       <c r="S38" s="6" t="s">
-        <v>2380</v>
+        <v>2394</v>
       </c>
       <c r="T38" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U38" s="6"/>
       <c r="V38" s="6" t="s">
         <v>47</v>
       </c>
       <c r="W38" s="6" t="s">
-        <v>2381</v>
+        <v>2395</v>
       </c>
       <c r="X38" s="6" t="s">
-        <v>2382</v>
+        <v>2396</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33754,11 +33872,11 @@
         <v>206</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D39" s="6"/>
       <c r="E39" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F39" s="6"/>
       <c r="G39" s="6"/>
@@ -33767,22 +33885,22 @@
       </c>
       <c r="I39" s="6"/>
       <c r="J39" s="6" t="s">
-        <v>2383</v>
+        <v>2397</v>
       </c>
       <c r="K39" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L39" s="6" t="s">
         <v>42</v>
       </c>
       <c r="M39" s="6" t="s">
-        <v>2384</v>
+        <v>2398</v>
       </c>
       <c r="N39" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O39" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="P39" s="6" t="s">
         <v>42</v>
@@ -33794,22 +33912,22 @@
         <v>42</v>
       </c>
       <c r="S39" s="6" t="s">
-        <v>2385</v>
+        <v>2399</v>
       </c>
       <c r="T39" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U39" s="6" t="s">
-        <v>2386</v>
+        <v>2400</v>
       </c>
       <c r="V39" s="6" t="s">
         <v>47</v>
       </c>
       <c r="W39" s="6" t="s">
-        <v>2387</v>
+        <v>2401</v>
       </c>
       <c r="X39" s="6" t="s">
-        <v>2388</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="236.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33820,38 +33938,38 @@
         <v>210</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D40" s="6"/>
       <c r="E40" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F40" s="6"/>
       <c r="G40" s="6"/>
       <c r="H40" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I40" s="6" t="n">
         <v>60</v>
       </c>
       <c r="J40" s="6" t="s">
-        <v>2389</v>
+        <v>2403</v>
       </c>
       <c r="K40" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L40" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="M40" s="6"/>
       <c r="N40" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O40" s="6" t="s">
         <v>42</v>
       </c>
       <c r="P40" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="Q40" s="6" t="s">
         <v>42</v>
@@ -33860,20 +33978,20 @@
         <v>42</v>
       </c>
       <c r="S40" s="6" t="s">
-        <v>2390</v>
+        <v>2404</v>
       </c>
       <c r="T40" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U40" s="6"/>
       <c r="V40" s="6" t="s">
         <v>47</v>
       </c>
       <c r="W40" s="6" t="s">
-        <v>2391</v>
+        <v>2405</v>
       </c>
       <c r="X40" s="6" t="s">
-        <v>2392</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="169.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33884,30 +34002,30 @@
         <v>215</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D41" s="6"/>
       <c r="E41" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F41" s="6"/>
       <c r="G41" s="6" t="s">
-        <v>2393</v>
+        <v>2407</v>
       </c>
       <c r="H41" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I41" s="6"/>
       <c r="J41" s="6"/>
       <c r="K41" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L41" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="M41" s="6"/>
       <c r="N41" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O41" s="6" t="s">
         <v>42</v>
@@ -33922,10 +34040,10 @@
         <v>42</v>
       </c>
       <c r="S41" s="6" t="s">
-        <v>2394</v>
+        <v>2408</v>
       </c>
       <c r="T41" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U41" s="6"/>
       <c r="V41" s="6" t="s">
@@ -33935,7 +34053,7 @@
         <v>594</v>
       </c>
       <c r="X41" s="6" t="s">
-        <v>2395</v>
+        <v>2409</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33946,28 +34064,28 @@
         <v>219</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D42" s="6"/>
       <c r="E42" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F42" s="6"/>
       <c r="G42" s="6"/>
       <c r="H42" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I42" s="6"/>
       <c r="J42" s="6"/>
       <c r="K42" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L42" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="M42" s="6"/>
       <c r="N42" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O42" s="6" t="s">
         <v>42</v>
@@ -33979,23 +34097,23 @@
         <v>42</v>
       </c>
       <c r="R42" s="6" t="s">
-        <v>2291</v>
+        <v>2305</v>
       </c>
       <c r="S42" s="6" t="s">
-        <v>2396</v>
+        <v>2410</v>
       </c>
       <c r="T42" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U42" s="6"/>
       <c r="V42" s="6" t="s">
         <v>47</v>
       </c>
       <c r="W42" s="6" t="s">
-        <v>2397</v>
+        <v>2411</v>
       </c>
       <c r="X42" s="6" t="s">
-        <v>2398</v>
+        <v>2412</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="169.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -34006,56 +34124,56 @@
         <v>221</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D43" s="6"/>
       <c r="E43" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F43" s="6"/>
       <c r="G43" s="6"/>
       <c r="H43" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I43" s="6"/>
       <c r="J43" s="6"/>
       <c r="K43" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L43" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="M43" s="6"/>
       <c r="N43" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O43" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="P43" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="Q43" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="R43" s="6" t="s">
         <v>42</v>
       </c>
       <c r="S43" s="6" t="s">
-        <v>2399</v>
+        <v>2413</v>
       </c>
       <c r="T43" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U43" s="6"/>
       <c r="V43" s="6" t="s">
         <v>61</v>
       </c>
       <c r="W43" s="6" t="s">
-        <v>2400</v>
+        <v>2414</v>
       </c>
       <c r="X43" s="6" t="s">
-        <v>2401</v>
+        <v>2415</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="169.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -34066,33 +34184,33 @@
         <v>223</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D44" s="6"/>
       <c r="E44" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F44" s="6"/>
       <c r="G44" s="6"/>
       <c r="H44" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I44" s="6"/>
       <c r="J44" s="6"/>
       <c r="K44" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L44" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="M44" s="6" t="s">
-        <v>2402</v>
+        <v>2416</v>
       </c>
       <c r="N44" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O44" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="P44" s="6" t="s">
         <v>42</v>
@@ -34104,20 +34222,20 @@
         <v>42</v>
       </c>
       <c r="S44" s="6" t="s">
-        <v>2403</v>
+        <v>2417</v>
       </c>
       <c r="T44" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U44" s="6"/>
       <c r="V44" s="6" t="s">
         <v>47</v>
       </c>
       <c r="W44" s="6" t="s">
-        <v>2404</v>
+        <v>2418</v>
       </c>
       <c r="X44" s="6" t="s">
-        <v>2405</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -34128,11 +34246,11 @@
         <v>229</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D45" s="6"/>
       <c r="E45" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F45" s="6"/>
       <c r="G45" s="6"/>
@@ -34143,19 +34261,19 @@
         <v>30</v>
       </c>
       <c r="J45" s="6" t="s">
-        <v>2406</v>
+        <v>2420</v>
       </c>
       <c r="K45" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L45" s="6" t="s">
         <v>42</v>
       </c>
       <c r="M45" s="6" t="s">
-        <v>2407</v>
+        <v>2421</v>
       </c>
       <c r="N45" s="6" t="s">
-        <v>2408</v>
+        <v>2422</v>
       </c>
       <c r="O45" s="6" t="s">
         <v>42</v>
@@ -34170,22 +34288,22 @@
         <v>42</v>
       </c>
       <c r="S45" s="6" t="s">
-        <v>2409</v>
+        <v>2423</v>
       </c>
       <c r="T45" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U45" s="6" t="s">
-        <v>2410</v>
+        <v>2424</v>
       </c>
       <c r="V45" s="6" t="s">
         <v>47</v>
       </c>
       <c r="W45" s="6" t="s">
-        <v>2411</v>
+        <v>2425</v>
       </c>
       <c r="X45" s="6" t="s">
-        <v>2412</v>
+        <v>2426</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -34196,32 +34314,32 @@
         <v>233</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D46" s="6"/>
       <c r="E46" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F46" s="6"/>
       <c r="G46" s="6"/>
       <c r="H46" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I46" s="6"/>
       <c r="J46" s="6" t="s">
-        <v>2413</v>
+        <v>2427</v>
       </c>
       <c r="K46" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L46" s="6" t="s">
         <v>42</v>
       </c>
       <c r="M46" s="6" t="s">
-        <v>2414</v>
+        <v>2428</v>
       </c>
       <c r="N46" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O46" s="6" t="s">
         <v>42</v>
@@ -34233,25 +34351,25 @@
         <v>42</v>
       </c>
       <c r="R46" s="6" t="s">
-        <v>2291</v>
+        <v>2305</v>
       </c>
       <c r="S46" s="6" t="s">
-        <v>2415</v>
+        <v>2429</v>
       </c>
       <c r="T46" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U46" s="6" t="s">
-        <v>2416</v>
+        <v>2430</v>
       </c>
       <c r="V46" s="6" t="s">
         <v>47</v>
       </c>
       <c r="W46" s="6" t="s">
-        <v>2417</v>
+        <v>2431</v>
       </c>
       <c r="X46" s="6" t="s">
-        <v>2418</v>
+        <v>2432</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -34262,35 +34380,35 @@
         <v>236</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D47" s="6"/>
       <c r="E47" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F47" s="6"/>
       <c r="G47" s="6"/>
       <c r="H47" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I47" s="6"/>
       <c r="J47" s="6" t="s">
-        <v>2419</v>
+        <v>2433</v>
       </c>
       <c r="K47" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L47" s="6" t="s">
         <v>42</v>
       </c>
       <c r="M47" s="6" t="s">
-        <v>2420</v>
+        <v>2434</v>
       </c>
       <c r="N47" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O47" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="P47" s="6" t="s">
         <v>42</v>
@@ -34302,22 +34420,22 @@
         <v>42</v>
       </c>
       <c r="S47" s="6" t="s">
-        <v>2421</v>
+        <v>2435</v>
       </c>
       <c r="T47" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U47" s="6" t="s">
-        <v>2422</v>
+        <v>2436</v>
       </c>
       <c r="V47" s="6" t="s">
         <v>47</v>
       </c>
       <c r="W47" s="6" t="s">
-        <v>2423</v>
+        <v>2437</v>
       </c>
       <c r="X47" s="6" t="s">
-        <v>2424</v>
+        <v>2438</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -34328,56 +34446,56 @@
         <v>239</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D48" s="6"/>
       <c r="E48" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F48" s="6"/>
       <c r="G48" s="6"/>
       <c r="H48" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I48" s="6"/>
       <c r="J48" s="6"/>
       <c r="K48" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L48" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="M48" s="6"/>
       <c r="N48" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O48" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="P48" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="Q48" s="6" t="s">
         <v>42</v>
       </c>
       <c r="R48" s="6" t="s">
-        <v>2291</v>
+        <v>2305</v>
       </c>
       <c r="S48" s="6" t="s">
-        <v>2425</v>
+        <v>2439</v>
       </c>
       <c r="T48" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U48" s="6"/>
       <c r="V48" s="6" t="s">
         <v>47</v>
       </c>
       <c r="W48" s="6" t="s">
-        <v>2426</v>
+        <v>2440</v>
       </c>
       <c r="X48" s="6" t="s">
-        <v>2427</v>
+        <v>2441</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -34388,34 +34506,34 @@
         <v>243</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D49" s="6"/>
       <c r="E49" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F49" s="6"/>
       <c r="G49" s="6"/>
       <c r="H49" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I49" s="6"/>
       <c r="J49" s="6"/>
       <c r="K49" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L49" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="M49" s="6"/>
       <c r="N49" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O49" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="P49" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="Q49" s="6" t="s">
         <v>42</v>
@@ -34424,20 +34542,20 @@
         <v>42</v>
       </c>
       <c r="S49" s="6" t="s">
-        <v>2428</v>
+        <v>2442</v>
       </c>
       <c r="T49" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U49" s="6"/>
       <c r="V49" s="6" t="s">
         <v>47</v>
       </c>
       <c r="W49" s="6" t="s">
-        <v>2429</v>
+        <v>2443</v>
       </c>
       <c r="X49" s="6" t="s">
-        <v>2430</v>
+        <v>2444</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -34448,32 +34566,32 @@
         <v>248</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D50" s="6"/>
       <c r="E50" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F50" s="6"/>
       <c r="G50" s="6"/>
       <c r="H50" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I50" s="6" t="n">
         <v>30</v>
       </c>
       <c r="J50" s="6" t="s">
-        <v>2431</v>
+        <v>2445</v>
       </c>
       <c r="K50" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L50" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="M50" s="6"/>
       <c r="N50" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O50" s="6" t="s">
         <v>42</v>
@@ -34488,22 +34606,22 @@
         <v>42</v>
       </c>
       <c r="S50" s="6" t="s">
-        <v>2432</v>
+        <v>2446</v>
       </c>
       <c r="T50" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U50" s="6" t="s">
-        <v>2433</v>
+        <v>2447</v>
       </c>
       <c r="V50" s="6" t="s">
         <v>47</v>
       </c>
       <c r="W50" s="6" t="s">
-        <v>2434</v>
+        <v>2448</v>
       </c>
       <c r="X50" s="6" t="s">
-        <v>2435</v>
+        <v>2449</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="169.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -34514,34 +34632,34 @@
         <v>252</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="D51" s="6"/>
       <c r="E51" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="F51" s="6"/>
       <c r="G51" s="6"/>
       <c r="H51" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="I51" s="6"/>
       <c r="J51" s="6"/>
       <c r="K51" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="L51" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="M51" s="6"/>
       <c r="N51" s="6" t="s">
-        <v>2207</v>
+        <v>2221</v>
       </c>
       <c r="O51" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="P51" s="6" t="s">
-        <v>2203</v>
+        <v>2217</v>
       </c>
       <c r="Q51" s="6" t="s">
         <v>42</v>
@@ -34550,20 +34668,20 @@
         <v>42</v>
       </c>
       <c r="S51" s="6" t="s">
-        <v>2436</v>
+        <v>2450</v>
       </c>
       <c r="T51" s="6" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="U51" s="6"/>
       <c r="V51" s="6" t="s">
         <v>47</v>
       </c>
       <c r="W51" s="6" t="s">
-        <v>2437</v>
+        <v>2451</v>
       </c>
       <c r="X51" s="6" t="s">
-        <v>2438</v>
+        <v>2452</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Tab intros, State Rules / Dashboard Overview / Map: U.S. Audit Climate / Cases & Laws names, pinned jump bar, map toggle on the map, downloads trimmed to Excel, PDFs and one JSON
</commit_message>
<xml_diff>
--- a/docs/downloads/warranty-atlas.xlsx
+++ b/docs/downloads/warranty-atlas.xlsx
@@ -17,11 +17,11 @@
     <sheet name="Weekly log" sheetId="7" state="visible" r:id="rId9"/>
     <sheet name="News" sheetId="8" state="visible" r:id="rId10"/>
     <sheet name="Audit procedures" sheetId="9" state="visible" r:id="rId11"/>
-    <sheet name="Audit index" sheetId="10" state="visible" r:id="rId12"/>
+    <sheet name="Audit climate" sheetId="10" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
+    <definedName function="false" hidden="true" localSheetId="9" name="_xlnm._FilterDatabase" vbProcedure="false">'Audit climate'!$A$1:$T$51</definedName>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'Audit fields'!$A$1:$AN$51</definedName>
-    <definedName function="false" hidden="true" localSheetId="9" name="_xlnm._FilterDatabase" vbProcedure="false">'Audit index'!$A$1:$T$51</definedName>
     <definedName function="false" hidden="true" localSheetId="8" name="_xlnm._FilterDatabase" vbProcedure="false">'Audit procedures'!$A$1:$X$51</definedName>
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Coverage!$A$1:$L$201</definedName>
     <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">'Law dates'!$A$1:$M$51</definedName>
@@ -69,7 +69,7 @@
     <t xml:space="preserve">Audit procedures: notice, selection basis, frequency, written reasons, response period, appeal, chargeback holds, extrapolation, clerical errors, documentation limits, fraud carve-outs, rate validation and consequences, with quotes.</t>
   </si>
   <si>
-    <t xml:space="preserve">Audit index: the audit restrictiveness index (0-100) with the points behind it, plus distributor-franchised states. Higher = more statutory limits on audits, chargebacks and rate validation. Statute text only.</t>
+    <t xml:space="preserve">Audit climate: the audit climate score (0-100) behind the Map: U.S. Audit Climate tab, with the points behind it, plus distributor-franchised states. Higher = more restrictive toward audits, chargebacks and rate validation. Statute text only.</t>
   </si>
   <si>
     <t xml:space="preserve">Weekly log and News: the Update log and News tabs.</t>
@@ -7401,7 +7401,7 @@
     <t xml:space="preserve">§ 31-16-117(d) covers predelivery, WARRANTY, SALES INCENTIVE and SERVICE INCENTIVE claims in one sentence. Warranty and incentive audits share the same 1-year window after payment for 'unsubstantiated or incorrect' claims, with 4 years on reasonable suspicion of fraud. No notice, selection, frequency, response, appeal, stay, documentation or extrapolation rules. The claim-stage resubmission right and the rate-submission process ((f)-(t)) were added by 2025 SF0106 (Enrolled Act 44, eff. 7/1/2025). Since 7/1/2025, non-house-trailer/semitrailer trailer dealers and manufacturers are exempt from § 31-16-117 (§ 31-16-124(g), 2025 HB0242). The only general penalty is a misdemeanor, fine up to $750 and/or 6 months (§ 31-16-112), not audit-specific. The official title compilation shows no section history. No 2026 amendment found.</t>
   </si>
   <si>
-    <t xml:space="preserve">Index (0-100)</t>
+    <t xml:space="preserve">Score (0-100)</t>
   </si>
   <si>
     <t xml:space="preserve">Tier</t>
@@ -7482,7 +7482,7 @@
     <t xml:space="preserve">Subaru Distributors Corp.</t>
   </si>
   <si>
-    <t xml:space="preserve">How the index is scored (higher = more statutory limits; statute text only, not legal advice)</t>
+    <t xml:space="preserve">How the audit climate score is built (higher = more restrictive; statute text only, not legal advice)</t>
   </si>
   <si>
     <t xml:space="preserve">Short audit and chargeback lookback (15 pts): 15 points if paid claims can be audited or charged back for 6 months or less, 10 for 9 months, 5 for 12 months, 0 if the statute sets no limit.</t>

</xml_diff>

<commit_message>
Audit climate score v2: 0-3 levels x separate weights (sum 100), two sub-scores, full scoring table
</commit_message>
<xml_diff>
--- a/docs/downloads/warranty-atlas.xlsx
+++ b/docs/downloads/warranty-atlas.xlsx
@@ -20,7 +20,7 @@
     <sheet name="Audit climate" sheetId="10" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="9" name="_xlnm._FilterDatabase" vbProcedure="false">'Audit climate'!$A$1:$T$51</definedName>
+    <definedName function="false" hidden="true" localSheetId="9" name="_xlnm._FilterDatabase" vbProcedure="false">'Audit climate'!$A$1:$V$51</definedName>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'Audit fields'!$A$1:$AN$51</definedName>
     <definedName function="false" hidden="true" localSheetId="8" name="_xlnm._FilterDatabase" vbProcedure="false">'Audit procedures'!$A$1:$X$51</definedName>
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Coverage!$A$1:$L$201</definedName>
@@ -40,12 +40,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6654" uniqueCount="2496">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6656" uniqueCount="2498">
   <si>
     <t xml:space="preserve">Warranty Atlas · workpaper export</t>
   </si>
   <si>
-    <t xml:space="preserve">Built 2026-09-28 from the live Atlas data files.</t>
+    <t xml:space="preserve">Built 2026-09-29 from the live Atlas data files.</t>
   </si>
   <si>
     <t xml:space="preserve">What is in this workbook</t>
@@ -69,7 +69,7 @@
     <t xml:space="preserve">Audit procedures: notice, selection basis, frequency, written reasons, response period, appeal, chargeback holds, extrapolation, clerical errors, documentation limits, fraud carve-outs, rate validation and consequences, with quotes.</t>
   </si>
   <si>
-    <t xml:space="preserve">Audit climate: the audit climate score (0-100) behind the Map: U.S. Audit Climate tab, with the points behind it, plus distributor-franchised states. Higher = more restrictive toward audits, chargebacks and rate validation. Statute text only.</t>
+    <t xml:space="preserve">Audit climate: the audit climate score (0-100) behind the Map: U.S. Audit Climate tab, its two sub-scores and each limit's level (0-3), with the weights, plus distributor-franchised states. Higher = more restrictive toward audits, chargebacks and rate validation. Statute text only.</t>
   </si>
   <si>
     <t xml:space="preserve">Weekly log and News: the Update log and News tabs.</t>
@@ -7410,46 +7410,52 @@
     <t xml:space="preserve">Rank</t>
   </si>
   <si>
-    <t xml:space="preserve">Short audit and chargeback lookback (15)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chargeback held while the dealer appeals (15)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Limits on extrapolating audit results (10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No chargebacks for clerical or paperwork errors (10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Limits on documentation requirements (5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Written reasons required before a chargeback (5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dealer response or cure period (5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Internal appeal required (5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Must tell the dealer why it was selected (5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Advance written notice of audit (5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cap on how often audits can occur (5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No fraud carve-out from the time limit (5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rate validation limited to the dealer's submission (5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Specific consequence for improper audits (5)</t>
+    <t xml:space="preserve">Chargeback limits (0-100)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Process and oversight (0-100)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Short audit and chargeback lookback: level 0-3 (weight 20)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Limits on extrapolating audit results: level 0-3 (weight 15)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No fraud carve-out from the time limit: level 0-3 (weight 4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No chargebacks for clerical or paperwork errors: level 0-3 (weight 12)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Limits on documentation requirements: level 0-3 (weight 8)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chargeback held while the dealer appeals: level 0-3 (weight 15)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Advance written notice of audit: level 0-3 (weight 2.5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Must tell the dealer why it was selected: level 0-3 (weight 2.5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Written reasons required before a chargeback: level 0-3 (weight 2.5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dealer response or cure period: level 0-3 (weight 2.5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Internal appeal required: level 0-3 (weight 2.5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cap on how often audits can occur: level 0-3 (weight 2.5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rate validation limited to the dealer's submission: level 0-3 (weight 5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Specific consequence for improper audits: level 0-3 (weight 6)</t>
   </si>
   <si>
     <t xml:space="preserve">Distributor-franchised</t>
@@ -7458,21 +7464,21 @@
     <t xml:space="preserve">Low</t>
   </si>
   <si>
+    <t xml:space="preserve">Elevated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Very high</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High</t>
+  </si>
+  <si>
     <t xml:space="preserve">Moderate</t>
   </si>
   <si>
-    <t xml:space="preserve">Elevated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Very high</t>
-  </si>
-  <si>
     <t xml:space="preserve">Subaru of New England, Inc.</t>
   </si>
   <si>
-    <t xml:space="preserve">High</t>
-  </si>
-  <si>
     <t xml:space="preserve">SUBARU Hawaii</t>
   </si>
   <si>
@@ -7485,46 +7491,46 @@
     <t xml:space="preserve">How the audit climate score is built (higher = more restrictive; statute text only, not legal advice)</t>
   </si>
   <si>
-    <t xml:space="preserve">Short audit and chargeback lookback (15 pts): 15 points if paid claims can be audited or charged back for 6 months or less, 10 for 9 months, 5 for 12 months, 0 if the statute sets no limit.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chargeback held while the dealer appeals (15 pts): The chargeback cannot be collected until the dealer's appeal, protest or hearing is resolved.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Limits on extrapolating audit results (10 pts): 10 points if projecting sample results across claims is prohibited, 5 if restricted (e.g., only from a valid random sample).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No chargebacks for clerical or paperwork errors (10 pts): Claims cannot be denied or charged back solely for clerical, administrative or technical errors when the work was done properly.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Limits on documentation requirements (5 pts): Documentation demands are limited (e.g., only reasonable written requirements in effect when the claim was paid).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Written reasons required before a chargeback (5 pts): The dealer must get written notice of the specific grounds for each chargeback.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dealer response or cure period (5 pts): The dealer gets a set period to respond, rebut or cure before the chargeback.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Internal appeal required (5 pts): The manufacturer or distributor must offer an internal appeal or review.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Must tell the dealer why it was selected (5 pts): The dealer must be told the basis for selecting it for audit (in some states only for certain audits).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Advance written notice of audit (5 pts): Written notice is required before an audit begins.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cap on how often audits can occur (5 pts): The statute limits how often a dealer can be audited.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No fraud carve-out from the time limit (5 pts): The lookback limit applies even to suspected fraud.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rate validation limited to the dealer's submission (5 pts): A retail-rate submission can be checked only against the dealer's own submitted ROs or by a single accuracy objection; no request for more ROs or outside data.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Specific consequence for improper audits (5 pts): The statute attaches a specific consequence to improper audits or chargebacks (void chargeback, violation finding, fines, interest or audit-cost reimbursement).</t>
+    <t xml:space="preserve">Points = weight × level ÷ 3. Score = sum of points (0–100). Weights are a judgment call about how much each limit constrains audits and chargebacks. Levels are read from the statute text.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Short audit and chargeback lookback (weight 20; How far back and how much can be charged back): level 3: 6 months or less; level 2: 9 months; level 1: 12 months; level 0: No limit in statute, or over 12 months</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Limits on extrapolating audit results (weight 15; How far back and how much can be charged back): level 3: Prohibited; level 2: Restricted (e.g., only from a valid random sample); level 0: Not addressed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No fraud carve-out from the time limit (weight 4; How far back and how much can be charged back): level 3: The time limit applies even to suspected fraud; level 0: Fraud is excepted, or not stated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No chargebacks for clerical or paperwork errors (weight 12; What counts as a valid chargeback): level 3: Applies; level 0: Not in statute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Limits on documentation requirements (weight 8; What counts as a valid chargeback): level 3: Applies; level 0: Not in statute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chargeback held while the dealer appeals (weight 15; When a chargeback can be collected): level 3: Applies; level 0: Not in statute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Advance written notice of audit (weight 2.5; Audit process steps): level 3: Applies; level 0: Not in statute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Must tell the dealer why it was selected (weight 2.5; Audit process steps): level 3: Applies; level 0: Not in statute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Written reasons required before a chargeback (weight 2.5; Audit process steps): level 3: Applies; level 0: Not in statute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dealer response or cure period (weight 2.5; Audit process steps): level 3: 60 days or more; level 2: 30 to 59 days; level 1: Under 30 days; level 0: None in statute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Internal appeal required (weight 2.5; Audit process steps): level 3: Applies; level 0: Not in statute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cap on how often audits can occur (weight 2.5; Audit process steps): level 3: At most one audit per 12 months; level 2: Cap allows more than one audit a year (e.g., one per 9 months); level 0: No cap in statute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rate validation limited to the dealer's submission (weight 5; Rate validation and consequences): level 3: Only the dealer's own ROs or a single accuracy objection; level 0: Not limited in statute</t>
   </si>
   <si>
     <t xml:space="preserve">Tiers: Very high 50+; High 40–49; Elevated 30–39; Moderate 20–29; Low under 20</t>
@@ -8113,7 +8119,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:T68"/>
+  <dimension ref="A1:V68"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -8121,8 +8127,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="6" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="6" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="34"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8186,6 +8192,12 @@
       <c r="T1" s="4" t="s">
         <v>2470</v>
       </c>
+      <c r="U1" s="4" t="s">
+        <v>2471</v>
+      </c>
+      <c r="V1" s="4" t="s">
+        <v>2472</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
@@ -8195,22 +8207,22 @@
         <v>38</v>
       </c>
       <c r="C2" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>2473</v>
+      </c>
+      <c r="E2" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="F2" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G2" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="D2" s="6" t="s">
-        <v>2471</v>
-      </c>
-      <c r="E2" s="6" t="n">
-        <v>44</v>
-      </c>
-      <c r="F2" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="G2" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="H2" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I2" s="6" t="n">
         <v>0</v>
@@ -8234,7 +8246,7 @@
         <v>0</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Q2" s="6" t="n">
         <v>0</v>
@@ -8243,9 +8255,15 @@
         <v>0</v>
       </c>
       <c r="S2" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T2" s="6"/>
+        <v>3</v>
+      </c>
+      <c r="T2" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U2" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V2" s="6"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
@@ -8255,34 +8273,34 @@
         <v>50</v>
       </c>
       <c r="C3" s="6" t="n">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>2472</v>
+        <v>2474</v>
       </c>
       <c r="E3" s="6" t="n">
         <v>31</v>
       </c>
       <c r="F3" s="6" t="n">
-        <v>5</v>
+        <v>41</v>
       </c>
       <c r="G3" s="6" t="n">
         <v>0</v>
       </c>
       <c r="H3" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I3" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J3" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K3" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M3" s="6" t="n">
         <v>0</v>
@@ -8297,7 +8315,7 @@
         <v>0</v>
       </c>
       <c r="Q3" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="R3" s="6" t="n">
         <v>0</v>
@@ -8305,7 +8323,13 @@
       <c r="S3" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T3" s="6"/>
+      <c r="T3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
@@ -8315,37 +8339,37 @@
         <v>58</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>2473</v>
+        <v>2474</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>5</v>
+        <v>46</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J4" s="6" t="n">
         <v>0</v>
       </c>
       <c r="K4" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L4" s="6" t="n">
         <v>0</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>0</v>
@@ -8365,7 +8389,13 @@
       <c r="S4" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T4" s="6"/>
+      <c r="T4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
@@ -8375,37 +8405,37 @@
         <v>64</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>2473</v>
+        <v>2474</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>5</v>
+        <v>46</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>0</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>0</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>0</v>
@@ -8425,7 +8455,13 @@
       <c r="S5" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T5" s="6"/>
+      <c r="T5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
@@ -8435,57 +8471,63 @@
         <v>69</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>2474</v>
+        <v>2475</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>10</v>
+        <v>79</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>15</v>
+        <v>51</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="J6" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K6" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R6" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T6" s="6"/>
+        <v>2</v>
+      </c>
+      <c r="T6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
@@ -8495,37 +8537,37 @@
         <v>74</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>2473</v>
+        <v>2476</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>10</v>
+        <v>49</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I7" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K7" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>0</v>
@@ -8543,9 +8585,15 @@
         <v>0</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="T7" s="6"/>
+        <v>0</v>
+      </c>
+      <c r="T7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="V7" s="6"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
@@ -8558,31 +8606,31 @@
         <v>20</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>2472</v>
+        <v>2477</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J8" s="6" t="n">
         <v>0</v>
       </c>
       <c r="K8" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="M8" s="6" t="n">
         <v>0</v>
@@ -8597,7 +8645,7 @@
         <v>0</v>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R8" s="6" t="n">
         <v>0</v>
@@ -8605,8 +8653,14 @@
       <c r="S8" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T8" s="6" t="s">
-        <v>2475</v>
+      <c r="T8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V8" s="6" t="s">
+        <v>2478</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8617,34 +8671,34 @@
         <v>87</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>2473</v>
+        <v>2476</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>15</v>
+        <v>54</v>
       </c>
       <c r="G9" s="6" t="n">
         <v>0</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M9" s="6" t="n">
         <v>0</v>
@@ -8667,7 +8721,13 @@
       <c r="S9" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T9" s="6"/>
+      <c r="T9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V9" s="6"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
@@ -8677,57 +8737,63 @@
         <v>92</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>2474</v>
+        <v>2475</v>
       </c>
       <c r="E10" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>62</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>78</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="K10" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="L10" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="M10" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="N10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="P10" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q10" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="F10" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="G10" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="H10" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="J10" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="K10" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="L10" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="M10" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="O10" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q10" s="6" t="n">
-        <v>5</v>
-      </c>
       <c r="R10" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="S10" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="T10" s="6"/>
+        <v>3</v>
+      </c>
+      <c r="T10" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="U10" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="V10" s="6"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
@@ -8737,37 +8803,37 @@
         <v>97</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>2476</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>0</v>
@@ -8779,7 +8845,7 @@
         <v>0</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R11" s="6" t="n">
         <v>0</v>
@@ -8787,7 +8853,13 @@
       <c r="S11" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T11" s="6"/>
+      <c r="T11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V11" s="6"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
@@ -8797,37 +8869,37 @@
         <v>102</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>2473</v>
+        <v>2474</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I12" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K12" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N12" s="6" t="n">
         <v>0</v>
@@ -8836,10 +8908,10 @@
         <v>0</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R12" s="6" t="n">
         <v>0</v>
@@ -8847,8 +8919,14 @@
       <c r="S12" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T12" s="6" t="s">
-        <v>2477</v>
+      <c r="T12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V12" s="6" t="s">
+        <v>2479</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8859,34 +8937,34 @@
         <v>106</v>
       </c>
       <c r="C13" s="6" t="n">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>2472</v>
+        <v>2474</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>5</v>
+        <v>36</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M13" s="6" t="n">
         <v>0</v>
@@ -8904,12 +8982,18 @@
         <v>0</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="S13" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T13" s="6"/>
+      <c r="T13" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="U13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V13" s="6"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
@@ -8919,34 +9003,34 @@
         <v>110</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>2472</v>
+        <v>2477</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>5</v>
+        <v>36</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J14" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K14" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M14" s="6" t="n">
         <v>0</v>
@@ -8961,7 +9045,7 @@
         <v>0</v>
       </c>
       <c r="Q14" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R14" s="6" t="n">
         <v>0</v>
@@ -8969,7 +9053,13 @@
       <c r="S14" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T14" s="6"/>
+      <c r="T14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V14" s="6"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
@@ -8979,34 +9069,34 @@
         <v>114</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>2472</v>
+        <v>2474</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>5</v>
+        <v>36</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M15" s="6" t="n">
         <v>0</v>
@@ -9024,12 +9114,18 @@
         <v>0</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="S15" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T15" s="6"/>
+      <c r="T15" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="U15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V15" s="6"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
@@ -9039,37 +9135,37 @@
         <v>120</v>
       </c>
       <c r="C16" s="6" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>2473</v>
+        <v>2474</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>5</v>
+        <v>36</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J16" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K16" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L16" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0</v>
@@ -9078,18 +9174,24 @@
         <v>0</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q16" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R16" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S16" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T16" s="6"/>
+      <c r="T16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V16" s="6"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
@@ -9099,37 +9201,37 @@
         <v>124</v>
       </c>
       <c r="C17" s="6" t="n">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>2476</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J17" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K17" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>0</v>
@@ -9144,12 +9246,18 @@
         <v>0</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="S17" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T17" s="6"/>
+      <c r="T17" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="U17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V17" s="6"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
@@ -9162,31 +9270,31 @@
         <v>30</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>2473</v>
+        <v>2474</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>5</v>
+        <v>36</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I18" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J18" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K18" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M18" s="6" t="n">
         <v>0</v>
@@ -9198,10 +9306,10 @@
         <v>0</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q18" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R18" s="6" t="n">
         <v>0</v>
@@ -9209,7 +9317,13 @@
       <c r="S18" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T18" s="6"/>
+      <c r="T18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V18" s="6"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
@@ -9219,34 +9333,34 @@
         <v>130</v>
       </c>
       <c r="C19" s="6" t="n">
+        <v>34</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>2474</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="G19" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="D19" s="6" t="s">
-        <v>2473</v>
-      </c>
-      <c r="E19" s="6" t="n">
-        <v>26</v>
-      </c>
-      <c r="F19" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="G19" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="H19" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M19" s="6" t="n">
         <v>0</v>
@@ -9258,7 +9372,7 @@
         <v>0</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Q19" s="6" t="n">
         <v>0</v>
@@ -9267,9 +9381,15 @@
         <v>0</v>
       </c>
       <c r="S19" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="T19" s="6"/>
+        <v>2</v>
+      </c>
+      <c r="T19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U19" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="V19" s="6"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
@@ -9279,58 +9399,64 @@
         <v>134</v>
       </c>
       <c r="C20" s="6" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D20" s="6" t="s">
         <v>2476</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="F20" s="6" t="n">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="G20" s="6" t="n">
-        <v>0</v>
+        <v>68</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I20" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J20" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K20" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M20" s="6" t="n">
         <v>0</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q20" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R20" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="S20" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="T20" s="6" t="s">
-        <v>2475</v>
+        <v>0</v>
+      </c>
+      <c r="T20" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="U20" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="V20" s="6" t="s">
+        <v>2478</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9341,34 +9467,34 @@
         <v>139</v>
       </c>
       <c r="C21" s="6" t="n">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>2473</v>
+        <v>2474</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M21" s="6" t="n">
         <v>0</v>
@@ -9389,9 +9515,15 @@
         <v>0</v>
       </c>
       <c r="S21" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="T21" s="6"/>
+        <v>0</v>
+      </c>
+      <c r="T21" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U21" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="V21" s="6"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
@@ -9401,31 +9533,31 @@
         <v>143</v>
       </c>
       <c r="C22" s="6" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>2471</v>
+        <v>2473</v>
       </c>
       <c r="E22" s="6" t="n">
         <v>43</v>
       </c>
       <c r="F22" s="6" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="G22" s="6" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="H22" s="6" t="n">
         <v>0</v>
       </c>
       <c r="I22" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J22" s="6" t="n">
         <v>0</v>
       </c>
       <c r="K22" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L22" s="6" t="n">
         <v>0</v>
@@ -9446,13 +9578,19 @@
         <v>0</v>
       </c>
       <c r="R22" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="S22" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T22" s="6" t="s">
-        <v>2475</v>
+      <c r="T22" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="U22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V22" s="6" t="s">
+        <v>2478</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9463,57 +9601,63 @@
         <v>146</v>
       </c>
       <c r="C23" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>2477</v>
+      </c>
+      <c r="E23" s="6" t="n">
+        <v>37</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="G23" s="6" t="n">
         <v>35</v>
       </c>
-      <c r="D23" s="6" t="s">
-        <v>2473</v>
-      </c>
-      <c r="E23" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="F23" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="G23" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="H23" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I23" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J23" s="6" t="n">
         <v>0</v>
       </c>
       <c r="K23" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S23" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T23" s="6"/>
+      <c r="T23" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U23" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V23" s="6"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
@@ -9526,31 +9670,31 @@
         <v>20</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>2472</v>
+        <v>2477</v>
       </c>
       <c r="E24" s="6" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="F24" s="6" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="G24" s="6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I24" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J24" s="6" t="n">
         <v>0</v>
       </c>
       <c r="K24" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="M24" s="6" t="n">
         <v>0</v>
@@ -9565,7 +9709,7 @@
         <v>0</v>
       </c>
       <c r="Q24" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R24" s="6" t="n">
         <v>0</v>
@@ -9573,7 +9717,13 @@
       <c r="S24" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T24" s="6"/>
+      <c r="T24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V24" s="6"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
@@ -9583,37 +9733,37 @@
         <v>153</v>
       </c>
       <c r="C25" s="6" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>2473</v>
+        <v>2474</v>
       </c>
       <c r="E25" s="6" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="G25" s="6" t="n">
-        <v>15</v>
+        <v>33</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I25" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J25" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K25" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L25" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>0</v>
@@ -9622,7 +9772,7 @@
         <v>0</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q25" s="6" t="n">
         <v>0</v>
@@ -9631,9 +9781,15 @@
         <v>0</v>
       </c>
       <c r="S25" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="T25" s="6"/>
+        <v>0</v>
+      </c>
+      <c r="T25" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U25" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="V25" s="6"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
@@ -9643,34 +9799,34 @@
         <v>157</v>
       </c>
       <c r="C26" s="6" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>2472</v>
+        <v>2477</v>
       </c>
       <c r="E26" s="6" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F26" s="6" t="n">
-        <v>5</v>
+        <v>36</v>
       </c>
       <c r="G26" s="6" t="n">
         <v>0</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I26" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J26" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K26" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L26" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M26" s="6" t="n">
         <v>0</v>
@@ -9693,7 +9849,13 @@
       <c r="S26" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T26" s="6"/>
+      <c r="T26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V26" s="6"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
@@ -9703,34 +9865,34 @@
         <v>161</v>
       </c>
       <c r="C27" s="6" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>2473</v>
+        <v>2474</v>
       </c>
       <c r="E27" s="6" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="F27" s="6" t="n">
-        <v>5</v>
+        <v>36</v>
       </c>
       <c r="G27" s="6" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I27" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J27" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K27" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L27" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M27" s="6" t="n">
         <v>0</v>
@@ -9745,15 +9907,21 @@
         <v>0</v>
       </c>
       <c r="Q27" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R27" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="S27" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T27" s="6"/>
+      <c r="T27" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="U27" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V27" s="6"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
@@ -9763,57 +9931,63 @@
         <v>165</v>
       </c>
       <c r="C28" s="6" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>2474</v>
+        <v>2475</v>
       </c>
       <c r="E28" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F28" s="6" t="n">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="G28" s="6" t="n">
-        <v>15</v>
+        <v>48</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I28" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J28" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K28" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L28" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N28" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Q28" s="6" t="n">
         <v>0</v>
       </c>
       <c r="R28" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="S28" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T28" s="6"/>
+        <v>3</v>
+      </c>
+      <c r="T28" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="U28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V28" s="6"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
@@ -9823,34 +9997,34 @@
         <v>167</v>
       </c>
       <c r="C29" s="6" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>2471</v>
+        <v>2473</v>
       </c>
       <c r="E29" s="6" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F29" s="6" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="G29" s="6" t="n">
         <v>0</v>
       </c>
       <c r="H29" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I29" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J29" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K29" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L29" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M29" s="6" t="n">
         <v>0</v>
@@ -9873,7 +10047,13 @@
       <c r="S29" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T29" s="6"/>
+      <c r="T29" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U29" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V29" s="6"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
@@ -9883,37 +10063,37 @@
         <v>171</v>
       </c>
       <c r="C30" s="6" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>2473</v>
+        <v>2476</v>
       </c>
       <c r="E30" s="6" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F30" s="6" t="n">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="G30" s="6" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H30" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I30" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J30" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K30" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L30" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>0</v>
@@ -9933,7 +10113,13 @@
       <c r="S30" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T30" s="6"/>
+      <c r="T30" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U30" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V30" s="6"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
@@ -9943,37 +10129,37 @@
         <v>175</v>
       </c>
       <c r="C31" s="6" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="D31" s="6" t="s">
         <v>2476</v>
       </c>
       <c r="E31" s="6" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="F31" s="6" t="n">
-        <v>10</v>
+        <v>65</v>
       </c>
       <c r="G31" s="6" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H31" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I31" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J31" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K31" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L31" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>0</v>
@@ -9993,8 +10179,14 @@
       <c r="S31" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T31" s="6" t="s">
-        <v>2475</v>
+      <c r="T31" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U31" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V31" s="6" t="s">
+        <v>2478</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10005,58 +10197,64 @@
         <v>179</v>
       </c>
       <c r="C32" s="6" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>2474</v>
+        <v>2475</v>
       </c>
       <c r="E32" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F32" s="6" t="n">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="G32" s="6" t="n">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="H32" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I32" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J32" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K32" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q32" s="6" t="n">
         <v>0</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="S32" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T32" s="6" t="s">
-        <v>2478</v>
+      <c r="T32" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="U32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V32" s="6" t="s">
+        <v>2480</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10067,34 +10265,34 @@
         <v>183</v>
       </c>
       <c r="C33" s="6" t="n">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>2473</v>
+        <v>2476</v>
       </c>
       <c r="E33" s="6" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="F33" s="6" t="n">
-        <v>15</v>
+        <v>54</v>
       </c>
       <c r="G33" s="6" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I33" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J33" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K33" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L33" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M33" s="6" t="n">
         <v>0</v>
@@ -10109,7 +10307,7 @@
         <v>0</v>
       </c>
       <c r="Q33" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R33" s="6" t="n">
         <v>0</v>
@@ -10117,7 +10315,13 @@
       <c r="S33" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T33" s="6"/>
+      <c r="T33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V33" s="6"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
@@ -10127,37 +10331,37 @@
         <v>187</v>
       </c>
       <c r="C34" s="6" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>2473</v>
+        <v>2474</v>
       </c>
       <c r="E34" s="6" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F34" s="6" t="n">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="G34" s="6" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I34" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J34" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K34" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L34" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="N34" s="6" t="n">
         <v>0</v>
@@ -10169,15 +10373,21 @@
         <v>0</v>
       </c>
       <c r="Q34" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R34" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S34" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T34" s="6"/>
+      <c r="T34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V34" s="6"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="6" t="s">
@@ -10187,43 +10397,43 @@
         <v>190</v>
       </c>
       <c r="C35" s="6" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="D35" s="6" t="s">
         <v>2476</v>
       </c>
       <c r="E35" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F35" s="6" t="n">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="G35" s="6" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H35" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I35" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J35" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K35" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L35" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M35" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N35" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O35" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P35" s="6" t="n">
         <v>0</v>
@@ -10237,8 +10447,14 @@
       <c r="S35" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T35" s="6" t="s">
-        <v>2479</v>
+      <c r="T35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V35" s="6" t="s">
+        <v>2481</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10249,37 +10465,37 @@
         <v>194</v>
       </c>
       <c r="C36" s="6" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="D36" s="6" t="s">
         <v>2476</v>
       </c>
       <c r="E36" s="6" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F36" s="6" t="n">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="G36" s="6" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="H36" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I36" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J36" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K36" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N36" s="6" t="n">
         <v>0</v>
@@ -10297,9 +10513,15 @@
         <v>0</v>
       </c>
       <c r="S36" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="T36" s="6"/>
+        <v>0</v>
+      </c>
+      <c r="T36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U36" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="V36" s="6"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="6" t="s">
@@ -10309,37 +10531,37 @@
         <v>198</v>
       </c>
       <c r="C37" s="6" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>2473</v>
+        <v>2474</v>
       </c>
       <c r="E37" s="6" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F37" s="6" t="n">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="G37" s="6" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H37" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I37" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J37" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K37" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L37" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>0</v>
@@ -10348,7 +10570,7 @@
         <v>0</v>
       </c>
       <c r="P37" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q37" s="6" t="n">
         <v>0</v>
@@ -10359,7 +10581,13 @@
       <c r="S37" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T37" s="6"/>
+      <c r="T37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V37" s="6"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="6" t="s">
@@ -10369,34 +10597,34 @@
         <v>202</v>
       </c>
       <c r="C38" s="6" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>2472</v>
+        <v>2477</v>
       </c>
       <c r="E38" s="6" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F38" s="6" t="n">
-        <v>5</v>
+        <v>36</v>
       </c>
       <c r="G38" s="6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H38" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I38" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J38" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K38" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L38" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M38" s="6" t="n">
         <v>0</v>
@@ -10411,7 +10639,7 @@
         <v>0</v>
       </c>
       <c r="Q38" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R38" s="6" t="n">
         <v>0</v>
@@ -10419,7 +10647,13 @@
       <c r="S38" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T38" s="6"/>
+      <c r="T38" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U38" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V38" s="6"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="6" t="s">
@@ -10429,37 +10663,37 @@
         <v>206</v>
       </c>
       <c r="C39" s="6" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>2473</v>
+        <v>2474</v>
       </c>
       <c r="E39" s="6" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F39" s="6" t="n">
+        <v>49</v>
+      </c>
+      <c r="G39" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="G39" s="6" t="n">
-        <v>15</v>
-      </c>
       <c r="H39" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I39" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J39" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K39" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L39" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>0</v>
@@ -10468,7 +10702,7 @@
         <v>0</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q39" s="6" t="n">
         <v>0</v>
@@ -10479,7 +10713,13 @@
       <c r="S39" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T39" s="6"/>
+      <c r="T39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V39" s="6"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="6" t="s">
@@ -10489,34 +10729,34 @@
         <v>210</v>
       </c>
       <c r="C40" s="6" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>2472</v>
+        <v>2477</v>
       </c>
       <c r="E40" s="6" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F40" s="6" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="G40" s="6" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H40" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I40" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J40" s="6" t="n">
         <v>0</v>
       </c>
       <c r="K40" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L40" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="M40" s="6" t="n">
         <v>0</v>
@@ -10531,7 +10771,7 @@
         <v>0</v>
       </c>
       <c r="Q40" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R40" s="6" t="n">
         <v>0</v>
@@ -10539,8 +10779,14 @@
       <c r="S40" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T40" s="6" t="s">
-        <v>2475</v>
+      <c r="T40" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U40" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V40" s="6" t="s">
+        <v>2478</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10551,34 +10797,34 @@
         <v>215</v>
       </c>
       <c r="C41" s="6" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>2472</v>
+        <v>2477</v>
       </c>
       <c r="E41" s="6" t="n">
+        <v>34</v>
+      </c>
+      <c r="F41" s="6" t="n">
         <v>36</v>
       </c>
-      <c r="F41" s="6" t="n">
-        <v>5</v>
-      </c>
       <c r="G41" s="6" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H41" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I41" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J41" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K41" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L41" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M41" s="6" t="n">
         <v>0</v>
@@ -10590,7 +10836,7 @@
         <v>0</v>
       </c>
       <c r="P41" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Q41" s="6" t="n">
         <v>0</v>
@@ -10599,9 +10845,15 @@
         <v>0</v>
       </c>
       <c r="S41" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T41" s="6"/>
+        <v>3</v>
+      </c>
+      <c r="T41" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U41" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V41" s="6"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="6" t="s">
@@ -10611,34 +10863,34 @@
         <v>219</v>
       </c>
       <c r="C42" s="6" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>2472</v>
+        <v>2477</v>
       </c>
       <c r="E42" s="6" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F42" s="6" t="n">
-        <v>5</v>
+        <v>36</v>
       </c>
       <c r="G42" s="6" t="n">
         <v>0</v>
       </c>
       <c r="H42" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I42" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J42" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K42" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L42" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M42" s="6" t="n">
         <v>0</v>
@@ -10661,7 +10913,13 @@
       <c r="S42" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T42" s="6"/>
+      <c r="T42" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U42" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V42" s="6"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="6" t="s">
@@ -10674,7 +10932,7 @@
         <v>0</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>2471</v>
+        <v>2473</v>
       </c>
       <c r="E43" s="6" t="n">
         <v>50</v>
@@ -10721,7 +10979,13 @@
       <c r="S43" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T43" s="6"/>
+      <c r="T43" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U43" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V43" s="6"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="6" t="s">
@@ -10731,34 +10995,34 @@
         <v>223</v>
       </c>
       <c r="C44" s="6" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>2471</v>
+        <v>2473</v>
       </c>
       <c r="E44" s="6" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F44" s="6" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="G44" s="6" t="n">
         <v>0</v>
       </c>
       <c r="H44" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I44" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J44" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K44" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L44" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M44" s="6" t="n">
         <v>0</v>
@@ -10781,7 +11045,13 @@
       <c r="S44" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T44" s="6"/>
+      <c r="T44" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U44" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V44" s="6"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="6" t="s">
@@ -10791,37 +11061,37 @@
         <v>229</v>
       </c>
       <c r="C45" s="6" t="n">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>2474</v>
+        <v>2475</v>
       </c>
       <c r="E45" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F45" s="6" t="n">
+        <v>95</v>
+      </c>
+      <c r="G45" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="H45" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F45" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="G45" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="H45" s="6" t="n">
-        <v>10</v>
-      </c>
       <c r="I45" s="6" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="J45" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K45" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L45" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M45" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N45" s="6" t="n">
         <v>0</v>
@@ -10830,10 +11100,10 @@
         <v>0</v>
       </c>
       <c r="P45" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q45" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R45" s="6" t="n">
         <v>0</v>
@@ -10841,7 +11111,13 @@
       <c r="S45" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T45" s="6"/>
+      <c r="T45" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U45" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V45" s="6"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="6" t="s">
@@ -10851,37 +11127,37 @@
         <v>233</v>
       </c>
       <c r="C46" s="6" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>2476</v>
+        <v>2475</v>
       </c>
       <c r="E46" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F46" s="6" t="n">
-        <v>15</v>
+        <v>74</v>
       </c>
       <c r="G46" s="6" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H46" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I46" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J46" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K46" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L46" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M46" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N46" s="6" t="n">
         <v>0</v>
@@ -10901,7 +11177,13 @@
       <c r="S46" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T46" s="6"/>
+      <c r="T46" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U46" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V46" s="6"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="6" t="s">
@@ -10911,37 +11193,37 @@
         <v>236</v>
       </c>
       <c r="C47" s="6" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>2472</v>
+        <v>2474</v>
       </c>
       <c r="E47" s="6" t="n">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="F47" s="6" t="n">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="G47" s="6" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H47" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I47" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J47" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K47" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L47" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M47" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N47" s="6" t="n">
         <v>0</v>
@@ -10961,8 +11243,14 @@
       <c r="S47" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T47" s="6" t="s">
-        <v>2475</v>
+      <c r="T47" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U47" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V47" s="6" t="s">
+        <v>2478</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10973,22 +11261,22 @@
         <v>239</v>
       </c>
       <c r="C48" s="6" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>2471</v>
+        <v>2473</v>
       </c>
       <c r="E48" s="6" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F48" s="6" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="G48" s="6" t="n">
         <v>0</v>
       </c>
       <c r="H48" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I48" s="6" t="n">
         <v>0</v>
@@ -11023,7 +11311,13 @@
       <c r="S48" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T48" s="6"/>
+      <c r="T48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V48" s="6"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="6" t="s">
@@ -11033,22 +11327,22 @@
         <v>243</v>
       </c>
       <c r="C49" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>2471</v>
+        <v>2473</v>
       </c>
       <c r="E49" s="6" t="n">
         <v>48</v>
       </c>
       <c r="F49" s="6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="G49" s="6" t="n">
         <v>0</v>
       </c>
       <c r="H49" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I49" s="6" t="n">
         <v>0</v>
@@ -11083,7 +11377,13 @@
       <c r="S49" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T49" s="6"/>
+      <c r="T49" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U49" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V49" s="6"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="6" t="s">
@@ -11093,34 +11393,34 @@
         <v>248</v>
       </c>
       <c r="C50" s="6" t="n">
+        <v>34</v>
+      </c>
+      <c r="D50" s="6" t="s">
+        <v>2474</v>
+      </c>
+      <c r="E50" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="F50" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="G50" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="D50" s="6" t="s">
-        <v>2473</v>
-      </c>
-      <c r="E50" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="F50" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="G50" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="H50" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I50" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J50" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K50" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L50" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M50" s="6" t="n">
         <v>0</v>
@@ -11135,15 +11435,21 @@
         <v>0</v>
       </c>
       <c r="Q50" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R50" s="6" t="n">
         <v>0</v>
       </c>
       <c r="S50" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="T50" s="6"/>
+        <v>0</v>
+      </c>
+      <c r="T50" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U50" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="V50" s="6"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="6" t="s">
@@ -11153,22 +11459,22 @@
         <v>252</v>
       </c>
       <c r="C51" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>2471</v>
+        <v>2473</v>
       </c>
       <c r="E51" s="6" t="n">
         <v>49</v>
       </c>
       <c r="F51" s="6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="G51" s="6" t="n">
         <v>0</v>
       </c>
       <c r="H51" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I51" s="6" t="n">
         <v>0</v>
@@ -11203,90 +11509,96 @@
       <c r="S51" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="T51" s="6"/>
+      <c r="T51" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U51" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V51" s="6"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="5" t="s">
-        <v>2480</v>
+        <v>2482</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="s">
-        <v>2481</v>
+        <v>2483</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="s">
-        <v>2482</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="s">
-        <v>2484</v>
+        <v>2486</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="s">
-        <v>2485</v>
+        <v>2487</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="7" t="s">
-        <v>2486</v>
+        <v>2488</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="7" t="s">
-        <v>2487</v>
+        <v>2489</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="7" t="s">
-        <v>2488</v>
+        <v>2490</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="7" t="s">
-        <v>2489</v>
+        <v>2491</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="7" t="s">
-        <v>2490</v>
+        <v>2492</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="s">
-        <v>2491</v>
+        <v>2493</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="7" t="s">
-        <v>2492</v>
+        <v>2494</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="7" t="s">
-        <v>2493</v>
+        <v>2495</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="7" t="s">
-        <v>2494</v>
+        <v>2496</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="7" t="s">
-        <v>2495</v>
+        <v>2497</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T51"/>
+  <autoFilter ref="A1:V51"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Whole-number audit climate weights (75/25 sub-scores), secondary tabs moved right, main tabs renamed
</commit_message>
<xml_diff>
--- a/docs/downloads/warranty-atlas.xlsx
+++ b/docs/downloads/warranty-atlas.xlsx
@@ -45,7 +45,7 @@
     <t xml:space="preserve">Warranty Atlas · workpaper export</t>
   </si>
   <si>
-    <t xml:space="preserve">Built 2026-09-29 from the live Atlas data files.</t>
+    <t xml:space="preserve">Built 2026-09-30 from the live Atlas data files.</t>
   </si>
   <si>
     <t xml:space="preserve">What is in this workbook</t>
@@ -7410,13 +7410,13 @@
     <t xml:space="preserve">Rank</t>
   </si>
   <si>
-    <t xml:space="preserve">Chargeback limits (0-100)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Process and oversight (0-100)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Short audit and chargeback lookback: level 0-3 (weight 20)</t>
+    <t xml:space="preserve">Chargeback limits (75%, of 75)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Process and oversight (25%, of 25)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Short audit and chargeback lookback: level 0-3 (weight 21)</t>
   </si>
   <si>
     <t xml:space="preserve">Limits on extrapolating audit results: level 0-3 (weight 15)</t>
@@ -7434,28 +7434,28 @@
     <t xml:space="preserve">Chargeback held while the dealer appeals: level 0-3 (weight 15)</t>
   </si>
   <si>
-    <t xml:space="preserve">Advance written notice of audit: level 0-3 (weight 2.5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Must tell the dealer why it was selected: level 0-3 (weight 2.5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Written reasons required before a chargeback: level 0-3 (weight 2.5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dealer response or cure period: level 0-3 (weight 2.5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Internal appeal required: level 0-3 (weight 2.5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cap on how often audits can occur: level 0-3 (weight 2.5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rate validation limited to the dealer's submission: level 0-3 (weight 5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Specific consequence for improper audits: level 0-3 (weight 6)</t>
+    <t xml:space="preserve">Advance written notice of audit: level 0-3 (weight 3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Must tell the dealer why it was selected: level 0-3 (weight 3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Written reasons required before a chargeback: level 0-3 (weight 3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dealer response or cure period: level 0-3 (weight 3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Internal appeal required: level 0-3 (weight 3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cap on how often audits can occur: level 0-3 (weight 3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rate validation limited to the dealer's submission: level 0-3 (weight 3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Specific consequence for improper audits: level 0-3 (weight 4)</t>
   </si>
   <si>
     <t xml:space="preserve">Distributor-franchised</t>
@@ -7494,7 +7494,7 @@
     <t xml:space="preserve">Points = weight × level ÷ 3. Score = sum of points (0–100). Weights are a judgment call about how much each limit constrains audits and chargebacks. Levels are read from the statute text.</t>
   </si>
   <si>
-    <t xml:space="preserve">Short audit and chargeback lookback (weight 20; How far back and how much can be charged back): level 3: 6 months or less; level 2: 9 months; level 1: 12 months; level 0: No limit in statute, or over 12 months</t>
+    <t xml:space="preserve">Short audit and chargeback lookback (weight 21; How far back and how much can be charged back): level 3: 6 months or less; level 2: 9 months; level 1: 12 months; level 0: No limit in statute, or over 12 months</t>
   </si>
   <si>
     <t xml:space="preserve">Limits on extrapolating audit results (weight 15; How far back and how much can be charged back): level 3: Prohibited; level 2: Restricted (e.g., only from a valid random sample); level 0: Not addressed</t>
@@ -7512,25 +7512,25 @@
     <t xml:space="preserve">Chargeback held while the dealer appeals (weight 15; When a chargeback can be collected): level 3: Applies; level 0: Not in statute</t>
   </si>
   <si>
-    <t xml:space="preserve">Advance written notice of audit (weight 2.5; Audit process steps): level 3: Applies; level 0: Not in statute</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Must tell the dealer why it was selected (weight 2.5; Audit process steps): level 3: Applies; level 0: Not in statute</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Written reasons required before a chargeback (weight 2.5; Audit process steps): level 3: Applies; level 0: Not in statute</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dealer response or cure period (weight 2.5; Audit process steps): level 3: 60 days or more; level 2: 30 to 59 days; level 1: Under 30 days; level 0: None in statute</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Internal appeal required (weight 2.5; Audit process steps): level 3: Applies; level 0: Not in statute</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cap on how often audits can occur (weight 2.5; Audit process steps): level 3: At most one audit per 12 months; level 2: Cap allows more than one audit a year (e.g., one per 9 months); level 0: No cap in statute</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rate validation limited to the dealer's submission (weight 5; Rate validation and consequences): level 3: Only the dealer's own ROs or a single accuracy objection; level 0: Not limited in statute</t>
+    <t xml:space="preserve">Advance written notice of audit (weight 3; Audit process steps): level 3: Applies; level 0: Not in statute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Must tell the dealer why it was selected (weight 3; Audit process steps): level 3: Applies; level 0: Not in statute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Written reasons required before a chargeback (weight 3; Audit process steps): level 3: Applies; level 0: Not in statute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dealer response or cure period (weight 3; Audit process steps): level 3: 60 days or more; level 2: 30 to 59 days; level 1: Under 30 days; level 0: None in statute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Internal appeal required (weight 3; Audit process steps): level 3: Applies; level 0: Not in statute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cap on how often audits can occur (weight 3; Audit process steps): level 3: At most one audit per 12 months; level 2: Cap allows more than one audit a year (e.g., one per 9 months); level 0: No cap in statute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rate validation limited to the dealer's submission (weight 3; Rate validation and consequences): level 3: Only the dealer's own ROs or a single accuracy objection; level 0: Not limited in statute</t>
   </si>
   <si>
     <t xml:space="preserve">Tiers: Very high 50+; High 40–49; Elevated 30–39; Moderate 20–29; Low under 20</t>
@@ -8207,7 +8207,7 @@
         <v>38</v>
       </c>
       <c r="C2" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>2473</v>
@@ -8216,10 +8216,10 @@
         <v>47</v>
       </c>
       <c r="F2" s="6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G2" s="6" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H2" s="6" t="n">
         <v>1</v>
@@ -8279,10 +8279,10 @@
         <v>2474</v>
       </c>
       <c r="E3" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="F3" s="6" t="n">
         <v>31</v>
-      </c>
-      <c r="F3" s="6" t="n">
-        <v>41</v>
       </c>
       <c r="G3" s="6" t="n">
         <v>0</v>
@@ -8345,10 +8345,10 @@
         <v>2474</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="G4" s="6" t="n">
         <v>0</v>
@@ -8411,10 +8411,10 @@
         <v>2474</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="G5" s="6" t="n">
         <v>0</v>
@@ -8471,7 +8471,7 @@
         <v>69</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>2475</v>
@@ -8480,10 +8480,10 @@
         <v>2</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>79</v>
+        <v>59</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>51</v>
+        <v>16</v>
       </c>
       <c r="H6" s="6" t="n">
         <v>2</v>
@@ -8537,7 +8537,7 @@
         <v>74</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>2476</v>
@@ -8546,10 +8546,10 @@
         <v>14</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="H7" s="6" t="n">
         <v>2</v>
@@ -8603,7 +8603,7 @@
         <v>80</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>2477</v>
@@ -8612,10 +8612,10 @@
         <v>41</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H8" s="6" t="n">
         <v>1</v>
@@ -8671,16 +8671,16 @@
         <v>87</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>2476</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>54</v>
+        <v>41</v>
       </c>
       <c r="G9" s="6" t="n">
         <v>0</v>
@@ -8737,7 +8737,7 @@
         <v>92</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>2475</v>
@@ -8746,10 +8746,10 @@
         <v>3</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>62</v>
+        <v>46</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>78</v>
+        <v>18</v>
       </c>
       <c r="H10" s="6" t="n">
         <v>1</v>
@@ -8803,7 +8803,7 @@
         <v>97</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>2476</v>
@@ -8812,10 +8812,10 @@
         <v>11</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H11" s="6" t="n">
         <v>1</v>
@@ -8869,19 +8869,19 @@
         <v>102</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>2474</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="H12" s="6" t="n">
         <v>1</v>
@@ -8937,19 +8937,19 @@
         <v>106</v>
       </c>
       <c r="C13" s="6" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>2474</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="H13" s="6" t="n">
         <v>1</v>
@@ -9003,19 +9003,19 @@
         <v>110</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>2477</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H14" s="6" t="n">
         <v>1</v>
@@ -9069,19 +9069,19 @@
         <v>114</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>2474</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="H15" s="6" t="n">
         <v>1</v>
@@ -9135,19 +9135,19 @@
         <v>120</v>
       </c>
       <c r="C16" s="6" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>2474</v>
       </c>
       <c r="E16" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="F16" s="6" t="n">
         <v>27</v>
       </c>
-      <c r="F16" s="6" t="n">
-        <v>36</v>
-      </c>
       <c r="G16" s="6" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="H16" s="6" t="n">
         <v>1</v>
@@ -9201,7 +9201,7 @@
         <v>124</v>
       </c>
       <c r="C17" s="6" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>2476</v>
@@ -9210,10 +9210,10 @@
         <v>9</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="H17" s="6" t="n">
         <v>1</v>
@@ -9267,19 +9267,19 @@
         <v>127</v>
       </c>
       <c r="C18" s="6" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>2474</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="H18" s="6" t="n">
         <v>1</v>
@@ -9333,19 +9333,19 @@
         <v>130</v>
       </c>
       <c r="C19" s="6" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D19" s="6" t="s">
         <v>2474</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F19" s="6" t="n">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="G19" s="6" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="H19" s="6" t="n">
         <v>1</v>
@@ -9399,19 +9399,19 @@
         <v>134</v>
       </c>
       <c r="C20" s="6" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D20" s="6" t="s">
         <v>2476</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F20" s="6" t="n">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="G20" s="6" t="n">
-        <v>68</v>
+        <v>15</v>
       </c>
       <c r="H20" s="6" t="n">
         <v>1</v>
@@ -9467,19 +9467,19 @@
         <v>139</v>
       </c>
       <c r="C21" s="6" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D21" s="6" t="s">
         <v>2474</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="H21" s="6" t="n">
         <v>2</v>
@@ -9533,7 +9533,7 @@
         <v>143</v>
       </c>
       <c r="C22" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D22" s="6" t="s">
         <v>2473</v>
@@ -9542,10 +9542,10 @@
         <v>43</v>
       </c>
       <c r="F22" s="6" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="G22" s="6" t="n">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="H22" s="6" t="n">
         <v>0</v>
@@ -9601,19 +9601,19 @@
         <v>146</v>
       </c>
       <c r="C23" s="6" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>2477</v>
+        <v>2474</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="G23" s="6" t="n">
-        <v>35</v>
+        <v>11</v>
       </c>
       <c r="H23" s="6" t="n">
         <v>1</v>
@@ -9667,7 +9667,7 @@
         <v>149</v>
       </c>
       <c r="C24" s="6" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D24" s="6" t="s">
         <v>2477</v>
@@ -9676,10 +9676,10 @@
         <v>42</v>
       </c>
       <c r="F24" s="6" t="n">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="G24" s="6" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H24" s="6" t="n">
         <v>1</v>
@@ -9733,7 +9733,7 @@
         <v>153</v>
       </c>
       <c r="C25" s="6" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D25" s="6" t="s">
         <v>2474</v>
@@ -9742,10 +9742,10 @@
         <v>20</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="G25" s="6" t="n">
-        <v>33</v>
+        <v>7</v>
       </c>
       <c r="H25" s="6" t="n">
         <v>1</v>
@@ -9808,7 +9808,7 @@
         <v>38</v>
       </c>
       <c r="F26" s="6" t="n">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="G26" s="6" t="n">
         <v>0</v>
@@ -9865,19 +9865,19 @@
         <v>161</v>
       </c>
       <c r="C27" s="6" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D27" s="6" t="s">
         <v>2474</v>
       </c>
       <c r="E27" s="6" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F27" s="6" t="n">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="G27" s="6" t="n">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="H27" s="6" t="n">
         <v>1</v>
@@ -9940,10 +9940,10 @@
         <v>5</v>
       </c>
       <c r="F28" s="6" t="n">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="G28" s="6" t="n">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="H28" s="6" t="n">
         <v>1</v>
@@ -10006,7 +10006,7 @@
         <v>44</v>
       </c>
       <c r="F29" s="6" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G29" s="6" t="n">
         <v>0</v>
@@ -10069,10 +10069,10 @@
         <v>2476</v>
       </c>
       <c r="E30" s="6" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F30" s="6" t="n">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="G30" s="6" t="n">
         <v>0</v>
@@ -10129,7 +10129,7 @@
         <v>175</v>
       </c>
       <c r="C31" s="6" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D31" s="6" t="s">
         <v>2476</v>
@@ -10138,7 +10138,7 @@
         <v>7</v>
       </c>
       <c r="F31" s="6" t="n">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="G31" s="6" t="n">
         <v>0</v>
@@ -10197,7 +10197,7 @@
         <v>179</v>
       </c>
       <c r="C32" s="6" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D32" s="6" t="s">
         <v>2475</v>
@@ -10206,10 +10206,10 @@
         <v>6</v>
       </c>
       <c r="F32" s="6" t="n">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="G32" s="6" t="n">
-        <v>38</v>
+        <v>9</v>
       </c>
       <c r="H32" s="6" t="n">
         <v>1</v>
@@ -10265,7 +10265,7 @@
         <v>183</v>
       </c>
       <c r="C33" s="6" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D33" s="6" t="s">
         <v>2476</v>
@@ -10274,10 +10274,10 @@
         <v>12</v>
       </c>
       <c r="F33" s="6" t="n">
-        <v>54</v>
+        <v>41</v>
       </c>
       <c r="G33" s="6" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H33" s="6" t="n">
         <v>3</v>
@@ -10331,19 +10331,19 @@
         <v>187</v>
       </c>
       <c r="C34" s="6" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>2474</v>
+        <v>2476</v>
       </c>
       <c r="E34" s="6" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F34" s="6" t="n">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="G34" s="6" t="n">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="H34" s="6" t="n">
         <v>2</v>
@@ -10397,7 +10397,7 @@
         <v>190</v>
       </c>
       <c r="C35" s="6" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D35" s="6" t="s">
         <v>2476</v>
@@ -10406,10 +10406,10 @@
         <v>10</v>
       </c>
       <c r="F35" s="6" t="n">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="G35" s="6" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H35" s="6" t="n">
         <v>1</v>
@@ -10465,7 +10465,7 @@
         <v>194</v>
       </c>
       <c r="C36" s="6" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D36" s="6" t="s">
         <v>2476</v>
@@ -10474,10 +10474,10 @@
         <v>8</v>
       </c>
       <c r="F36" s="6" t="n">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="G36" s="6" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="H36" s="6" t="n">
         <v>1</v>
@@ -10531,19 +10531,19 @@
         <v>198</v>
       </c>
       <c r="C37" s="6" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D37" s="6" t="s">
         <v>2474</v>
       </c>
       <c r="E37" s="6" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F37" s="6" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="G37" s="6" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H37" s="6" t="n">
         <v>1</v>
@@ -10597,19 +10597,19 @@
         <v>202</v>
       </c>
       <c r="C38" s="6" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D38" s="6" t="s">
         <v>2477</v>
       </c>
       <c r="E38" s="6" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F38" s="6" t="n">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="G38" s="6" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H38" s="6" t="n">
         <v>1</v>
@@ -10663,19 +10663,19 @@
         <v>206</v>
       </c>
       <c r="C39" s="6" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>2474</v>
+        <v>2476</v>
       </c>
       <c r="E39" s="6" t="n">
         <v>18</v>
       </c>
       <c r="F39" s="6" t="n">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="G39" s="6" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H39" s="6" t="n">
         <v>2</v>
@@ -10729,7 +10729,7 @@
         <v>210</v>
       </c>
       <c r="C40" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D40" s="6" t="s">
         <v>2477</v>
@@ -10738,10 +10738,10 @@
         <v>40</v>
       </c>
       <c r="F40" s="6" t="n">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="G40" s="6" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H40" s="6" t="n">
         <v>1</v>
@@ -10797,19 +10797,19 @@
         <v>215</v>
       </c>
       <c r="C41" s="6" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>2477</v>
+        <v>2474</v>
       </c>
       <c r="E41" s="6" t="n">
         <v>34</v>
       </c>
       <c r="F41" s="6" t="n">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="G41" s="6" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H41" s="6" t="n">
         <v>1</v>
@@ -10872,7 +10872,7 @@
         <v>39</v>
       </c>
       <c r="F42" s="6" t="n">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="G42" s="6" t="n">
         <v>0</v>
@@ -11004,7 +11004,7 @@
         <v>45</v>
       </c>
       <c r="F44" s="6" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G44" s="6" t="n">
         <v>0</v>
@@ -11061,7 +11061,7 @@
         <v>229</v>
       </c>
       <c r="C45" s="6" t="n">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D45" s="6" t="s">
         <v>2475</v>
@@ -11070,10 +11070,10 @@
         <v>1</v>
       </c>
       <c r="F45" s="6" t="n">
-        <v>95</v>
+        <v>71</v>
       </c>
       <c r="G45" s="6" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="H45" s="6" t="n">
         <v>3</v>
@@ -11127,7 +11127,7 @@
         <v>233</v>
       </c>
       <c r="C46" s="6" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D46" s="6" t="s">
         <v>2475</v>
@@ -11136,7 +11136,7 @@
         <v>4</v>
       </c>
       <c r="F46" s="6" t="n">
-        <v>74</v>
+        <v>56</v>
       </c>
       <c r="G46" s="6" t="n">
         <v>0</v>
@@ -11199,10 +11199,10 @@
         <v>2474</v>
       </c>
       <c r="E47" s="6" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F47" s="6" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="G47" s="6" t="n">
         <v>0</v>
@@ -11261,7 +11261,7 @@
         <v>239</v>
       </c>
       <c r="C48" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D48" s="6" t="s">
         <v>2473</v>
@@ -11270,7 +11270,7 @@
         <v>46</v>
       </c>
       <c r="F48" s="6" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="G48" s="6" t="n">
         <v>0</v>
@@ -11336,7 +11336,7 @@
         <v>48</v>
       </c>
       <c r="F49" s="6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G49" s="6" t="n">
         <v>0</v>
@@ -11393,19 +11393,19 @@
         <v>248</v>
       </c>
       <c r="C50" s="6" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D50" s="6" t="s">
         <v>2474</v>
       </c>
       <c r="E50" s="6" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="G50" s="6" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="H50" s="6" t="n">
         <v>1</v>
@@ -11468,7 +11468,7 @@
         <v>49</v>
       </c>
       <c r="F51" s="6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G51" s="6" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Governing Bodies tab with agency and statute links; one source per fact on state pages; build-time consistency check
</commit_message>
<xml_diff>
--- a/docs/downloads/warranty-atlas.xlsx
+++ b/docs/downloads/warranty-atlas.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit fields" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rate sample rules" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Law dates" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Who governs" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governing bodies" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly log" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="News" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit procedures" sheetId="10" state="visible" r:id="rId10"/>
@@ -25,7 +25,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Audit fields'!$A$1:$AN$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Rate sample rules'!$A$1:$L$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Law dates'!$A$1:$M$51</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Who governs'!$A$1:$H$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Governing bodies'!$A$1:$J$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Weekly log'!$A$1:$J$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'News'!$A$1:$J$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Audit procedures'!$A$1:$X$51</definedName>
@@ -549,7 +549,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Who governs: whether the rules come from the statute alone or also an agency rule, the agency, and where a dealer takes a dispute.</t>
+          <t>Governing bodies: whether the rules come from the statute alone or also an agency rule, the agency and its website, and where a dealer takes a dispute.</t>
         </is>
       </c>
     </row>
@@ -39616,7 +39616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:J51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -39625,8 +39625,10 @@
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="50" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -39662,12 +39664,22 @@
       </c>
       <c r="G1" s="4" t="inlineStr">
         <is>
+          <t>Agency website</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
           <t>Dispute forum type</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>Where disputes go</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Statute source</t>
         </is>
       </c>
     </row>
@@ -39700,12 +39712,22 @@
       </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
+          <t>https://dmv.alaska.gov/</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
           <t>Court</t>
         </is>
       </c>
-      <c r="H2" s="6" t="inlineStr">
+      <c r="I2" s="6" t="inlineStr">
         <is>
           <t>Court</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="inlineStr">
+        <is>
+          <t>https://www.akleg.gov/basis/statutes.asp?media=print&amp;secStart=45.25.200&amp;secEnd=45.25.320</t>
         </is>
       </c>
     </row>
@@ -39738,12 +39760,22 @@
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
+          <t>https://www.revenue.alabama.gov/division/motor-vehicle/</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
           <t>Court</t>
         </is>
       </c>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="I3" s="6" t="inlineStr">
         <is>
           <t>Court</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>https://alison.legislature.state.al.us/code-of-alabama?section=8-20-7</t>
         </is>
       </c>
     </row>
@@ -39776,12 +39808,22 @@
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
+          <t>https://labor.arkansas.gov/licensing/motor-vehicle-commission/</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
           <t>Agency or court</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="I4" s="6" t="inlineStr">
         <is>
           <t>Commission (chargeback appeals) or court</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>https://arkleg.state.ar.us/Acts/FTPDocument?path=%2FACTS%2F2021R%2FPublic%2F&amp;file=1077.pdf&amp;ddBienniumSession=2021%2F2021R</t>
         </is>
       </c>
     </row>
@@ -39814,12 +39856,22 @@
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
+          <t>https://azdot.gov/motor-vehicles</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
           <t>Agency</t>
         </is>
       </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="I5" s="6" t="inlineStr">
         <is>
           <t>ADOT director (administrative law judge hearing)</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>https://www.azleg.gov/ars/28/04451.htm</t>
         </is>
       </c>
     </row>
@@ -39856,12 +39908,22 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
+          <t>https://www.nmvb.ca.gov/</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
           <t>Agency</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="I6" s="6" t="inlineStr">
         <is>
           <t>New Motor Vehicle Board</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>https://leginfo.legislature.ca.gov/faces/codes_displaySection.xhtml?lawCode=VEH&amp;sectionNum=3065</t>
         </is>
       </c>
     </row>
@@ -39894,12 +39956,22 @@
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
+          <t>https://sbg.colorado.gov/auto-industry</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
           <t>Agency or court</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="I7" s="6" t="inlineStr">
         <is>
           <t>DOR executive director or court</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>https://content.leg.colorado.gov/sites/default/files/2023a_078_signed.pdf</t>
         </is>
       </c>
     </row>
@@ -39932,12 +40004,22 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
+          <t>https://portal.ct.gov/dmv</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
           <t>Agency</t>
         </is>
       </c>
-      <c r="H8" s="6" t="inlineStr">
+      <c r="I8" s="6" t="inlineStr">
         <is>
           <t>DMV Commissioner</t>
+        </is>
+      </c>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>https://www.cga.ct.gov/current/pub/chap_739.htm</t>
         </is>
       </c>
     </row>
@@ -39970,12 +40052,22 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
+          <t>https://depsc.delaware.gov/</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
           <t>Agency</t>
         </is>
       </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="I9" s="6" t="inlineStr">
         <is>
           <t>Public Service Commission</t>
+        </is>
+      </c>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>https://delcode.delaware.gov/title6/c049/index.html</t>
         </is>
       </c>
     </row>
@@ -40008,12 +40100,22 @@
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
+          <t>https://www.flhsmv.gov/</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
           <t>Agency or court</t>
         </is>
       </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="I10" s="6" t="inlineStr">
         <is>
           <t>DHSMV proceeding or court</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
+          <t>http://www.leg.state.fl.us/statutes/index.cfm?App_mode=Display_Statute&amp;URL=0300-0399/0320/Sections/0320.696.html</t>
         </is>
       </c>
     </row>
@@ -40046,12 +40148,22 @@
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
+          <t>https://dor.georgia.gov/</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
           <t>Agency</t>
         </is>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>Revenue commissioner</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>https://law.justia.com/codes/georgia/title-10/chapter-1/article-22/part-3/section-10-1-641/</t>
         </is>
       </c>
     </row>
@@ -40084,12 +40196,22 @@
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
+          <t>https://cca.hawaii.gov/pvl/boards/motorvehicle/</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
           <t>Agency</t>
         </is>
       </c>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="I12" s="6" t="inlineStr">
         <is>
           <t>DCCA administrative hearing</t>
+        </is>
+      </c>
+      <c r="J12" s="6" t="inlineStr">
+        <is>
+          <t>https://data.capitol.hawaii.gov/hrscurrent/Vol10_Ch0436-0474/HRS0437/HRS_0437-0056.htm (also HRS_0437-0028.htm, HRS_0437-0057.htm, HRS_0437-0051.htm; legislature data host, files dated 1/5/2026)</t>
         </is>
       </c>
     </row>
@@ -40122,12 +40244,22 @@
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
+          <t>https://iowadot.gov/dmv-services</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
           <t>Agency</t>
         </is>
       </c>
-      <c r="H13" s="6" t="inlineStr">
+      <c r="I13" s="6" t="inlineStr">
         <is>
           <t>DOT contested case</t>
+        </is>
+      </c>
+      <c r="J13" s="6" t="inlineStr">
+        <is>
+          <t>https://www.legis.iowa.gov/docs/code/322A.pdf (Iowa Code 2026; ch. 322 at https://www.legis.iowa.gov/docs/code/322.pdf)</t>
         </is>
       </c>
     </row>
@@ -40160,12 +40292,22 @@
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
+          <t>https://itd.idaho.gov/dmv/</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
           <t>Agency or court</t>
         </is>
       </c>
-      <c r="H14" s="6" t="inlineStr">
+      <c r="I14" s="6" t="inlineStr">
         <is>
           <t>ITD contested case (after mediation) or court</t>
+        </is>
+      </c>
+      <c r="J14" s="6" t="inlineStr">
+        <is>
+          <t>https://legislature.idaho.gov/wp-content/uploads/statutesrules/idstat/Title49/T49CH16.pdf (section page: https://legislature.idaho.gov/statutesrules/idstat/title49/t49ch16/sect49-1626/)</t>
         </is>
       </c>
     </row>
@@ -40198,12 +40340,22 @@
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
+          <t>https://www.ilsos.gov/departments/administrative-hearings/mvrb.html</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
           <t>Agency or court</t>
         </is>
       </c>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="I15" s="6" t="inlineStr">
         <is>
           <t>Review Board, arbitration or court</t>
+        </is>
+      </c>
+      <c r="J15" s="6" t="inlineStr">
+        <is>
+          <t>https://www.ilga.gov/Documents/legislation/ilcs/documents/081507100K6.htm (full Act: https://www.ilga.gov/legislation/ilcs/ilcs3.asp?ActID=2382&amp;ChapterID=67)</t>
         </is>
       </c>
     </row>
@@ -40236,12 +40388,22 @@
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
+          <t>https://www.in.gov/sos/dealer/</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
           <t>Agency</t>
         </is>
       </c>
-      <c r="H16" s="6" t="inlineStr">
+      <c r="I16" s="6" t="inlineStr">
         <is>
           <t>Secretary of State</t>
+        </is>
+      </c>
+      <c r="J16" s="6" t="inlineStr">
+        <is>
+          <t>https://iga.in.gov/ic/2026/Title_9.pdf (Indiana Code 2026, Title 9; ch. 9-32-13)</t>
         </is>
       </c>
     </row>
@@ -40274,12 +40436,22 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
+          <t>https://www.ksrevenue.gov/dovdealer.html</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
           <t>Agency</t>
         </is>
       </c>
-      <c r="H17" s="6" t="inlineStr">
+      <c r="I17" s="6" t="inlineStr">
         <is>
           <t>Director of Vehicles</t>
+        </is>
+      </c>
+      <c r="J17" s="6" t="inlineStr">
+        <is>
+          <t>https://ksrevisor.gov/statutes/chapters/ch08/008_024_0015.html</t>
         </is>
       </c>
     </row>
@@ -40312,12 +40484,22 @@
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
+          <t>https://mvc.ky.gov/</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
           <t>Agency</t>
         </is>
       </c>
-      <c r="H18" s="6" t="inlineStr">
+      <c r="I18" s="6" t="inlineStr">
         <is>
           <t>Commission hearing</t>
+        </is>
+      </c>
+      <c r="J18" s="6" t="inlineStr">
+        <is>
+          <t>https://apps.legislature.ky.gov/law/statutes/statute.aspx?id=57533 (KRS 190.046, effective July 15, 2026)</t>
         </is>
       </c>
     </row>
@@ -40350,12 +40532,22 @@
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
+          <t>https://www.lmvc.la.gov/</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
           <t>Agency</t>
         </is>
       </c>
-      <c r="H19" s="6" t="inlineStr">
+      <c r="I19" s="6" t="inlineStr">
         <is>
           <t>Commission</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="inlineStr">
+        <is>
+          <t>https://legis.la.gov/Legis/LawPrint.aspx?d=321503</t>
         </is>
       </c>
     </row>
@@ -40386,14 +40578,20 @@
           <t>None (enforced by dealer lawsuits)</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr">
+      <c r="G20" s="6" t="inlineStr"/>
+      <c r="H20" s="6" t="inlineStr">
         <is>
           <t>Court</t>
         </is>
       </c>
-      <c r="H20" s="6" t="inlineStr">
+      <c r="I20" s="6" t="inlineStr">
         <is>
           <t>Court</t>
+        </is>
+      </c>
+      <c r="J20" s="6" t="inlineStr">
+        <is>
+          <t>https://malegislature.gov/Laws/GeneralLaws/PartI/TitleXV/Chapter93B/Section9</t>
         </is>
       </c>
     </row>
@@ -40426,12 +40624,22 @@
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
+          <t>https://mva.maryland.gov/</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
           <t>Agency or court</t>
         </is>
       </c>
-      <c r="H21" s="6" t="inlineStr">
+      <c r="I21" s="6" t="inlineStr">
         <is>
           <t>MVA or court</t>
+        </is>
+      </c>
+      <c r="J21" s="6" t="inlineStr">
+        <is>
+          <t>https://mgaleg.maryland.gov/mgawebsite/Laws/StatuteText?article=gtr&amp;section=15-212&amp;enactments=false</t>
         </is>
       </c>
     </row>
@@ -40464,12 +40672,22 @@
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
+          <t>https://www.maine.gov/sos/bmv/more-bmv/motor-vehicle-franchise-board</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
           <t>Agency or court</t>
         </is>
       </c>
-      <c r="H22" s="6" t="inlineStr">
+      <c r="I22" s="6" t="inlineStr">
         <is>
           <t>Franchise Board or court</t>
+        </is>
+      </c>
+      <c r="J22" s="6" t="inlineStr">
+        <is>
+          <t>https://legislature.maine.gov/statutes/10/title10sec1176.html</t>
         </is>
       </c>
     </row>
@@ -40500,14 +40718,20 @@
           <t>None (enforced by dealer lawsuits)</t>
         </is>
       </c>
-      <c r="G23" s="6" t="inlineStr">
+      <c r="G23" s="6" t="inlineStr"/>
+      <c r="H23" s="6" t="inlineStr">
         <is>
           <t>Court</t>
         </is>
       </c>
-      <c r="H23" s="6" t="inlineStr">
+      <c r="I23" s="6" t="inlineStr">
         <is>
           <t>Court</t>
+        </is>
+      </c>
+      <c r="J23" s="6" t="inlineStr">
+        <is>
+          <t>https://www.legislature.mi.gov/Laws/MCL?objectName=mcl-445-1577 ; https://www.legislature.mi.gov/Laws/MCL?objectName=mcl-445-1577a</t>
         </is>
       </c>
     </row>
@@ -40540,12 +40764,22 @@
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
+          <t>https://www.ag.state.mn.us/</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
           <t>Court</t>
         </is>
       </c>
-      <c r="H24" s="6" t="inlineStr">
+      <c r="I24" s="6" t="inlineStr">
         <is>
           <t>Court</t>
+        </is>
+      </c>
+      <c r="J24" s="6" t="inlineStr">
+        <is>
+          <t>https://www.revisor.mn.gov/statutes/cite/80E.041</t>
         </is>
       </c>
     </row>
@@ -40578,12 +40812,22 @@
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
+          <t>https://dor.mo.gov/motor-vehicle/</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
           <t>Agency</t>
         </is>
       </c>
-      <c r="H25" s="6" t="inlineStr">
+      <c r="I25" s="6" t="inlineStr">
         <is>
           <t>Administrative Hearing Commission</t>
+        </is>
+      </c>
+      <c r="J25" s="6" t="inlineStr">
+        <is>
+          <t>https://revisor.mo.gov/main/OneSection.aspx?section=407.828</t>
         </is>
       </c>
     </row>
@@ -40616,12 +40860,22 @@
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
+          <t>https://www.mmvc.ms.gov/</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
           <t>Agency</t>
         </is>
       </c>
-      <c r="H26" s="6" t="inlineStr">
+      <c r="I26" s="6" t="inlineStr">
         <is>
           <t>Commission</t>
+        </is>
+      </c>
+      <c r="J26" s="6" t="inlineStr">
+        <is>
+          <t>https://billstatus.ls.state.ms.us/documents/2021/html/HB/0700-0799/HB0746SG.htm (enrolled HB 746, Laws 2021 ch. 315). Current code mirror: https://law.justia.com/codes/mississippi/title-63/chapter-17/distribution-and-sales/ (2025 code)</t>
         </is>
       </c>
     </row>
@@ -40654,12 +40908,22 @@
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
+          <t>https://mvdmt.gov/</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
           <t>Agency or court</t>
         </is>
       </c>
-      <c r="H27" s="6" t="inlineStr">
+      <c r="I27" s="6" t="inlineStr">
         <is>
           <t>Department or court</t>
+        </is>
+      </c>
+      <c r="J27" s="6" t="inlineStr">
+        <is>
+          <t>https://mca.legmt.gov/bills/mca/title_0610/chapter_0040/part_0020/section_0130/0610-0040-0020-0130.html</t>
         </is>
       </c>
     </row>
@@ -40692,12 +40956,22 @@
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
+          <t>https://www.ncdot.gov/dmv/</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
           <t>Agency</t>
         </is>
       </c>
-      <c r="H28" s="6" t="inlineStr">
+      <c r="I28" s="6" t="inlineStr">
         <is>
           <t>DMV Commissioner</t>
+        </is>
+      </c>
+      <c r="J28" s="6" t="inlineStr">
+        <is>
+          <t>https://www.ncleg.gov/EnactedLegislation/Statutes/HTML/BySection/Chapter_20/GS_20-305.1.html</t>
         </is>
       </c>
     </row>
@@ -40730,12 +41004,22 @@
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
+          <t>https://www.dot.nd.gov/</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="inlineStr">
+        <is>
           <t>Court</t>
         </is>
       </c>
-      <c r="H29" s="6" t="inlineStr">
+      <c r="I29" s="6" t="inlineStr">
         <is>
           <t>Court</t>
+        </is>
+      </c>
+      <c r="J29" s="6" t="inlineStr">
+        <is>
+          <t>https://www.ndlegis.gov/cencode/t51c07.pdf ; session law: https://ndlegis.gov/assembly/69-2025/session-laws/documents/SALES.pdf (ch. 463)</t>
         </is>
       </c>
     </row>
@@ -40768,12 +41052,22 @@
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
+          <t>https://mvilb.nebraska.gov/</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
           <t>Agency</t>
         </is>
       </c>
-      <c r="H30" s="6" t="inlineStr">
+      <c r="I30" s="6" t="inlineStr">
         <is>
           <t>Board</t>
+        </is>
+      </c>
+      <c r="J30" s="6" t="inlineStr">
+        <is>
+          <t>https://nebraskalegislature.gov/laws/statutes.php?statute=60-1438</t>
         </is>
       </c>
     </row>
@@ -40806,12 +41100,22 @@
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
+          <t>https://www.dos.nh.gov/commissions-boards-bureaus/motor-vehicle-industry-board</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
           <t>Agency</t>
         </is>
       </c>
-      <c r="H31" s="6" t="inlineStr">
+      <c r="I31" s="6" t="inlineStr">
         <is>
           <t>Board</t>
+        </is>
+      </c>
+      <c r="J31" s="6" t="inlineStr">
+        <is>
+          <t>https://gc.nh.gov/rsa/html/XXXI/357-C/357-C-5.htm</t>
         </is>
       </c>
     </row>
@@ -40842,14 +41146,20 @@
           <t>None (enforced by dealer lawsuits)</t>
         </is>
       </c>
-      <c r="G32" s="6" t="inlineStr">
+      <c r="G32" s="6" t="inlineStr"/>
+      <c r="H32" s="6" t="inlineStr">
         <is>
           <t>Court</t>
         </is>
       </c>
-      <c r="H32" s="6" t="inlineStr">
+      <c r="I32" s="6" t="inlineStr">
         <is>
           <t>Superior Court</t>
+        </is>
+      </c>
+      <c r="J32" s="6" t="inlineStr">
+        <is>
+          <t>https://pub.njleg.gov/Bills/2024/PL25/140_.PDF</t>
         </is>
       </c>
     </row>
@@ -40880,14 +41190,20 @@
           <t>None (enforced by dealer lawsuits)</t>
         </is>
       </c>
-      <c r="G33" s="6" t="inlineStr">
+      <c r="G33" s="6" t="inlineStr"/>
+      <c r="H33" s="6" t="inlineStr">
         <is>
           <t>Court</t>
         </is>
       </c>
-      <c r="H33" s="6" t="inlineStr">
+      <c r="I33" s="6" t="inlineStr">
         <is>
           <t>Court</t>
+        </is>
+      </c>
+      <c r="J33" s="6" t="inlineStr">
+        <is>
+          <t>https://nmonesource.com/nmos/nmsa/en/4423/1/document.do (official NMOneSource NMSA 1978 Chapter 57 PDF; site 'last modified 09/24/2026'). Section page: https://nmonesource.com/nmos/nmsa/en/item/4423/index.do</t>
         </is>
       </c>
     </row>
@@ -40920,12 +41236,22 @@
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
+          <t>https://dmv.nv.gov/</t>
+        </is>
+      </c>
+      <c r="H34" s="6" t="inlineStr">
+        <is>
           <t>Court</t>
         </is>
       </c>
-      <c r="H34" s="6" t="inlineStr">
+      <c r="I34" s="6" t="inlineStr">
         <is>
           <t>Court</t>
+        </is>
+      </c>
+      <c r="J34" s="6" t="inlineStr">
+        <is>
+          <t>https://www.leg.state.nv.us/NRS/NRS-482.html#NRS482Sec36385</t>
         </is>
       </c>
     </row>
@@ -40958,12 +41284,22 @@
       </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
+          <t>https://dmv.ny.gov/</t>
+        </is>
+      </c>
+      <c r="H35" s="6" t="inlineStr">
+        <is>
           <t>Agency or court</t>
         </is>
       </c>
-      <c r="H35" s="6" t="inlineStr">
+      <c r="I35" s="6" t="inlineStr">
         <is>
           <t>DMV Commissioner or court</t>
+        </is>
+      </c>
+      <c r="J35" s="6" t="inlineStr">
+        <is>
+          <t>https://www.nysenate.gov/legislation/laws/VAT/465 (official; Cloudflare blocks scripted fetch). Text read at https://newyork.public.law/laws/n.y._vehicle_and_traffic_law_section_465 (sourced from nysenate.gov, 'last modified Sep. 6, 2024', verified 9/19/2026). 2024 amendment checked against A4066-B on https://assembly.state.ny.us/leg/?bn=A04066&amp;term=2023</t>
         </is>
       </c>
     </row>
@@ -40996,12 +41332,22 @@
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
+          <t>https://www.bmv.ohio.gov/</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr">
+        <is>
           <t>Court</t>
         </is>
       </c>
-      <c r="H36" s="6" t="inlineStr">
+      <c r="I36" s="6" t="inlineStr">
         <is>
           <t>Franchisor's internal process, then court</t>
+        </is>
+      </c>
+      <c r="J36" s="6" t="inlineStr">
+        <is>
+          <t>https://codes.ohio.gov/ohio-revised-code/section-4517.52 ; https://codes.ohio.gov/ohio-revised-code/section-4517.59</t>
         </is>
       </c>
     </row>
@@ -41034,12 +41380,22 @@
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
+          <t>https://oklahoma.gov/onmvc.html</t>
+        </is>
+      </c>
+      <c r="H37" s="6" t="inlineStr">
+        <is>
           <t>Agency</t>
         </is>
       </c>
-      <c r="H37" s="6" t="inlineStr">
+      <c r="I37" s="6" t="inlineStr">
         <is>
           <t>Commission</t>
+        </is>
+      </c>
+      <c r="J37" s="6" t="inlineStr">
+        <is>
+          <t>Codified: https://law.justia.com/codes/oklahoma/title-47/section-47-565v1/ and .../section-47-565v2/ (2025 Okla. Stat.); enrolled HB2158/HB2160 on oklegislature.gov. OSCN not accessible.</t>
         </is>
       </c>
     </row>
@@ -41070,14 +41426,20 @@
           <t>None (enforced by dealer lawsuits)</t>
         </is>
       </c>
-      <c r="G38" s="6" t="inlineStr">
+      <c r="G38" s="6" t="inlineStr"/>
+      <c r="H38" s="6" t="inlineStr">
         <is>
           <t>Court</t>
         </is>
       </c>
-      <c r="H38" s="6" t="inlineStr">
+      <c r="I38" s="6" t="inlineStr">
         <is>
           <t>Court</t>
+        </is>
+      </c>
+      <c r="J38" s="6" t="inlineStr">
+        <is>
+          <t>https://www.oregonlegislature.gov/bills_laws/ors/ors650.html (2025 edition); pre-2026 text: https://www.oregonlegislature.gov/bills_laws/archive/2023ors650.pdf ; enrolled HB 2127: https://olis.oregonlegislature.gov/liz/2025R1/Downloads/MeasureDocument/HB2127</t>
         </is>
       </c>
     </row>
@@ -41110,12 +41472,22 @@
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
+          <t>https://www.pa.gov/agencies/dos/department-and-offices/bpoa/boards-commissions/vehicle-manufacturers-dealers-salespersons</t>
+        </is>
+      </c>
+      <c r="H39" s="6" t="inlineStr">
+        <is>
           <t>Agency</t>
         </is>
       </c>
-      <c r="H39" s="6" t="inlineStr">
+      <c r="I39" s="6" t="inlineStr">
         <is>
           <t>Board (with a mediation demand)</t>
+        </is>
+      </c>
+      <c r="J39" s="6" t="inlineStr">
+        <is>
+          <t>https://www.legis.state.pa.us/WU01/LI/LI/US/HTM/1983/0/0084..HTM (official unconsolidated statute; § 307 last amended by Act 134 of 2018; page as fetched 10/6/2026 shows no 2026 amendment notes)</t>
         </is>
       </c>
     </row>
@@ -41148,12 +41520,22 @@
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
+          <t>https://dmv.ri.gov/</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="inlineStr">
+        <is>
           <t>Agency</t>
         </is>
       </c>
-      <c r="H40" s="6" t="inlineStr">
+      <c r="I40" s="6" t="inlineStr">
         <is>
           <t>Department</t>
+        </is>
+      </c>
+      <c r="J40" s="6" t="inlineStr">
+        <is>
+          <t>https://webserver.rilegislature.gov/Statutes/TITLE31/31-5.1/31-5.1-6.htm (current codified text). 10/1/2026 changes: https://webserver.rilegislature.gov/BillText/BillText26/SenateText26/S2347A.pdf and P.L. 2026 ch. 180: https://webserver.rilegislature.gov/PublicLaws/law26/law26180.htm</t>
         </is>
       </c>
     </row>
@@ -41184,14 +41566,20 @@
           <t>None (enforced by dealer lawsuits)</t>
         </is>
       </c>
-      <c r="G41" s="6" t="inlineStr">
+      <c r="G41" s="6" t="inlineStr"/>
+      <c r="H41" s="6" t="inlineStr">
         <is>
           <t>Court</t>
         </is>
       </c>
-      <c r="H41" s="6" t="inlineStr">
+      <c r="I41" s="6" t="inlineStr">
         <is>
           <t>Court</t>
+        </is>
+      </c>
+      <c r="J41" s="6" t="inlineStr">
+        <is>
+          <t>https://www.scstatehouse.gov/code/t56c015.php</t>
         </is>
       </c>
     </row>
@@ -41224,12 +41612,22 @@
       </c>
       <c r="G42" s="6" t="inlineStr">
         <is>
+          <t>https://dor.sd.gov/individuals/motor-vehicle/</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="inlineStr">
+        <is>
           <t>Court</t>
         </is>
       </c>
-      <c r="H42" s="6" t="inlineStr">
+      <c r="I42" s="6" t="inlineStr">
         <is>
           <t>Court</t>
+        </is>
+      </c>
+      <c r="J42" s="6" t="inlineStr">
+        <is>
+          <t>https://sdlegislature.gov/Statutes/32-6B-61 (full chapter via https://sdlegislature.gov/api/Statutes/32-6B.html?all=true)</t>
         </is>
       </c>
     </row>
@@ -41266,12 +41664,22 @@
       </c>
       <c r="G43" s="6" t="inlineStr">
         <is>
+          <t>https://www.tn.gov/commerce/regboards/mvc.html</t>
+        </is>
+      </c>
+      <c r="H43" s="6" t="inlineStr">
+        <is>
           <t>Agency</t>
         </is>
       </c>
-      <c r="H43" s="6" t="inlineStr">
+      <c r="I43" s="6" t="inlineStr">
         <is>
           <t>Commission</t>
+        </is>
+      </c>
+      <c r="J43" s="6" t="inlineStr">
+        <is>
+          <t>https://law.justia.com/codes/tennessee/2025/title-55/chapter-17/part-1/section-55-17-121/ (mirror; official T.C.A. is LexisNexis-only)</t>
         </is>
       </c>
     </row>
@@ -41304,12 +41712,22 @@
       </c>
       <c r="G44" s="6" t="inlineStr">
         <is>
+          <t>https://www.txdmv.gov/</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="inlineStr">
+        <is>
           <t>Agency</t>
         </is>
       </c>
-      <c r="H44" s="6" t="inlineStr">
+      <c r="I44" s="6" t="inlineStr">
         <is>
           <t>TxDMV (mediation first), then State Office of Administrative Hearings</t>
+        </is>
+      </c>
+      <c r="J44" s="6" t="inlineStr">
+        <is>
+          <t>https://statutes.capitol.texas.gov/Docs/OC/htm/OC.2301.htm (read via Legislature file server https://tcss.legis.texas.gov/resources/OC/htm/OC.2301.htm)</t>
         </is>
       </c>
     </row>
@@ -41342,12 +41760,22 @@
       </c>
       <c r="G45" s="6" t="inlineStr">
         <is>
+          <t>https://commerce.utah.gov/</t>
+        </is>
+      </c>
+      <c r="H45" s="6" t="inlineStr">
+        <is>
           <t>Agency or court</t>
         </is>
       </c>
-      <c r="H45" s="6" t="inlineStr">
+      <c r="I45" s="6" t="inlineStr">
         <is>
           <t>Commerce (informal proceeding) or court</t>
+        </is>
+      </c>
+      <c r="J45" s="6" t="inlineStr">
+        <is>
+          <t>https://le.utah.gov/xcode/Title13/Chapter14/13-14-S204.html (version C13-14-S204_2023050320230503, effective 5/3/2023)</t>
         </is>
       </c>
     </row>
@@ -41380,12 +41808,22 @@
       </c>
       <c r="G46" s="6" t="inlineStr">
         <is>
+          <t>https://www.dmv.virginia.gov/</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="inlineStr">
+        <is>
           <t>Agency</t>
         </is>
       </c>
-      <c r="H46" s="6" t="inlineStr">
+      <c r="I46" s="6" t="inlineStr">
         <is>
           <t>DMV Commissioner</t>
+        </is>
+      </c>
+      <c r="J46" s="6" t="inlineStr">
+        <is>
+          <t>https://law.lis.virginia.gov/vacode/title46.2/chapter15/section46.2-1571/</t>
         </is>
       </c>
     </row>
@@ -41418,12 +41856,22 @@
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
+          <t>https://tboard.vermont.gov/</t>
+        </is>
+      </c>
+      <c r="H47" s="6" t="inlineStr">
+        <is>
           <t>Agency or court</t>
         </is>
       </c>
-      <c r="H47" s="6" t="inlineStr">
+      <c r="I47" s="6" t="inlineStr">
         <is>
           <t>Board or court</t>
+        </is>
+      </c>
+      <c r="J47" s="6" t="inlineStr">
+        <is>
+          <t>https://legislature.vermont.gov/statutes/section/09/108/04086 (full chapter https://legislature.vermont.gov/statutes/fullchapter/09/108)</t>
         </is>
       </c>
     </row>
@@ -41460,12 +41908,22 @@
       </c>
       <c r="G48" s="6" t="inlineStr">
         <is>
+          <t>https://dol.wa.gov/</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="inlineStr">
+        <is>
           <t>Agency or court</t>
         </is>
       </c>
-      <c r="H48" s="6" t="inlineStr">
+      <c r="I48" s="6" t="inlineStr">
         <is>
           <t>DOL proceeding or court</t>
+        </is>
+      </c>
+      <c r="J48" s="6" t="inlineStr">
+        <is>
+          <t>https://app.leg.wa.gov/RCW/default.aspx?cite=46.96.105</t>
         </is>
       </c>
     </row>
@@ -41498,12 +41956,22 @@
       </c>
       <c r="G49" s="6" t="inlineStr">
         <is>
+          <t>https://wisconsindot.gov/</t>
+        </is>
+      </c>
+      <c r="H49" s="6" t="inlineStr">
+        <is>
           <t>Agency or court</t>
         </is>
       </c>
-      <c r="H49" s="6" t="inlineStr">
+      <c r="I49" s="6" t="inlineStr">
         <is>
           <t>Court or DOT licensing case</t>
+        </is>
+      </c>
+      <c r="J49" s="6" t="inlineStr">
+        <is>
+          <t>https://docs.legis.wisconsin.gov/statutes/statutes/218/i/0125</t>
         </is>
       </c>
     </row>
@@ -41536,12 +42004,22 @@
       </c>
       <c r="G50" s="6" t="inlineStr">
         <is>
+          <t>https://dmv.wv.gov/</t>
+        </is>
+      </c>
+      <c r="H50" s="6" t="inlineStr">
+        <is>
           <t>Court</t>
         </is>
       </c>
-      <c r="H50" s="6" t="inlineStr">
+      <c r="I50" s="6" t="inlineStr">
         <is>
           <t>Court</t>
+        </is>
+      </c>
+      <c r="J50" s="6" t="inlineStr">
+        <is>
+          <t>https://code.wvlegislature.gov/17A-6A-8a/</t>
         </is>
       </c>
     </row>
@@ -41574,17 +42052,27 @@
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
+          <t>https://www.dot.state.wy.us/</t>
+        </is>
+      </c>
+      <c r="H51" s="6" t="inlineStr">
+        <is>
           <t>Court</t>
         </is>
       </c>
-      <c r="H51" s="6" t="inlineStr">
+      <c r="I51" s="6" t="inlineStr">
         <is>
           <t>Mediation, then court</t>
         </is>
       </c>
+      <c r="J51" s="6" t="inlineStr">
+        <is>
+          <t>https://wyoleg.gov/statutes/compress/title31.pdf (current Title 31) and enrolled act https://wyoleg.gov/2025/Enroll/SF0106.pdf</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H51"/>
+  <autoFilter ref="A1:J51"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
UX updates: Go to state picker on every tab; matrix shows conditions and Silent vs Not covered; Copy quote + cite; score caveat and draft weights; score table runs Level 0 to 3; banner reads Research summary, not legal advice
</commit_message>
<xml_diff>
--- a/docs/downloads/warranty-atlas.xlsx
+++ b/docs/downloads/warranty-atlas.xlsx
@@ -9748,98 +9748,98 @@
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>Points = weight × level ÷ 3. Score = sum of points (0–100). Weights are a judgment call about how much each limit constrains audits and chargebacks. Levels are read from the statute text and, where a state agency rule sets the limit, from that rule.</t>
+          <t>Points = weight × level ÷ 3. Score = sum of points (0–100). Weights are a judgment call about how much each limit constrains audits and chargebacks, and are a draft pending S&amp;Q and Legal review. Levels are read from the statute text and, where a state agency rule sets the limit, from that rule. The score measures how strict the law is, not how likely an audit dispute is.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
         <is>
-          <t>Short audit and chargeback lookback (weight 21; How far back and how much can be charged back): level 3: 6 months or less; level 2: 9 months; level 1: 12 months; level 0: No limit in statute, or over 12 months</t>
+          <t>Short audit and chargeback lookback (weight 21; How far back and how much can be charged back): level 0: No limit in statute, or over 12 months; level 1: 12 months; level 2: 9 months; level 3: 6 months or less</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>Limits on extrapolating audit results (weight 15; How far back and how much can be charged back): level 3: Prohibited; level 2: Restricted (e.g., only from a valid random sample); level 0: Not addressed</t>
+          <t>Limits on extrapolating audit results (weight 15; How far back and how much can be charged back): level 0: Not addressed; level 2: Restricted (e.g., only from a valid random sample); level 3: Prohibited</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
         <is>
-          <t>No fraud carve-out from the time limit (weight 4; How far back and how much can be charged back): level 3: The time limit applies even to suspected fraud; level 0: Fraud is excepted, or not stated</t>
+          <t>No fraud carve-out from the time limit (weight 4; How far back and how much can be charged back): level 0: Fraud is excepted, or not stated; level 3: The time limit applies even to suspected fraud</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>No chargebacks for clerical or paperwork errors (weight 12; What counts as a valid chargeback): level 3: Applies; level 0: Not in statute</t>
+          <t>No chargebacks for clerical or paperwork errors (weight 12; What counts as a valid chargeback): level 0: Not in statute; level 3: Applies</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
         <is>
-          <t>Limits on documentation requirements (weight 8; What counts as a valid chargeback): level 3: Applies; level 0: Not in statute</t>
+          <t>Limits on documentation requirements (weight 8; What counts as a valid chargeback): level 0: Not in statute; level 3: Applies</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>Chargeback held while the dealer appeals (weight 15; When a chargeback can be collected): level 3: Applies; level 0: Not in statute</t>
+          <t>Chargeback held while the dealer appeals (weight 15; When a chargeback can be collected): level 0: Not in statute; level 3: Applies</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
-          <t>Advance written notice of audit (weight 3; Audit process steps): level 3: Applies; level 0: Not in statute</t>
+          <t>Advance written notice of audit (weight 3; Audit process steps): level 0: Not in statute; level 3: Applies</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t>Must tell the dealer why it was selected (weight 3; Audit process steps): level 3: Applies; level 0: Not in statute</t>
+          <t>Must tell the dealer why it was selected (weight 3; Audit process steps): level 0: Not in statute; level 3: Applies</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
         <is>
-          <t>Written reasons required before a chargeback (weight 3; Audit process steps): level 3: Applies; level 0: Not in statute</t>
+          <t>Written reasons required before a chargeback (weight 3; Audit process steps): level 0: Not in statute; level 3: Applies</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
         <is>
-          <t>Dealer response or cure period (weight 3; Audit process steps): level 3: 60 days or more; level 2: 30 to 59 days; level 1: Under 30 days; level 0: None in statute</t>
+          <t>Dealer response or cure period (weight 3; Audit process steps): level 0: None in statute; level 1: Under 30 days; level 2: 30 to 59 days; level 3: 60 days or more</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
         <is>
-          <t>Internal appeal required (weight 3; Audit process steps): level 3: Applies; level 0: Not in statute</t>
+          <t>Internal appeal required (weight 3; Audit process steps): level 0: Not in statute; level 3: Applies</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
         <is>
-          <t>Cap on how often audits can occur (weight 3; Audit process steps): level 3: At most one audit per 12 months; level 2: Cap allows more than one audit a year (e.g., one per 9 months); level 0: No cap in statute</t>
+          <t>Cap on how often audits can occur (weight 3; Audit process steps): level 0: No cap in statute; level 2: Cap allows more than one audit a year (e.g., one per 9 months); level 3: At most one audit per 12 months</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
         <is>
-          <t>Rate validation limited to the dealer's submission (weight 3; Rate validation and consequences): level 3: Only the dealer's own ROs or a single accuracy objection; level 0: Not limited in statute</t>
+          <t>Rate validation limited to the dealer's submission (weight 3; Rate validation and consequences): level 0: Not limited in statute; level 3: Only the dealer's own ROs or a single accuracy objection</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Neutral labels: flagged states keep gold outline and badges labeled Flagged; remove company-specific names; build check blocks them
</commit_message>
<xml_diff>
--- a/docs/downloads/warranty-atlas.xlsx
+++ b/docs/downloads/warranty-atlas.xlsx
@@ -497,7 +497,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Built 2026-10-06 from the live Atlas data files.</t>
+          <t>Built 2026-10-07 from the live Atlas data files.</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Audit climate: the audit climate score (0-100) behind the Map: U.S. Audit Climate tab, its two sub-scores and each limit's level (0-3), with the weights, plus distributor-franchised states. Higher = more restrictive toward audits, chargebacks and rate validation. Statute text only.</t>
+          <t>Audit climate: the audit climate score (0-100) behind the Map: U.S. Audit Climate tab, its two sub-scores and each limit's level (0-3), with the weights, plus flagged states. Higher = more restrictive toward audits, chargebacks and rate validation. Statute text only.</t>
         </is>
       </c>
     </row>
@@ -618,7 +618,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Public-source research summary for audit planning. It is not legal advice and does not contain SOA-approved rates or dealer payment data. Confirm against the cited statute before relying on a specific rule; escalate disputes to Legal.</t>
+          <t>Public-source research summary for audit planning. It is not legal advice and does not contain any company-approved rates or dealer payment data. Confirm against the cited statute before relying on a specific rule; escalate disputes to Legal.</t>
         </is>
       </c>
     </row>
@@ -6098,7 +6098,7 @@
       </c>
       <c r="V1" s="4" t="inlineStr">
         <is>
-          <t>Distributor-franchised</t>
+          <t>Flagged state</t>
         </is>
       </c>
     </row>
@@ -6606,7 +6606,7 @@
       </c>
       <c r="V8" s="6" t="inlineStr">
         <is>
-          <t>Subaru of New England, Inc.</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -6898,7 +6898,7 @@
       </c>
       <c r="V12" s="6" t="inlineStr">
         <is>
-          <t>SUBARU Hawaii</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -7478,7 +7478,7 @@
       </c>
       <c r="V20" s="6" t="inlineStr">
         <is>
-          <t>Subaru of New England, Inc.</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -7626,7 +7626,7 @@
       </c>
       <c r="V22" s="6" t="inlineStr">
         <is>
-          <t>Subaru of New England, Inc.</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -8278,7 +8278,7 @@
       </c>
       <c r="V31" s="6" t="inlineStr">
         <is>
-          <t>Subaru of New England, Inc.</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -8354,7 +8354,7 @@
       </c>
       <c r="V32" s="6" t="inlineStr">
         <is>
-          <t>Subaru Distributors Corp. (northern counties only)</t>
+          <t>Yes (northern counties only)</t>
         </is>
       </c>
     </row>
@@ -8574,7 +8574,7 @@
       </c>
       <c r="V35" s="6" t="inlineStr">
         <is>
-          <t>Subaru Distributors Corp.</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -8938,7 +8938,7 @@
       </c>
       <c r="V40" s="6" t="inlineStr">
         <is>
-          <t>Subaru of New England, Inc.</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -9446,7 +9446,7 @@
       </c>
       <c r="V47" s="6" t="inlineStr">
         <is>
-          <t>Subaru of New England, Inc.</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -9748,7 +9748,7 @@
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>Points = weight × level ÷ 3. Score = sum of points (0–100). Weights are a judgment call about how much each limit constrains audits and chargebacks, and are a draft pending S&amp;Q and Legal review. Levels are read from the statute text and, where a state agency rule sets the limit, from that rule. The score measures how strict the law is, not how likely an audit dispute is.</t>
+          <t>Points = weight × level ÷ 3. Score = sum of points (0–100). Weights are a judgment call about how much each limit constrains audits and chargebacks, and are a draft that may change. Levels are read from the statute text and, where a state agency rule sets the limit, from that rule. The score measures how strict the law is, not how likely an audit dispute is.</t>
         </is>
       </c>
     </row>
@@ -43672,7 +43672,7 @@
       </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>From 10/1/2026 Subaru's recall and warranty claim systems must accept and pay Connecticut used-inventory stop-sale claims on the 30-day/1-year-audit timetable, and may not claw these payments back through chargebacks or incentive programs unless the action applies uniformly to every same-line-make dealer in the state.</t>
+          <t>From 10/1/2026 manufacturers' recall and warranty claim systems must accept and pay Connecticut used-inventory stop-sale claims on the 30-day/1-year-audit timetable, and may not claw these payments back through chargebacks or incentive programs unless the action applies uniformly to every same-line-make dealer in the state.</t>
         </is>
       </c>
       <c r="J4" s="6" t="inlineStr">
@@ -43724,7 +43724,7 @@
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>This is the first board ruling that recovering statutory warranty uplift through per-vehicle or parts-account debits is an illegal surcharge. Subaru should confirm that nothing in its Illinois pricing or charge structure is tied to warranty reimbursement, and should watch for the same argument under other anti-cost-recovery statutes, such as RI § 31-5.1-6(g).</t>
+          <t>This is the first board ruling that recovering statutory warranty uplift through per-vehicle or parts-account debits is an illegal surcharge. Manufacturers should confirm that nothing in their Illinois pricing or charge structure is tied to warranty reimbursement, and should watch for the same argument under other anti-cost-recovery statutes, such as RI § 31-5.1-6(g).</t>
         </is>
       </c>
       <c r="J5" s="6" t="inlineStr">
@@ -43776,7 +43776,7 @@
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>It explains the first statute that pays warranty labor on actual technician time for all line-makes. From 10/1/2026 Subaru must adjust Rhode Island claim intake and audit to take time-punch evidence and carry the burden of proof on time disallowances.</t>
+          <t>It explains the first statute that pays warranty labor on actual technician time for all line-makes. From 10/1/2026 manufacturers must adjust Rhode Island claim intake and audit to take time-punch evidence and carry the burden of proof on time disallowances.</t>
         </is>
       </c>
       <c r="J6" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Weekly check 2026-10-12: 0 enacted changes, 3 pending bills unchanged, 0 law-data updates
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A91PSkGryMhMdphpzADuWa
</commit_message>
<xml_diff>
--- a/docs/downloads/warranty-atlas.xlsx
+++ b/docs/downloads/warranty-atlas.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit fields" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rate sample rules" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Law dates" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governing bodies" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly log" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="News" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit procedures" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit climate" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Coverage" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Audit fields" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Rate sample rules" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Law dates" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Governing bodies" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Weekly log" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="News" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Audit procedures" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Audit climate" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Summary'!$A$1:$R$51</definedName>
@@ -26,7 +26,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Rate sample rules'!$A$1:$L$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Law dates'!$A$1:$M$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Governing bodies'!$A$1:$J$51</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Weekly log'!$A$1:$J$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Weekly log'!$A$1:$J$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'News'!$A$1:$J$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Audit procedures'!$A$1:$X$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Audit climate'!$A$1:$V$51</definedName>
@@ -497,7 +497,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Built 2026-10-07 from the live Atlas data files.</t>
+          <t>Built 2026-10-12 from the live Atlas data files.</t>
         </is>
       </c>
     </row>
@@ -42083,7 +42083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:J30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -42153,12 +42153,12 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>Source review: all 50 states' agency rules checked; Tennessee limits added from Commission rules; Rhode Island 10/1 law moved into current data; 23 matrix fields updated</t>
+          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
@@ -42179,7 +42179,7 @@
       <c r="F2" s="6" t="inlineStr"/>
       <c r="G2" s="6" t="inlineStr">
         <is>
-          <t>Pending in House Commerce (hearing listed 10/5/2026); not law.</t>
+          <t>Official page returned HTTP 503 this run; search found no new action. Prior status carried forward (House Commerce, last action 07/01/2026). Not law.</t>
         </is>
       </c>
       <c r="H2" s="6" t="inlineStr">
@@ -42201,12 +42201,12 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Source review: all 50 states' agency rules checked; Tennessee limits added from Commission rules; Rhode Island 10/1 law moved into current data; 23 matrix fields updated</t>
+          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -42227,7 +42227,7 @@
       <c r="F3" s="6" t="inlineStr"/>
       <c r="G3" s="6" t="inlineStr">
         <is>
-          <t>Passed Assembly 06/01/2026; in Senate Rules. No Senate action (official record checked 10/6/2026).</t>
+          <t>Re-checked on nyassembly.gov 10/12/2026: passed Assembly 06/01/2026, referred to Senate Rules; no Senate action.</t>
         </is>
       </c>
       <c r="H3" s="6" t="inlineStr">
@@ -42249,12 +42249,12 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Source review: all 50 states' agency rules checked; Tennessee limits added from Commission rules; Rhode Island 10/1 law moved into current data; 23 matrix fields updated</t>
+          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -42275,7 +42275,7 @@
       <c r="F4" s="6" t="inlineStr"/>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>No new action found in search this run (not re-verified on the official site; prior status carried forward). Still pending as of 10/6/2026 (HB5197, introduced 2/10/2026, also in House Rules).</t>
+          <t>Official page returned HTTP 503 this run; search found no new action. Prior status carried forward (House Rules). Not law.</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
@@ -42297,156 +42297,144 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>0 enacted changes, 3 pending bills (1 moved earlier than logged), 0 law-data updates; 4 laws reached 10/1/2026 effective date</t>
+          <t>Source review: all 50 states' agency rules checked; Tennessee limits added from Commission rules; Rhode Island 10/1 law moved into current data; 23 matrix fields updated</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>enacted_recent</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>RI</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>2026 S 2347 Sub A (P.L. 2026, ch. 180) / H 8213 Sub A (P.L. 2026, ch. 179)</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>SB 1182 (2025-26), PN 1866</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr"/>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>Effective 10/01/2026 reached; no lawsuit or injunction found in search.</t>
+          <t>Pending in House Commerce (hearing listed 10/5/2026); not law.</t>
         </is>
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>Actual-technician-time warranty labor rule; no change since baseline.</t>
+          <t>No committee action since referral; still pending.</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>Now in effect; site date selector applies it automatically. No data change.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
-          <t>https://webserver.rilegislature.gov/PublicLaws/law26/law26180.htm</t>
+          <t>https://www.palegis.us/legislation/bills/2025/sb1182</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>0 enacted changes, 3 pending bills (1 moved earlier than logged), 0 law-data updates; 4 laws reached 10/1/2026 effective date</t>
+          <t>Source review: all 50 states' agency rules checked; Tennessee limits added from Commission rules; Rhode Island 10/1 law moved into current data; 23 matrix fields updated</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>enacted_recent</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>LB972 (2026), Sec. 70</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>A8773 (Magnarelli) / S8360 (Cooney), 2025-26</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr"/>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Effective 10/01/2026 reached; no lawsuit or injunction found in search.</t>
+          <t>Passed Assembly 06/01/2026; in Senate Rules. No Senate action (official record checked 10/6/2026).</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>RV scope carve-out; no change since baseline.</t>
+          <t>No Senate action since referral; still pending.</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>Now in effect; site date selector applies it automatically. No data change.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>https://nebraskalegislature.gov/FloorDocs/109/PDF/Slip/LB972.pdf</t>
+          <t>https://nyassembly.gov/leg/?default_fld=&amp;leg_video=&amp;bn=A08773&amp;term=2025&amp;Summary=Y&amp;Actions=Y</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>0 enacted changes, 3 pending bills (1 moved earlier than logged), 0 law-data updates; 4 laws reached 10/1/2026 effective date</t>
+          <t>Source review: all 50 states' agency rules checked; Tennessee limits added from Commission rules; Rhode Island 10/1 law moved into current data; 23 matrix fields updated</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>enacted_recent</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>CT</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Public Act 26-24 (sSB 413), §§ 20-25</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>SB1939 (104th GA), as amended by Senate Floor Amendments 1-2</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr"/>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>Effective 10/01/2026 reached; no lawsuit or injunction found in search.</t>
+          <t>No new action found in search this run (not re-verified on the official site; prior status carried forward). Still pending as of 10/6/2026 (HB5197, introduced 2/10/2026, also in House Rules).</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>Stop-sale/recall inventory compensation; no change since baseline.</t>
+          <t>No House action since Rules re-assignment; still pending.</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>Now in effect; site date selector applies it automatically. No data change.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>https://www.cga.ct.gov/2026/ACT/PA/PDF/2026PA-00024-R00SB-00413-PA.PDF</t>
+          <t>https://www.ilga.gov/Legislation/BillStatus?DocNum=1939&amp;GAID=18&amp;DocTypeID=SB&amp;SessionID=114</t>
         </is>
       </c>
     </row>
@@ -42468,12 +42456,12 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>RI</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>2026 SB 345 (Chapter 463; cross-filed HB 1214)</t>
+          <t>2026 S 2347 Sub A (P.L. 2026, ch. 180) / H 8213 Sub A (P.L. 2026, ch. 179)</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
@@ -42488,7 +42476,7 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>MVA hearing route for association disputes; no change since baseline.</t>
+          <t>Actual-technician-time warranty labor rule; no change since baseline.</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
@@ -42498,7 +42486,7 @@
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>https://mgaleg.maryland.gov/mgawebsite/Legislation/Details/sb0345?ys=2026RS</t>
+          <t>https://webserver.rilegislature.gov/PublicLaws/law26/law26180.htm</t>
         </is>
       </c>
     </row>
@@ -42515,38 +42503,42 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_recent</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>SB 1182 (2025-26), PN 1866</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr"/>
+          <t>LB972 (2026), Sec. 70</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>No new action found in search this run (not re-verified on the official site; prior status carried forward).</t>
+          <t>Effective 10/01/2026 reached; no lawsuit or injunction found in search.</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>No committee action since referral; still pending.</t>
+          <t>RV scope carve-out; no change since baseline.</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>Watch only, unchanged.</t>
+          <t>Now in effect; site date selector applies it automatically. No data change.</t>
         </is>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>https://www.palegis.us/legislation/bills/2025/sb1182</t>
+          <t>https://nebraskalegislature.gov/FloorDocs/109/PDF/Slip/LB972.pdf</t>
         </is>
       </c>
     </row>
@@ -42563,38 +42555,42 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_recent</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>CT</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>A8773 (Magnarelli) / S8360 (Cooney), 2025-26</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr"/>
+          <t>Public Act 26-24 (sSB 413), §§ 20-25</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Official record: passed Assembly 06/01/2026, delivered to Senate, referred to Rules. No Senate action since.</t>
+          <t>Effective 10/01/2026 reached; no lawsuit or injunction found in search.</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>No Senate action since referral; still pending.</t>
+          <t>Stop-sale/recall inventory compensation; no change since baseline.</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>Watch only, unchanged.</t>
+          <t>Now in effect; site date selector applies it automatically. No data change.</t>
         </is>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>https://nyassembly.gov/leg/?default_fld=&amp;leg_video=&amp;bn=A08773&amp;term=2025&amp;Summary=Y&amp;Actions=Y</t>
+          <t>https://www.cga.ct.gov/2026/ACT/PA/PDF/2026PA-00024-R00SB-00413-PA.PDF</t>
         </is>
       </c>
     </row>
@@ -42611,194 +42607,186 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_recent</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>MD</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>SB1939 (104th GA), as amended by Senate Floor Amendments 1-2</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr"/>
+          <t>2026 SB 345 (Chapter 463; cross-filed HB 1214)</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>No new action found in search this run (not re-verified on the official site; prior status carried forward).</t>
+          <t>Effective 10/01/2026 reached; no lawsuit or injunction found in search.</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>No House action since Rules re-assignment; still pending.</t>
+          <t>MVA hearing route for association disputes; no change since baseline.</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>Watch only, unchanged.</t>
+          <t>Now in effect; site date selector applies it automatically. No data change.</t>
         </is>
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>https://www.ilga.gov/Legislation/BillStatus?DocNum=1939&amp;GAID=18&amp;DocTypeID=SB&amp;SessionID=114</t>
+          <t>https://mgaleg.maryland.gov/mgawebsite/Legislation/Details/sb0345?ys=2026RS</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
+          <t>0 enacted changes, 3 pending bills (1 moved earlier than logged), 0 law-data updates; 4 laws reached 10/1/2026 effective date</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>enacted_upcoming</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>RI</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>2026 S 2347 Sub A (P.L. 2026, ch. 180) / H 8213 Sub A (P.L. 2026, ch. 179)</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>SB 1182 (2025-26), PN 1866</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr"/>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Confirmed unchanged: signed 06/22/2026, takes effect 10/01/2026. No lawsuit or injunction against the actual-time law found in a fresh search.</t>
+          <t>No new action found in search this run (not re-verified on the official site; prior status carried forward).</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>Actual-technician-time warranty labor rule; no change since baseline.</t>
+          <t>No committee action since referral; still pending.</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>No change from baseline.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>https://webserver.rilegislature.gov/PublicLaws/law26/law26180.htm</t>
+          <t>https://www.palegis.us/legislation/bills/2025/sb1182</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
+          <t>0 enacted changes, 3 pending bills (1 moved earlier than logged), 0 law-data updates; 4 laws reached 10/1/2026 effective date</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>enacted_upcoming</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>LB972 (2026), Sec. 70</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>A8773 (Magnarelli) / S8360 (Cooney), 2025-26</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr"/>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Confirmed unchanged: approved 04/14/2026, Sec. 70 operative 10/01/2026 per Sec. 84.</t>
+          <t>Official record: passed Assembly 06/01/2026, delivered to Senate, referred to Rules. No Senate action since.</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>RV scope carve-out; no change since baseline.</t>
+          <t>No Senate action since referral; still pending.</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>No change from baseline.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>https://nebraskalegislature.gov/FloorDocs/109/PDF/Slip/LB972.pdf</t>
+          <t>https://nyassembly.gov/leg/?default_fld=&amp;leg_video=&amp;bn=A08773&amp;term=2025&amp;Summary=Y&amp;Actions=Y</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
+          <t>0 enacted changes, 3 pending bills (1 moved earlier than logged), 0 law-data updates; 4 laws reached 10/1/2026 effective date</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>enacted_upcoming</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>CT</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>Public Act 26-24 (sSB 413), §§ 20-25</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>SB1939 (104th GA), as amended by Senate Floor Amendments 1-2</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr"/>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>Confirmed unchanged: signed 05/27/2026, §§ 20-25 effective 10/01/2026.</t>
+          <t>No new action found in search this run (not re-verified on the official site; prior status carried forward).</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>Stop-sale/recall inventory compensation; no change since baseline.</t>
+          <t>No House action since Rules re-assignment; still pending.</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>No change from baseline.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>https://www.cga.ct.gov/2026/ACT/PA/PDF/2026PA-00024-R00SB-00413-PA.PDF</t>
+          <t>https://www.ilga.gov/Legislation/BillStatus?DocNum=1939&amp;GAID=18&amp;DocTypeID=SB&amp;SessionID=114</t>
         </is>
       </c>
     </row>
@@ -42820,12 +42808,12 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>RI</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>2026 SB 345 (Chapter 463; cross-filed HB 1214)</t>
+          <t>2026 S 2347 Sub A (P.L. 2026, ch. 180) / H 8213 Sub A (P.L. 2026, ch. 179)</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -42835,12 +42823,12 @@
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Confirmed unchanged: approved 05/12/2026, effective 10/01/2026.</t>
+          <t>Confirmed unchanged: signed 06/22/2026, takes effect 10/01/2026. No lawsuit or injunction against the actual-time law found in a fresh search.</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>MVA hearing route for association disputes; no change since baseline.</t>
+          <t>Actual-technician-time warranty labor rule; no change since baseline.</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr">
@@ -42850,7 +42838,7 @@
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
-          <t>https://mgaleg.maryland.gov/mgawebsite/Legislation/Details/sb0345?ys=2026RS</t>
+          <t>https://webserver.rilegislature.gov/PublicLaws/law26/law26180.htm</t>
         </is>
       </c>
     </row>
@@ -42867,38 +42855,42 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_upcoming</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>SB 1182 (2025-26), PN 1866</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr"/>
+          <t>LB972 (2026), Sec. 70</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>Re-checked via palegis.us (bill page returned a server error on two attempts; corroborated via a bill-tracking aggregator citing the official record) and web search. Still 'in committee': House Commerce Committee, last action 07/01/2026. No House floor action found.</t>
+          <t>Confirmed unchanged: approved 04/14/2026, Sec. 70 operative 10/01/2026 per Sec. 84.</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>No committee action since referral; still pending.</t>
+          <t>RV scope carve-out; no change since baseline.</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>Watch only, unchanged.</t>
+          <t>No change from baseline.</t>
         </is>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>https://www.palegis.us/legislation/bills/2025/sb1182</t>
+          <t>https://nebraskalegislature.gov/FloorDocs/109/PDF/Slip/LB972.pdf</t>
         </is>
       </c>
     </row>
@@ -42915,38 +42907,42 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_upcoming</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>CT</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>A8773 (Magnarelli) / S8360 (Cooney), 2025-26</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="inlineStr"/>
+          <t>Public Act 26-24 (sSB 413), §§ 20-25</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Re-checked on nyassembly.gov: A8773's last action is still 06/01/2026 (referred to Senate Rules); no further Senate action found.</t>
+          <t>Confirmed unchanged: signed 05/27/2026, §§ 20-25 effective 10/01/2026.</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>No Senate action since referral; still pending.</t>
+          <t>Stop-sale/recall inventory compensation; no change since baseline.</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>Watch only, unchanged.</t>
+          <t>No change from baseline.</t>
         </is>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
-          <t>https://nyassembly.gov/leg/?default_fld=&amp;leg_video=&amp;bn=A08773&amp;term=2025&amp;Summary=Y&amp;Actions=Y</t>
+          <t>https://www.cga.ct.gov/2026/ACT/PA/PDF/2026PA-00024-R00SB-00413-PA.PDF</t>
         </is>
       </c>
     </row>
@@ -42963,194 +42959,186 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_upcoming</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>MD</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>SB1939 (104th GA), as amended by Senate Floor Amendments 1-2</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="inlineStr"/>
+          <t>2026 SB 345 (Chapter 463; cross-filed HB 1214)</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>Re-checked via web search (ilga.gov bill-status page returned a server error). Still pending in House Rules Committee since 03/20/2026; spring session adjourned 06/01/2026 with no further action.</t>
+          <t>Confirmed unchanged: approved 05/12/2026, effective 10/01/2026.</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>No House action since Rules re-assignment; still pending.</t>
+          <t>MVA hearing route for association disputes; no change since baseline.</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>Watch only, unchanged.</t>
+          <t>No change from baseline.</t>
         </is>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t>https://www.ilga.gov/Legislation/BillStatus?DocNum=1939&amp;GAID=18&amp;DocTypeID=SB&amp;SessionID=114</t>
+          <t>https://mgaleg.maryland.gov/mgawebsite/Legislation/Details/sb0345?ys=2026RS</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Baseline: 4 enacted changes take effect Oct 1, 2026 (RI, NE, CT, MD); 3 bills still pending (PA, NY, IL)</t>
+          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>enacted_upcoming</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>RI</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>2026 S 2347 Sub A (P.L. 2026, ch. 180) / H 8213 Sub A (P.L. 2026, ch. 179)</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>SB 1182 (2025-26), PN 1866</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr"/>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>Signed by Governor 06/22/2026 (S 2347 Sub A = Chapter 180; H 8213 Sub A = Chapter 179); takes effect 10/01/2026</t>
+          <t>Re-checked via palegis.us (bill page returned a server error on two attempts; corroborated via a bill-tracking aggregator citing the official record) and web search. Still 'in committee': House Commerce Committee, last action 07/01/2026. No House floor action found.</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>Amends R.I. Gen. Laws § 31-5.1-6 and related sections. Warranty labor is paid at the dealer's non-warranty labor rate multiplied by the ACTUAL time the technician worked.</t>
+          <t>No committee action since referral; still pending.</t>
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr">
         <is>
-          <t>Already reflected: date selector switches RI to actual technician time and CPO Required on 10/1/2026.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t>https://webserver.rilegislature.gov/PublicLaws/law26/law26180.htm</t>
+          <t>https://www.palegis.us/legislation/bills/2025/sb1182</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Baseline: 4 enacted changes take effect Oct 1, 2026 (RI, NE, CT, MD); 3 bills still pending (PA, NY, IL)</t>
+          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>enacted_upcoming</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>LB972 (2026), Sec. 70</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>A8773 (Magnarelli) / S8360 (Cooney), 2025-26</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr"/>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Passed 48-1-0 on 04/10/2026; approved by Governor 04/14/2026. Sec. 84 makes Sec. 70 operative 10/01/2026.</t>
+          <t>Re-checked on nyassembly.gov: A8773's last action is still 06/01/2026 (referred to Senate Rules); no further Senate action found.</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>Sec. 70 adds § 60-1438(7): 'This section does not apply to recreational vehicles.' RVs move to the new Recreational Vehicle Industry Regulation Act. A word diff of Sec.</t>
+          <t>No Senate action since referral; still pending.</t>
         </is>
       </c>
       <c r="I20" s="6" t="inlineStr">
         <is>
-          <t>Scope only (RVs removed). No change to passenger-vehicle cells.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
-          <t>https://nebraskalegislature.gov/FloorDocs/109/PDF/Slip/LB972.pdf</t>
+          <t>https://nyassembly.gov/leg/?default_fld=&amp;leg_video=&amp;bn=A08773&amp;term=2025&amp;Summary=Y&amp;Actions=Y</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Baseline: 4 enacted changes take effect Oct 1, 2026 (RI, NE, CT, MD); 3 bills still pending (PA, NY, IL)</t>
+          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>enacted_upcoming</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>CT</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Public Act 26-24 (sSB 413), §§ 20-25</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>SB1939 (104th GA), as amended by Senate Floor Amendments 1-2</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr"/>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>Signed by Governor 05/27/2026 (per the cga.ct.gov bill status page); §§ 20-25 effective 10/01/2026</t>
+          <t>Re-checked via web search (ilga.gov bill-status page returned a server error). Still pending in House Rules Committee since 03/20/2026; spring session adjourned 06/01/2026 with no further action.</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>New § 22 covers used vehicles in a dealer's inventory that are under a stop-sale or do-not-drive order for a federal safety or emissions recall.</t>
+          <t>No House action since Rules re-assignment; still pending.</t>
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr">
         <is>
-          <t>Claim rules extend to stop-sale compensation claims. Labor rate and time cells unchanged.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
-          <t>https://www.cga.ct.gov/2026/ACT/PA/PDF/2026PA-00024-R00SB-00413-PA.PDF</t>
+          <t>https://www.ilga.gov/Legislation/BillStatus?DocNum=1939&amp;GAID=18&amp;DocTypeID=SB&amp;SessionID=114</t>
         </is>
       </c>
     </row>
@@ -43172,12 +43160,12 @@
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>RI</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>2026 SB 345 (Chapter 463; cross-filed HB 1214)</t>
+          <t>2026 S 2347 Sub A (P.L. 2026, ch. 180) / H 8213 Sub A (P.L. 2026, ch. 179)</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
@@ -43187,22 +43175,22 @@
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>Approved by Governor 05/12/2026 (Chapter 463); effective 10/01/2026</t>
+          <t>Signed by Governor 06/22/2026 (S 2347 Sub A = Chapter 180; H 8213 Sub A = Chapter 179); takes effect 10/01/2026</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>Procedural, with an indirect effect on warranty. A dealer association or manufacturer association may request an MVA administrative hearing to resolve a dispute or to get an interpretation of the franchise law, which includes the § 15-212 warranty rules.</t>
+          <t>Amends R.I. Gen. Laws § 31-5.1-6 and related sections. Warranty labor is paid at the dealer's non-warranty labor rate multiplied by the ACTUAL time the technician worked.</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr">
         <is>
-          <t>Procedural (association hearings). No change to § 15-212 cells.</t>
+          <t>Already reflected: date selector switches RI to actual technician time and CPO Required on 10/1/2026.</t>
         </is>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
-          <t>https://mgaleg.maryland.gov/mgawebsite/Legislation/Details/sb0345?ys=2026RS</t>
+          <t>https://webserver.rilegislature.gov/PublicLaws/law26/law26180.htm</t>
         </is>
       </c>
     </row>
@@ -43219,42 +43207,42 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>enacted_recent</t>
+          <t>enacted_upcoming</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>2026 HB 648 (2026 Ky. Acts ch. 83), amending KRS 190.046</t>
+          <t>LB972 (2026), Sec. 70</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>Signed by Governor 04/10/2026 (Acts Ch. 83); the official KRS 190.046 page shows 'Effective: July 15, 2026'</t>
+          <t>Passed 48-1-0 on 04/10/2026; approved by Governor 04/14/2026. Sec. 84 makes Sec. 70 operative 10/01/2026.</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>Rewrites KRS 190.046(2)(d) for vehicles in Class 7 and above (49 C.F.R. 565.15, heavy trucks) and makes component manufacturers liable. Parts are paid at acquisition cost plus a 30% gross margin.</t>
+          <t>Sec. 70 adds § 60-1438(7): 'This section does not apply to recreational vehicles.' RVs move to the new Recreational Vehicle Industry Regulation Act. A word diff of Sec.</t>
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr">
         <is>
-          <t>Class 7+ heavy trucks only; noted in KY record. Light-duty cells unchanged.</t>
+          <t>Scope only (RVs removed). No change to passenger-vehicle cells.</t>
         </is>
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
-          <t>https://apps.legislature.ky.gov/record/26rs/hb648.html</t>
+          <t>https://nebraskalegislature.gov/FloorDocs/109/PDF/Slip/LB972.pdf</t>
         </is>
       </c>
     </row>
@@ -43271,38 +43259,42 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_upcoming</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>CT</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>SB 1182 (2025-26), PN 1866</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr"/>
+          <t>Public Act 26-24 (sSB 413), §§ 20-25</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>Passed Senate 50-0 on 06/30/2026; referred to House COMMERCE Committee 07/01/2026; no House action since. The 2025-26 session ends 11/30/2026 and the bill dies if not enacted.</t>
+          <t>Signed by Governor 05/27/2026 (per the cga.ct.gov bill status page); §§ 20-25 effective 10/01/2026</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>Would amend Board of Vehicles Act § 307 to expressly cover extended warranty, CPO warranty, manufacturer-sponsored maintenance programs, parts-exchange programs and 'a service contract issued by a manufacturer or distributor or its common entity'.</t>
+          <t>New § 22 covers used vehicles in a dealer's inventory that are under a stop-sale or do-not-drive order for a federal safety or emissions recall.</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr">
         <is>
-          <t>Watch only. If enacted, PA service-contract and CPO cells would change.</t>
+          <t>Claim rules extend to stop-sale compensation claims. Labor rate and time cells unchanged.</t>
         </is>
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
-          <t>https://www.palegis.us/legislation/bills/2025/sb1182</t>
+          <t>https://www.cga.ct.gov/2026/ACT/PA/PDF/2026PA-00024-R00SB-00413-PA.PDF</t>
         </is>
       </c>
     </row>
@@ -43319,38 +43311,42 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_upcoming</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>MD</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>A8773 (Magnarelli) / S8360 (Cooney), 2025-26</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr"/>
+          <t>2026 SB 345 (Chapter 463; cross-filed HB 1214)</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>A8773 passed the Assembly 06/01/2026, went to the Senate and was referred to Senate RULES the same day. S8360 has been in Senate TRANSPORTATION since 01/07/2026. The Senate has not acted; the bills die 12/31/2026.</t>
+          <t>Approved by Governor 05/12/2026 (Chapter 463); effective 10/01/2026</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>Would amend VTL § 465 to cover affiliates and subsidiaries and to list 'extended service contract repairs', 'component part warranties' and 'any other franchisor compensated repairs'.</t>
+          <t>Procedural, with an indirect effect on warranty. A dealer association or manufacturer association may request an MVA administrative hearing to resolve a dispute or to get an interpretation of the franchise law, which includes the § 15-212 warranty rules.</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
         <is>
-          <t>Watch only. If enacted, NY paid-hours rules would add 1.5× and actual-time fallbacks.</t>
+          <t>Procedural (association hearings). No change to § 15-212 cells.</t>
         </is>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
-          <t>https://nyassembly.gov/leg/?default_fld=&amp;leg_video=&amp;bn=A08773&amp;term=2025&amp;Summary=Y&amp;Actions=Y</t>
+          <t>https://mgaleg.maryland.gov/mgawebsite/Legislation/Details/sb0345?ys=2026RS</t>
         </is>
       </c>
     </row>
@@ -43367,38 +43363,42 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_recent</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>KY</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>SB1939 (104th GA), as amended by Senate Floor Amendments 1-2</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr"/>
+          <t>2026 HB 648 (2026 Ky. Acts ch. 83), amending KRS 190.046</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>Passed Senate 55-0 on 04/10/2025. In the House it was re-assigned to the Rules Committee on 03/20/2026. It could move in the fall veto session (House session days Nov 17-19 and Dec 1-3, 2026) or the lame-duck session before the 104th GA ends in January 2027.</t>
+          <t>Signed by Governor 04/10/2026 (Acts Ch. 83); the official KRS 190.046 page shows 'Effective: July 15, 2026'</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>Mainly a direct-sales ban: an OEM not licensed to sell direct before 1/1/2022 may not own or operate a dealership or sell direct. It also amends 815 ILCS 710/6.</t>
+          <t>Rewrites KRS 190.046(2)(d) for vehicles in Class 7 and above (49 C.F.R. 565.15, heavy trucks) and makes component manufacturers liable. Parts are paid at acquisition cost plus a 30% gross margin.</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
         <is>
-          <t>Watch only. Mostly a direct-sales bill; parts-markup maintenance definition would change.</t>
+          <t>Class 7+ heavy trucks only; noted in KY record. Light-duty cells unchanged.</t>
         </is>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
-          <t>https://www.ilga.gov/Legislation/BillStatus?DocNum=1939&amp;GAID=18&amp;DocTypeID=SB&amp;SessionID=114</t>
+          <t>https://apps.legislature.ky.gov/record/26rs/hb648.html</t>
         </is>
       </c>
     </row>
@@ -43415,43 +43415,187 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>dead_or_stalled</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>H4019 (194th General Court), 'An Act to ensure fair compensation for warranty service labor'</t>
+          <t>SB 1182 (2025-26), PN 1866</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr"/>
       <c r="G27" s="6" t="inlineStr">
         <is>
+          <t>Passed Senate 50-0 on 06/30/2026; referred to House COMMERCE Committee 07/01/2026; no House action since. The 2025-26 session ends 11/30/2026 and the bill dies if not enacted.</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>Would amend Board of Vehicles Act § 307 to expressly cover extended warranty, CPO warranty, manufacturer-sponsored maintenance programs, parts-exchange programs and 'a service contract issued by a manufacturer or distributor or its common entity'.</t>
+        </is>
+      </c>
+      <c r="I27" s="6" t="inlineStr">
+        <is>
+          <t>Watch only. If enacted, PA service-contract and CPO cells would change.</t>
+        </is>
+      </c>
+      <c r="J27" s="6" t="inlineStr">
+        <is>
+          <t>https://www.palegis.us/legislation/bills/2025/sb1182</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>Baseline: 4 enacted changes take effect Oct 1, 2026 (RI, NE, CT, MD); 3 bills still pending (PA, NY, IL)</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>A8773 (Magnarelli) / S8360 (Cooney), 2025-26</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr"/>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>A8773 passed the Assembly 06/01/2026, went to the Senate and was referred to Senate RULES the same day. S8360 has been in Senate TRANSPORTATION since 01/07/2026. The Senate has not acted; the bills die 12/31/2026.</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>Would amend VTL § 465 to cover affiliates and subsidiaries and to list 'extended service contract repairs', 'component part warranties' and 'any other franchisor compensated repairs'.</t>
+        </is>
+      </c>
+      <c r="I28" s="6" t="inlineStr">
+        <is>
+          <t>Watch only. If enacted, NY paid-hours rules would add 1.5× and actual-time fallbacks.</t>
+        </is>
+      </c>
+      <c r="J28" s="6" t="inlineStr">
+        <is>
+          <t>https://nyassembly.gov/leg/?default_fld=&amp;leg_video=&amp;bn=A08773&amp;term=2025&amp;Summary=Y&amp;Actions=Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>Baseline: 4 enacted changes take effect Oct 1, 2026 (RI, NE, CT, MD); 3 bills still pending (PA, NY, IL)</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>SB1939 (104th GA), as amended by Senate Floor Amendments 1-2</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr"/>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>Passed Senate 55-0 on 04/10/2025. In the House it was re-assigned to the Rules Committee on 03/20/2026. It could move in the fall veto session (House session days Nov 17-19 and Dec 1-3, 2026) or the lame-duck session before the 104th GA ends in January 2027.</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="inlineStr">
+        <is>
+          <t>Mainly a direct-sales ban: an OEM not licensed to sell direct before 1/1/2022 may not own or operate a dealership or sell direct. It also amends 815 ILCS 710/6.</t>
+        </is>
+      </c>
+      <c r="I29" s="6" t="inlineStr">
+        <is>
+          <t>Watch only. Mostly a direct-sales bill; parts-markup maintenance definition would change.</t>
+        </is>
+      </c>
+      <c r="J29" s="6" t="inlineStr">
+        <is>
+          <t>https://www.ilga.gov/Legislation/BillStatus?DocNum=1939&amp;GAID=18&amp;DocTypeID=SB&amp;SessionID=114</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>Baseline: 4 enacted changes take effect Oct 1, 2026 (RI, NE, CT, MD); 3 bills still pending (PA, NY, IL)</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>dead_or_stalled</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>H4019 (194th General Court), 'An Act to ensure fair compensation for warranty service labor'</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr"/>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
           <t>Accompanied a study order (see H5320) on 04/02/2026, which means it is effectively dead. Formal sessions ended 07/31/2026.</t>
         </is>
       </c>
-      <c r="H27" s="6" t="inlineStr">
+      <c r="H30" s="6" t="inlineStr">
         <is>
           <t>Would have let dealers base warranty labor time on aftermarket or retail time guides. Hearing held 02/04/2026 before the Joint Committee on Consumer Protection and Professional Licensure.</t>
         </is>
       </c>
-      <c r="I27" s="6" t="inlineStr">
+      <c r="I30" s="6" t="inlineStr">
         <is>
           <t>Effectively dead (study order). No action.</t>
         </is>
       </c>
-      <c r="J27" s="6" t="inlineStr">
+      <c r="J30" s="6" t="inlineStr">
         <is>
           <t>https://malegislature.gov/Bills/194/H4019/BillHistory</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J27"/>
+  <autoFilter ref="A1:J30"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Weekly check 2026-10-19: 0 enacted changes, 3 pending bills unchanged, 0 law-data updates
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B1CBCdsoP4q81Xjhrst1XW
</commit_message>
<xml_diff>
--- a/docs/downloads/warranty-atlas.xlsx
+++ b/docs/downloads/warranty-atlas.xlsx
@@ -26,7 +26,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Rate sample rules'!$A$1:$L$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Law dates'!$A$1:$M$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Governing bodies'!$A$1:$J$51</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Weekly log'!$A$1:$J$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Weekly log'!$A$1:$J$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'News'!$A$1:$J$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Audit procedures'!$A$1:$X$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Audit climate'!$A$1:$V$51</definedName>
@@ -497,7 +497,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Built 2026-10-12 from the live Atlas data files.</t>
+          <t>Built 2026-10-19 from the live Atlas data files.</t>
         </is>
       </c>
     </row>
@@ -42083,7 +42083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J30"/>
+  <dimension ref="A1:J33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -42153,7 +42153,7 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B2" s="6" t="inlineStr">
@@ -42179,7 +42179,7 @@
       <c r="F2" s="6" t="inlineStr"/>
       <c r="G2" s="6" t="inlineStr">
         <is>
-          <t>Official page returned HTTP 503 this run; search found no new action. Prior status carried forward (House Commerce, last action 07/01/2026). Not law.</t>
+          <t>Official page returned HTTP 503 this run; search found no new action. Prior status carried forward. Not law.</t>
         </is>
       </c>
       <c r="H2" s="6" t="inlineStr">
@@ -42201,7 +42201,7 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
@@ -42227,7 +42227,7 @@
       <c r="F3" s="6" t="inlineStr"/>
       <c r="G3" s="6" t="inlineStr">
         <is>
-          <t>Re-checked on nyassembly.gov 10/12/2026: passed Assembly 06/01/2026, referred to Senate Rules; no Senate action.</t>
+          <t>Re-checked on nyassembly.gov 10/19/2026: passed Assembly 06/01/2026, delivered to Senate, referred to Rules; no Senate action since.</t>
         </is>
       </c>
       <c r="H3" s="6" t="inlineStr">
@@ -42249,7 +42249,7 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -42275,7 +42275,7 @@
       <c r="F4" s="6" t="inlineStr"/>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>Official page returned HTTP 503 this run; search found no new action. Prior status carried forward (House Rules). Not law.</t>
+          <t>Official page returned HTTP 503 this run; search found no new action. Prior status carried forward. Not law.</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
@@ -42297,12 +42297,12 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Source review: all 50 states' agency rules checked; Tennessee limits added from Commission rules; Rhode Island 10/1 law moved into current data; 23 matrix fields updated</t>
+          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -42323,7 +42323,7 @@
       <c r="F5" s="6" t="inlineStr"/>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>Pending in House Commerce (hearing listed 10/5/2026); not law.</t>
+          <t>Official page returned HTTP 503 this run; search found no new action. Prior status carried forward (House Commerce, last action 07/01/2026). Not law.</t>
         </is>
       </c>
       <c r="H5" s="6" t="inlineStr">
@@ -42345,12 +42345,12 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Source review: all 50 states' agency rules checked; Tennessee limits added from Commission rules; Rhode Island 10/1 law moved into current data; 23 matrix fields updated</t>
+          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -42371,7 +42371,7 @@
       <c r="F6" s="6" t="inlineStr"/>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Passed Assembly 06/01/2026; in Senate Rules. No Senate action (official record checked 10/6/2026).</t>
+          <t>Re-checked on nyassembly.gov 10/12/2026: passed Assembly 06/01/2026, referred to Senate Rules; no Senate action.</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
@@ -42393,12 +42393,12 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Source review: all 50 states' agency rules checked; Tennessee limits added from Commission rules; Rhode Island 10/1 law moved into current data; 23 matrix fields updated</t>
+          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -42419,7 +42419,7 @@
       <c r="F7" s="6" t="inlineStr"/>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>No new action found in search this run (not re-verified on the official site; prior status carried forward). Still pending as of 10/6/2026 (HB5197, introduced 2/10/2026, also in House Rules).</t>
+          <t>Official page returned HTTP 503 this run; search found no new action. Prior status carried forward (House Rules). Not law.</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr">
@@ -42441,156 +42441,144 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>0 enacted changes, 3 pending bills (1 moved earlier than logged), 0 law-data updates; 4 laws reached 10/1/2026 effective date</t>
+          <t>Source review: all 50 states' agency rules checked; Tennessee limits added from Commission rules; Rhode Island 10/1 law moved into current data; 23 matrix fields updated</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>enacted_recent</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>RI</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>2026 S 2347 Sub A (P.L. 2026, ch. 180) / H 8213 Sub A (P.L. 2026, ch. 179)</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>SB 1182 (2025-26), PN 1866</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr"/>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Effective 10/01/2026 reached; no lawsuit or injunction found in search.</t>
+          <t>Pending in House Commerce (hearing listed 10/5/2026); not law.</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>Actual-technician-time warranty labor rule; no change since baseline.</t>
+          <t>No committee action since referral; still pending.</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>Now in effect; site date selector applies it automatically. No data change.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>https://webserver.rilegislature.gov/PublicLaws/law26/law26180.htm</t>
+          <t>https://www.palegis.us/legislation/bills/2025/sb1182</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>0 enacted changes, 3 pending bills (1 moved earlier than logged), 0 law-data updates; 4 laws reached 10/1/2026 effective date</t>
+          <t>Source review: all 50 states' agency rules checked; Tennessee limits added from Commission rules; Rhode Island 10/1 law moved into current data; 23 matrix fields updated</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>enacted_recent</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>LB972 (2026), Sec. 70</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>A8773 (Magnarelli) / S8360 (Cooney), 2025-26</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr"/>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Effective 10/01/2026 reached; no lawsuit or injunction found in search.</t>
+          <t>Passed Assembly 06/01/2026; in Senate Rules. No Senate action (official record checked 10/6/2026).</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>RV scope carve-out; no change since baseline.</t>
+          <t>No Senate action since referral; still pending.</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>Now in effect; site date selector applies it automatically. No data change.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>https://nebraskalegislature.gov/FloorDocs/109/PDF/Slip/LB972.pdf</t>
+          <t>https://nyassembly.gov/leg/?default_fld=&amp;leg_video=&amp;bn=A08773&amp;term=2025&amp;Summary=Y&amp;Actions=Y</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>0 enacted changes, 3 pending bills (1 moved earlier than logged), 0 law-data updates; 4 laws reached 10/1/2026 effective date</t>
+          <t>Source review: all 50 states' agency rules checked; Tennessee limits added from Commission rules; Rhode Island 10/1 law moved into current data; 23 matrix fields updated</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>enacted_recent</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>CT</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Public Act 26-24 (sSB 413), §§ 20-25</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>SB1939 (104th GA), as amended by Senate Floor Amendments 1-2</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr"/>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Effective 10/01/2026 reached; no lawsuit or injunction found in search.</t>
+          <t>No new action found in search this run (not re-verified on the official site; prior status carried forward). Still pending as of 10/6/2026 (HB5197, introduced 2/10/2026, also in House Rules).</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>Stop-sale/recall inventory compensation; no change since baseline.</t>
+          <t>No House action since Rules re-assignment; still pending.</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>Now in effect; site date selector applies it automatically. No data change.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>https://www.cga.ct.gov/2026/ACT/PA/PDF/2026PA-00024-R00SB-00413-PA.PDF</t>
+          <t>https://www.ilga.gov/Legislation/BillStatus?DocNum=1939&amp;GAID=18&amp;DocTypeID=SB&amp;SessionID=114</t>
         </is>
       </c>
     </row>
@@ -42612,12 +42600,12 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>RI</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>2026 SB 345 (Chapter 463; cross-filed HB 1214)</t>
+          <t>2026 S 2347 Sub A (P.L. 2026, ch. 180) / H 8213 Sub A (P.L. 2026, ch. 179)</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
@@ -42632,7 +42620,7 @@
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>MVA hearing route for association disputes; no change since baseline.</t>
+          <t>Actual-technician-time warranty labor rule; no change since baseline.</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
@@ -42642,7 +42630,7 @@
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>https://mgaleg.maryland.gov/mgawebsite/Legislation/Details/sb0345?ys=2026RS</t>
+          <t>https://webserver.rilegislature.gov/PublicLaws/law26/law26180.htm</t>
         </is>
       </c>
     </row>
@@ -42659,38 +42647,42 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_recent</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>SB 1182 (2025-26), PN 1866</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr"/>
+          <t>LB972 (2026), Sec. 70</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>No new action found in search this run (not re-verified on the official site; prior status carried forward).</t>
+          <t>Effective 10/01/2026 reached; no lawsuit or injunction found in search.</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>No committee action since referral; still pending.</t>
+          <t>RV scope carve-out; no change since baseline.</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>Watch only, unchanged.</t>
+          <t>Now in effect; site date selector applies it automatically. No data change.</t>
         </is>
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>https://www.palegis.us/legislation/bills/2025/sb1182</t>
+          <t>https://nebraskalegislature.gov/FloorDocs/109/PDF/Slip/LB972.pdf</t>
         </is>
       </c>
     </row>
@@ -42707,38 +42699,42 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_recent</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>CT</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>A8773 (Magnarelli) / S8360 (Cooney), 2025-26</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr"/>
+          <t>Public Act 26-24 (sSB 413), §§ 20-25</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Official record: passed Assembly 06/01/2026, delivered to Senate, referred to Rules. No Senate action since.</t>
+          <t>Effective 10/01/2026 reached; no lawsuit or injunction found in search.</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>No Senate action since referral; still pending.</t>
+          <t>Stop-sale/recall inventory compensation; no change since baseline.</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>Watch only, unchanged.</t>
+          <t>Now in effect; site date selector applies it automatically. No data change.</t>
         </is>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>https://nyassembly.gov/leg/?default_fld=&amp;leg_video=&amp;bn=A08773&amp;term=2025&amp;Summary=Y&amp;Actions=Y</t>
+          <t>https://www.cga.ct.gov/2026/ACT/PA/PDF/2026PA-00024-R00SB-00413-PA.PDF</t>
         </is>
       </c>
     </row>
@@ -42755,194 +42751,186 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_recent</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>MD</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>SB1939 (104th GA), as amended by Senate Floor Amendments 1-2</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr"/>
+          <t>2026 SB 345 (Chapter 463; cross-filed HB 1214)</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>No new action found in search this run (not re-verified on the official site; prior status carried forward).</t>
+          <t>Effective 10/01/2026 reached; no lawsuit or injunction found in search.</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>No House action since Rules re-assignment; still pending.</t>
+          <t>MVA hearing route for association disputes; no change since baseline.</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>Watch only, unchanged.</t>
+          <t>Now in effect; site date selector applies it automatically. No data change.</t>
         </is>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>https://www.ilga.gov/Legislation/BillStatus?DocNum=1939&amp;GAID=18&amp;DocTypeID=SB&amp;SessionID=114</t>
+          <t>https://mgaleg.maryland.gov/mgawebsite/Legislation/Details/sb0345?ys=2026RS</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
+          <t>0 enacted changes, 3 pending bills (1 moved earlier than logged), 0 law-data updates; 4 laws reached 10/1/2026 effective date</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>enacted_upcoming</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>RI</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>2026 S 2347 Sub A (P.L. 2026, ch. 180) / H 8213 Sub A (P.L. 2026, ch. 179)</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>SB 1182 (2025-26), PN 1866</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr"/>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Confirmed unchanged: signed 06/22/2026, takes effect 10/01/2026. No lawsuit or injunction against the actual-time law found in a fresh search.</t>
+          <t>No new action found in search this run (not re-verified on the official site; prior status carried forward).</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>Actual-technician-time warranty labor rule; no change since baseline.</t>
+          <t>No committee action since referral; still pending.</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>No change from baseline.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
-          <t>https://webserver.rilegislature.gov/PublicLaws/law26/law26180.htm</t>
+          <t>https://www.palegis.us/legislation/bills/2025/sb1182</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
+          <t>0 enacted changes, 3 pending bills (1 moved earlier than logged), 0 law-data updates; 4 laws reached 10/1/2026 effective date</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>enacted_upcoming</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>LB972 (2026), Sec. 70</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>A8773 (Magnarelli) / S8360 (Cooney), 2025-26</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr"/>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>Confirmed unchanged: approved 04/14/2026, Sec. 70 operative 10/01/2026 per Sec. 84.</t>
+          <t>Official record: passed Assembly 06/01/2026, delivered to Senate, referred to Rules. No Senate action since.</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>RV scope carve-out; no change since baseline.</t>
+          <t>No Senate action since referral; still pending.</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>No change from baseline.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>https://nebraskalegislature.gov/FloorDocs/109/PDF/Slip/LB972.pdf</t>
+          <t>https://nyassembly.gov/leg/?default_fld=&amp;leg_video=&amp;bn=A08773&amp;term=2025&amp;Summary=Y&amp;Actions=Y</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
+          <t>0 enacted changes, 3 pending bills (1 moved earlier than logged), 0 law-data updates; 4 laws reached 10/1/2026 effective date</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>enacted_upcoming</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>CT</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Public Act 26-24 (sSB 413), §§ 20-25</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>SB1939 (104th GA), as amended by Senate Floor Amendments 1-2</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr"/>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Confirmed unchanged: signed 05/27/2026, §§ 20-25 effective 10/01/2026.</t>
+          <t>No new action found in search this run (not re-verified on the official site; prior status carried forward).</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>Stop-sale/recall inventory compensation; no change since baseline.</t>
+          <t>No House action since Rules re-assignment; still pending.</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>No change from baseline.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
-          <t>https://www.cga.ct.gov/2026/ACT/PA/PDF/2026PA-00024-R00SB-00413-PA.PDF</t>
+          <t>https://www.ilga.gov/Legislation/BillStatus?DocNum=1939&amp;GAID=18&amp;DocTypeID=SB&amp;SessionID=114</t>
         </is>
       </c>
     </row>
@@ -42964,12 +42952,12 @@
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>RI</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>2026 SB 345 (Chapter 463; cross-filed HB 1214)</t>
+          <t>2026 S 2347 Sub A (P.L. 2026, ch. 180) / H 8213 Sub A (P.L. 2026, ch. 179)</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
@@ -42979,12 +42967,12 @@
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>Confirmed unchanged: approved 05/12/2026, effective 10/01/2026.</t>
+          <t>Confirmed unchanged: signed 06/22/2026, takes effect 10/01/2026. No lawsuit or injunction against the actual-time law found in a fresh search.</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>MVA hearing route for association disputes; no change since baseline.</t>
+          <t>Actual-technician-time warranty labor rule; no change since baseline.</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr">
@@ -42994,7 +42982,7 @@
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t>https://mgaleg.maryland.gov/mgawebsite/Legislation/Details/sb0345?ys=2026RS</t>
+          <t>https://webserver.rilegislature.gov/PublicLaws/law26/law26180.htm</t>
         </is>
       </c>
     </row>
@@ -43011,38 +42999,42 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_upcoming</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>SB 1182 (2025-26), PN 1866</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr"/>
+          <t>LB972 (2026), Sec. 70</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>Re-checked via palegis.us (bill page returned a server error on two attempts; corroborated via a bill-tracking aggregator citing the official record) and web search. Still 'in committee': House Commerce Committee, last action 07/01/2026. No House floor action found.</t>
+          <t>Confirmed unchanged: approved 04/14/2026, Sec. 70 operative 10/01/2026 per Sec. 84.</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>No committee action since referral; still pending.</t>
+          <t>RV scope carve-out; no change since baseline.</t>
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr">
         <is>
-          <t>Watch only, unchanged.</t>
+          <t>No change from baseline.</t>
         </is>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t>https://www.palegis.us/legislation/bills/2025/sb1182</t>
+          <t>https://nebraskalegislature.gov/FloorDocs/109/PDF/Slip/LB972.pdf</t>
         </is>
       </c>
     </row>
@@ -43059,38 +43051,42 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_upcoming</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>CT</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>A8773 (Magnarelli) / S8360 (Cooney), 2025-26</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr"/>
+          <t>Public Act 26-24 (sSB 413), §§ 20-25</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Re-checked on nyassembly.gov: A8773's last action is still 06/01/2026 (referred to Senate Rules); no further Senate action found.</t>
+          <t>Confirmed unchanged: signed 05/27/2026, §§ 20-25 effective 10/01/2026.</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>No Senate action since referral; still pending.</t>
+          <t>Stop-sale/recall inventory compensation; no change since baseline.</t>
         </is>
       </c>
       <c r="I20" s="6" t="inlineStr">
         <is>
-          <t>Watch only, unchanged.</t>
+          <t>No change from baseline.</t>
         </is>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
-          <t>https://nyassembly.gov/leg/?default_fld=&amp;leg_video=&amp;bn=A08773&amp;term=2025&amp;Summary=Y&amp;Actions=Y</t>
+          <t>https://www.cga.ct.gov/2026/ACT/PA/PDF/2026PA-00024-R00SB-00413-PA.PDF</t>
         </is>
       </c>
     </row>
@@ -43107,194 +43103,186 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_upcoming</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>MD</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>SB1939 (104th GA), as amended by Senate Floor Amendments 1-2</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr"/>
+          <t>2026 SB 345 (Chapter 463; cross-filed HB 1214)</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>Re-checked via web search (ilga.gov bill-status page returned a server error). Still pending in House Rules Committee since 03/20/2026; spring session adjourned 06/01/2026 with no further action.</t>
+          <t>Confirmed unchanged: approved 05/12/2026, effective 10/01/2026.</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>No House action since Rules re-assignment; still pending.</t>
+          <t>MVA hearing route for association disputes; no change since baseline.</t>
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr">
         <is>
-          <t>Watch only, unchanged.</t>
+          <t>No change from baseline.</t>
         </is>
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
-          <t>https://www.ilga.gov/Legislation/BillStatus?DocNum=1939&amp;GAID=18&amp;DocTypeID=SB&amp;SessionID=114</t>
+          <t>https://mgaleg.maryland.gov/mgawebsite/Legislation/Details/sb0345?ys=2026RS</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>Baseline: 4 enacted changes take effect Oct 1, 2026 (RI, NE, CT, MD); 3 bills still pending (PA, NY, IL)</t>
+          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>enacted_upcoming</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>RI</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>2026 S 2347 Sub A (P.L. 2026, ch. 180) / H 8213 Sub A (P.L. 2026, ch. 179)</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>SB 1182 (2025-26), PN 1866</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr"/>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>Signed by Governor 06/22/2026 (S 2347 Sub A = Chapter 180; H 8213 Sub A = Chapter 179); takes effect 10/01/2026</t>
+          <t>Re-checked via palegis.us (bill page returned a server error on two attempts; corroborated via a bill-tracking aggregator citing the official record) and web search. Still 'in committee': House Commerce Committee, last action 07/01/2026. No House floor action found.</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>Amends R.I. Gen. Laws § 31-5.1-6 and related sections. Warranty labor is paid at the dealer's non-warranty labor rate multiplied by the ACTUAL time the technician worked.</t>
+          <t>No committee action since referral; still pending.</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr">
         <is>
-          <t>Already reflected: date selector switches RI to actual technician time and CPO Required on 10/1/2026.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
-          <t>https://webserver.rilegislature.gov/PublicLaws/law26/law26180.htm</t>
+          <t>https://www.palegis.us/legislation/bills/2025/sb1182</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Baseline: 4 enacted changes take effect Oct 1, 2026 (RI, NE, CT, MD); 3 bills still pending (PA, NY, IL)</t>
+          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>enacted_upcoming</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>LB972 (2026), Sec. 70</t>
-        </is>
-      </c>
-      <c r="F23" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>A8773 (Magnarelli) / S8360 (Cooney), 2025-26</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr"/>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>Passed 48-1-0 on 04/10/2026; approved by Governor 04/14/2026. Sec. 84 makes Sec. 70 operative 10/01/2026.</t>
+          <t>Re-checked on nyassembly.gov: A8773's last action is still 06/01/2026 (referred to Senate Rules); no further Senate action found.</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>Sec. 70 adds § 60-1438(7): 'This section does not apply to recreational vehicles.' RVs move to the new Recreational Vehicle Industry Regulation Act. A word diff of Sec.</t>
+          <t>No Senate action since referral; still pending.</t>
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr">
         <is>
-          <t>Scope only (RVs removed). No change to passenger-vehicle cells.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
-          <t>https://nebraskalegislature.gov/FloorDocs/109/PDF/Slip/LB972.pdf</t>
+          <t>https://nyassembly.gov/leg/?default_fld=&amp;leg_video=&amp;bn=A08773&amp;term=2025&amp;Summary=Y&amp;Actions=Y</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>Baseline: 4 enacted changes take effect Oct 1, 2026 (RI, NE, CT, MD); 3 bills still pending (PA, NY, IL)</t>
+          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>enacted_upcoming</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>CT</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>Public Act 26-24 (sSB 413), §§ 20-25</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>SB1939 (104th GA), as amended by Senate Floor Amendments 1-2</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr"/>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>Signed by Governor 05/27/2026 (per the cga.ct.gov bill status page); §§ 20-25 effective 10/01/2026</t>
+          <t>Re-checked via web search (ilga.gov bill-status page returned a server error). Still pending in House Rules Committee since 03/20/2026; spring session adjourned 06/01/2026 with no further action.</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>New § 22 covers used vehicles in a dealer's inventory that are under a stop-sale or do-not-drive order for a federal safety or emissions recall.</t>
+          <t>No House action since Rules re-assignment; still pending.</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr">
         <is>
-          <t>Claim rules extend to stop-sale compensation claims. Labor rate and time cells unchanged.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
-          <t>https://www.cga.ct.gov/2026/ACT/PA/PDF/2026PA-00024-R00SB-00413-PA.PDF</t>
+          <t>https://www.ilga.gov/Legislation/BillStatus?DocNum=1939&amp;GAID=18&amp;DocTypeID=SB&amp;SessionID=114</t>
         </is>
       </c>
     </row>
@@ -43316,12 +43304,12 @@
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>RI</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>2026 SB 345 (Chapter 463; cross-filed HB 1214)</t>
+          <t>2026 S 2347 Sub A (P.L. 2026, ch. 180) / H 8213 Sub A (P.L. 2026, ch. 179)</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
@@ -43331,22 +43319,22 @@
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>Approved by Governor 05/12/2026 (Chapter 463); effective 10/01/2026</t>
+          <t>Signed by Governor 06/22/2026 (S 2347 Sub A = Chapter 180; H 8213 Sub A = Chapter 179); takes effect 10/01/2026</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>Procedural, with an indirect effect on warranty. A dealer association or manufacturer association may request an MVA administrative hearing to resolve a dispute or to get an interpretation of the franchise law, which includes the § 15-212 warranty rules.</t>
+          <t>Amends R.I. Gen. Laws § 31-5.1-6 and related sections. Warranty labor is paid at the dealer's non-warranty labor rate multiplied by the ACTUAL time the technician worked.</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
         <is>
-          <t>Procedural (association hearings). No change to § 15-212 cells.</t>
+          <t>Already reflected: date selector switches RI to actual technician time and CPO Required on 10/1/2026.</t>
         </is>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
-          <t>https://mgaleg.maryland.gov/mgawebsite/Legislation/Details/sb0345?ys=2026RS</t>
+          <t>https://webserver.rilegislature.gov/PublicLaws/law26/law26180.htm</t>
         </is>
       </c>
     </row>
@@ -43363,42 +43351,42 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>enacted_recent</t>
+          <t>enacted_upcoming</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>2026 HB 648 (2026 Ky. Acts ch. 83), amending KRS 190.046</t>
+          <t>LB972 (2026), Sec. 70</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>Signed by Governor 04/10/2026 (Acts Ch. 83); the official KRS 190.046 page shows 'Effective: July 15, 2026'</t>
+          <t>Passed 48-1-0 on 04/10/2026; approved by Governor 04/14/2026. Sec. 84 makes Sec. 70 operative 10/01/2026.</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>Rewrites KRS 190.046(2)(d) for vehicles in Class 7 and above (49 C.F.R. 565.15, heavy trucks) and makes component manufacturers liable. Parts are paid at acquisition cost plus a 30% gross margin.</t>
+          <t>Sec. 70 adds § 60-1438(7): 'This section does not apply to recreational vehicles.' RVs move to the new Recreational Vehicle Industry Regulation Act. A word diff of Sec.</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
         <is>
-          <t>Class 7+ heavy trucks only; noted in KY record. Light-duty cells unchanged.</t>
+          <t>Scope only (RVs removed). No change to passenger-vehicle cells.</t>
         </is>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
-          <t>https://apps.legislature.ky.gov/record/26rs/hb648.html</t>
+          <t>https://nebraskalegislature.gov/FloorDocs/109/PDF/Slip/LB972.pdf</t>
         </is>
       </c>
     </row>
@@ -43415,38 +43403,42 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_upcoming</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>CT</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>SB 1182 (2025-26), PN 1866</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr"/>
+          <t>Public Act 26-24 (sSB 413), §§ 20-25</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>Passed Senate 50-0 on 06/30/2026; referred to House COMMERCE Committee 07/01/2026; no House action since. The 2025-26 session ends 11/30/2026 and the bill dies if not enacted.</t>
+          <t>Signed by Governor 05/27/2026 (per the cga.ct.gov bill status page); §§ 20-25 effective 10/01/2026</t>
         </is>
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>Would amend Board of Vehicles Act § 307 to expressly cover extended warranty, CPO warranty, manufacturer-sponsored maintenance programs, parts-exchange programs and 'a service contract issued by a manufacturer or distributor or its common entity'.</t>
+          <t>New § 22 covers used vehicles in a dealer's inventory that are under a stop-sale or do-not-drive order for a federal safety or emissions recall.</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
         <is>
-          <t>Watch only. If enacted, PA service-contract and CPO cells would change.</t>
+          <t>Claim rules extend to stop-sale compensation claims. Labor rate and time cells unchanged.</t>
         </is>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
-          <t>https://www.palegis.us/legislation/bills/2025/sb1182</t>
+          <t>https://www.cga.ct.gov/2026/ACT/PA/PDF/2026PA-00024-R00SB-00413-PA.PDF</t>
         </is>
       </c>
     </row>
@@ -43463,38 +43455,42 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_upcoming</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>MD</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>A8773 (Magnarelli) / S8360 (Cooney), 2025-26</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr"/>
+          <t>2026 SB 345 (Chapter 463; cross-filed HB 1214)</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>A8773 passed the Assembly 06/01/2026, went to the Senate and was referred to Senate RULES the same day. S8360 has been in Senate TRANSPORTATION since 01/07/2026. The Senate has not acted; the bills die 12/31/2026.</t>
+          <t>Approved by Governor 05/12/2026 (Chapter 463); effective 10/01/2026</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>Would amend VTL § 465 to cover affiliates and subsidiaries and to list 'extended service contract repairs', 'component part warranties' and 'any other franchisor compensated repairs'.</t>
+          <t>Procedural, with an indirect effect on warranty. A dealer association or manufacturer association may request an MVA administrative hearing to resolve a dispute or to get an interpretation of the franchise law, which includes the § 15-212 warranty rules.</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr">
         <is>
-          <t>Watch only. If enacted, NY paid-hours rules would add 1.5× and actual-time fallbacks.</t>
+          <t>Procedural (association hearings). No change to § 15-212 cells.</t>
         </is>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>https://nyassembly.gov/leg/?default_fld=&amp;leg_video=&amp;bn=A08773&amp;term=2025&amp;Summary=Y&amp;Actions=Y</t>
+          <t>https://mgaleg.maryland.gov/mgawebsite/Legislation/Details/sb0345?ys=2026RS</t>
         </is>
       </c>
     </row>
@@ -43511,38 +43507,42 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_recent</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>KY</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>SB1939 (104th GA), as amended by Senate Floor Amendments 1-2</t>
-        </is>
-      </c>
-      <c r="F29" s="6" t="inlineStr"/>
+          <t>2026 HB 648 (2026 Ky. Acts ch. 83), amending KRS 190.046</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>Passed Senate 55-0 on 04/10/2025. In the House it was re-assigned to the Rules Committee on 03/20/2026. It could move in the fall veto session (House session days Nov 17-19 and Dec 1-3, 2026) or the lame-duck session before the 104th GA ends in January 2027.</t>
+          <t>Signed by Governor 04/10/2026 (Acts Ch. 83); the official KRS 190.046 page shows 'Effective: July 15, 2026'</t>
         </is>
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>Mainly a direct-sales ban: an OEM not licensed to sell direct before 1/1/2022 may not own or operate a dealership or sell direct. It also amends 815 ILCS 710/6.</t>
+          <t>Rewrites KRS 190.046(2)(d) for vehicles in Class 7 and above (49 C.F.R. 565.15, heavy trucks) and makes component manufacturers liable. Parts are paid at acquisition cost plus a 30% gross margin.</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
         <is>
-          <t>Watch only. Mostly a direct-sales bill; parts-markup maintenance definition would change.</t>
+          <t>Class 7+ heavy trucks only; noted in KY record. Light-duty cells unchanged.</t>
         </is>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
-          <t>https://www.ilga.gov/Legislation/BillStatus?DocNum=1939&amp;GAID=18&amp;DocTypeID=SB&amp;SessionID=114</t>
+          <t>https://apps.legislature.ky.gov/record/26rs/hb648.html</t>
         </is>
       </c>
     </row>
@@ -43559,43 +43559,187 @@
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>dead_or_stalled</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>H4019 (194th General Court), 'An Act to ensure fair compensation for warranty service labor'</t>
+          <t>SB 1182 (2025-26), PN 1866</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr"/>
       <c r="G30" s="6" t="inlineStr">
         <is>
+          <t>Passed Senate 50-0 on 06/30/2026; referred to House COMMERCE Committee 07/01/2026; no House action since. The 2025-26 session ends 11/30/2026 and the bill dies if not enacted.</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t>Would amend Board of Vehicles Act § 307 to expressly cover extended warranty, CPO warranty, manufacturer-sponsored maintenance programs, parts-exchange programs and 'a service contract issued by a manufacturer or distributor or its common entity'.</t>
+        </is>
+      </c>
+      <c r="I30" s="6" t="inlineStr">
+        <is>
+          <t>Watch only. If enacted, PA service-contract and CPO cells would change.</t>
+        </is>
+      </c>
+      <c r="J30" s="6" t="inlineStr">
+        <is>
+          <t>https://www.palegis.us/legislation/bills/2025/sb1182</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>Baseline: 4 enacted changes take effect Oct 1, 2026 (RI, NE, CT, MD); 3 bills still pending (PA, NY, IL)</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>A8773 (Magnarelli) / S8360 (Cooney), 2025-26</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr"/>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>A8773 passed the Assembly 06/01/2026, went to the Senate and was referred to Senate RULES the same day. S8360 has been in Senate TRANSPORTATION since 01/07/2026. The Senate has not acted; the bills die 12/31/2026.</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t>Would amend VTL § 465 to cover affiliates and subsidiaries and to list 'extended service contract repairs', 'component part warranties' and 'any other franchisor compensated repairs'.</t>
+        </is>
+      </c>
+      <c r="I31" s="6" t="inlineStr">
+        <is>
+          <t>Watch only. If enacted, NY paid-hours rules would add 1.5× and actual-time fallbacks.</t>
+        </is>
+      </c>
+      <c r="J31" s="6" t="inlineStr">
+        <is>
+          <t>https://nyassembly.gov/leg/?default_fld=&amp;leg_video=&amp;bn=A08773&amp;term=2025&amp;Summary=Y&amp;Actions=Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>Baseline: 4 enacted changes take effect Oct 1, 2026 (RI, NE, CT, MD); 3 bills still pending (PA, NY, IL)</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>SB1939 (104th GA), as amended by Senate Floor Amendments 1-2</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr"/>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>Passed Senate 55-0 on 04/10/2025. In the House it was re-assigned to the Rules Committee on 03/20/2026. It could move in the fall veto session (House session days Nov 17-19 and Dec 1-3, 2026) or the lame-duck session before the 104th GA ends in January 2027.</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
+        <is>
+          <t>Mainly a direct-sales ban: an OEM not licensed to sell direct before 1/1/2022 may not own or operate a dealership or sell direct. It also amends 815 ILCS 710/6.</t>
+        </is>
+      </c>
+      <c r="I32" s="6" t="inlineStr">
+        <is>
+          <t>Watch only. Mostly a direct-sales bill; parts-markup maintenance definition would change.</t>
+        </is>
+      </c>
+      <c r="J32" s="6" t="inlineStr">
+        <is>
+          <t>https://www.ilga.gov/Legislation/BillStatus?DocNum=1939&amp;GAID=18&amp;DocTypeID=SB&amp;SessionID=114</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>Baseline: 4 enacted changes take effect Oct 1, 2026 (RI, NE, CT, MD); 3 bills still pending (PA, NY, IL)</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>dead_or_stalled</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>H4019 (194th General Court), 'An Act to ensure fair compensation for warranty service labor'</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="inlineStr"/>
+      <c r="G33" s="6" t="inlineStr">
+        <is>
           <t>Accompanied a study order (see H5320) on 04/02/2026, which means it is effectively dead. Formal sessions ended 07/31/2026.</t>
         </is>
       </c>
-      <c r="H30" s="6" t="inlineStr">
+      <c r="H33" s="6" t="inlineStr">
         <is>
           <t>Would have let dealers base warranty labor time on aftermarket or retail time guides. Hearing held 02/04/2026 before the Joint Committee on Consumer Protection and Professional Licensure.</t>
         </is>
       </c>
-      <c r="I30" s="6" t="inlineStr">
+      <c r="I33" s="6" t="inlineStr">
         <is>
           <t>Effectively dead (study order). No action.</t>
         </is>
       </c>
-      <c r="J30" s="6" t="inlineStr">
+      <c r="J33" s="6" t="inlineStr">
         <is>
           <t>https://malegislature.gov/Bills/194/H4019/BillHistory</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J30"/>
+  <autoFilter ref="A1:J33"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Governing Bodies explanation; quieter layout with task-style tabs, one-line intros and answer chips
</commit_message>
<xml_diff>
--- a/docs/downloads/warranty-atlas.xlsx
+++ b/docs/downloads/warranty-atlas.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Coverage" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Audit fields" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Rate sample rules" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Law dates" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Governing bodies" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Weekly log" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="News" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Audit procedures" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Audit climate" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit fields" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rate sample rules" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Law dates" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governing bodies" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly log" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="News" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit procedures" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit climate" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Summary'!$A$1:$R$51</definedName>
@@ -497,7 +497,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Built 2026-10-19 from the live Atlas data files.</t>
+          <t>Built 2026-10-22 from the live Atlas data files.</t>
         </is>
       </c>
     </row>
@@ -563,14 +563,14 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Audit climate: the audit climate score (0-100) behind the Map: U.S. Audit Climate tab, its two sub-scores and each limit's level (0-3), with the weights, plus flagged states. Higher = more restrictive toward audits, chargebacks and rate validation. Statute text only.</t>
+          <t>Audit climate: the audit climate score (0-100) behind the Audit Climate tab, its two sub-scores and each limit's level (0-3), with the weights, plus flagged states. Higher = more restrictive toward audits, chargebacks and rate validation. Statute text only.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Weekly log and News: the Update log and News tabs.</t>
+          <t>Weekly log and News: the Updates and News tabs.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit brief for FL, CA, IL and AR: state-page block, one-page PDFs, research files; 10 matrix corrections
</commit_message>
<xml_diff>
--- a/docs/downloads/warranty-atlas.xlsx
+++ b/docs/downloads/warranty-atlas.xlsx
@@ -26,7 +26,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Rate sample rules'!$A$1:$L$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Law dates'!$A$1:$M$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Governing bodies'!$A$1:$J$51</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Weekly log'!$A$1:$J$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Weekly log'!$A$1:$J$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'News'!$A$1:$J$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Audit procedures'!$A$1:$X$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Audit climate'!$A$1:$V$51</definedName>
@@ -497,7 +497,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Built 2026-10-22 from the live Atlas data files.</t>
+          <t>Built 2026-10-23 from the live Atlas data files.</t>
         </is>
       </c>
     </row>
@@ -1088,7 +1088,7 @@
       </c>
       <c r="S4" s="6" t="inlineStr">
         <is>
-          <t>The manufacturer must approve or disapprove a rate-change request within 45 days, or it is deemed approved. If the calculated rate is substantially higher or lower than the rate on record, it may request additional documentation for 45 days before or after the submitted period. The rate must be reasonable compared with same line-make dealers in an economically similar area or the dealer's competitive market area (§ 23-112-313(c)(3)). There is no frequency limit.</t>
+          <t>The manufacturer must approve or disapprove a rate-change request within 45 days, or it is deemed approved. If the calculated rate is substantially higher or lower than the rate on record, it may request additional documentation for 45 days before or after the submitted period. The rate must be reasonable (§ 23-112-313(c)(3)); § 23-112-310(d)(1)(A) measures reasonableness against other same line-make dealers in the dealer's relevant market area or competitive market area. There is no frequency limit.</t>
         </is>
       </c>
       <c r="T4" s="6" t="inlineStr">
@@ -1236,7 +1236,7 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Not in statute</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr"/>
@@ -1720,7 +1720,7 @@
       </c>
       <c r="M10" s="6" t="inlineStr">
         <is>
-          <t>The dealer may protest to the Department of Highway Safety and Motor Vehicles within 30 days of the final notice. The licensee may not act to recover until the department makes a final, unappealable determination. The licensee bears the burden of proof.</t>
+          <t>The dealer may protest to the Department of Highway Safety and Motor Vehicles within 30 days after receiving the written notice of the final proposed chargeback amount. The licensee may not take any action to recover until the department makes a final determination that is not subject to further appeal. The licensee bears the burden of proof.</t>
         </is>
       </c>
       <c r="N10" s="6" t="inlineStr">
@@ -6402,7 +6402,7 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
@@ -6416,7 +6416,7 @@
         <v>59</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="H6" s="6" t="n">
         <v>2</v>
@@ -6437,7 +6437,7 @@
         <v>3</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O6" s="6" t="n">
         <v>3</v>
@@ -10233,7 +10233,7 @@
       <c r="P4" s="6" t="inlineStr"/>
       <c r="Q4" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="R4" s="6" t="inlineStr">
@@ -10411,7 +10411,7 @@
       <c r="P6" s="6" t="inlineStr"/>
       <c r="Q6" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="R6" s="6" t="inlineStr">
@@ -10761,7 +10761,7 @@
       <c r="P10" s="6" t="inlineStr"/>
       <c r="Q10" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="R10" s="6" t="inlineStr">
@@ -11173,7 +11173,7 @@
       <c r="P15" s="6" t="inlineStr"/>
       <c r="Q15" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="R15" s="6" t="inlineStr">
@@ -25795,7 +25795,7 @@
       </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>Written notice within the 30-day period stating the specific grounds. A claim may not be disapproved for a clerical error that does not make the claim amount incorrect, including errors from the manufacturer's prior-approval process. The dealer may contest a disapproval through the manufacturer's appeals process.</t>
+          <t>Written notice within the 30-day period stating the specific grounds (§ 313(e)(2)(A)(i); § 310(d)(2)(B)). A claim may not be disapproved for a clerical error that does not make the claim amount incorrect, including errors from the manufacturer's prior-approval process (§ 313(e)(3)(A)). The manufacturer must pay for warranty work properly performed in accordance with its requirements (§ 310(d)(3)). The dealer may contest a disapproval through the manufacturer's appeals process (§ 313(e)(3)(B)).</t>
         </is>
       </c>
       <c r="J4" s="6" t="inlineStr">
@@ -25818,7 +25818,7 @@
       </c>
       <c r="N4" s="6" t="inlineStr">
         <is>
-          <t>Audits must occur within 1 year from payment or credit. Only false or unsubstantiated claims may be charged back. The dealer may appeal a chargeback to the Motor Vehicle Commission within 90 days of notice. The chargeback cannot be levied until the appeal is resolved, and the hearing must be held within 120 days.</t>
+          <t>The manufacturer or franchiser may audit warranty and recall claims within one year from the date the claim was paid or credit issued; incentive and reimbursement programs are auditable for 12 months after the date of the transactions. Only false or unsubstantiated claims may be charged back. The dealer may appeal any chargeback to the Arkansas Motor Vehicle Commission within 90 days of notification; once an appeal is filed the chargeback may not be levied until the appeal is resolved, and the Commission must hold a hearing within 120 days of filing unless all parties have agreed to settle. The one-year period is stated for the audit; no separate deadline is stated for levying the chargeback.</t>
         </is>
       </c>
       <c r="O4" s="6" t="inlineStr">
@@ -25907,7 +25907,7 @@
       </c>
       <c r="AG4" s="6" t="inlineStr">
         <is>
-          <t>The Commission may deny, suspend or revoke a license if a manufacturer 'failed to properly fulfill any warranty agreement or to adequately and fairly compensate' dealers (§ 23-112-308). A monetary penalty may be imposed instead: up to $10,000 in place of revocation, or $50-$500 per day capped at $5,000 in place of suspension. Each instance is a separate violation (§ 23-112-309).</t>
+          <t>The Commission may deny, suspend or revoke a license on satisfactory proof that a manufacturer 'unfairly and without due regard to the equities of the parties or to the detriment of the public welfare' failed to properly fulfill any warranty agreement or to adequately and fairly compensate dealers for labor, parts or incidental expenses under factory warranty agreements (§ 23-112-308(a)(18)(A)). A monetary penalty may be imposed instead, only if the Commission finds the public interest would not be impaired: up to $10,000 in place of revocation, or $50-$500 per day capped at $5,000 in place of suspension. Each instance is a separate violation (§ 23-112-309(a)(3), (b), (d)).</t>
         </is>
       </c>
       <c r="AH4" s="6" t="inlineStr">
@@ -25937,7 +25937,7 @@
       </c>
       <c r="AM4" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="AN4" s="6" t="inlineStr">
@@ -26194,7 +26194,7 @@
       </c>
       <c r="N6" s="6" t="inlineStr">
         <is>
-          <t>Audits on a reasonable basis, never punitive, retaliatory or discriminatory, and no more than one random audit per 9 months. Chargeback grounds are the same as the denial grounds. No extrapolation unless the sample is random and statistically valid. Written notice within 30 days after the audit, then at least 30 days to rebut or cure. No chargeback until 45 days after the notice, and it must be taken within 90 days. Chargebacks are stayed while a Board protest (filed within 6 months) is pending.</t>
+          <t>Audits on a reasonable basis, never punitive, retaliatory or unfairly discriminatory, and no more than one random audit per 9 months (any additional audit needs written disclosure of its basis). Chargeback grounds are the same four as the denial grounds. No extrapolation unless the sample is random and the method statistically valid. Written notice of specific grounds within 30 days after the audit, then at least 30 days (scaled to claim volume) to rebut or cure. No chargeback until 45 days after the later of the disapproval or Final Denial notice, and it must be taken within 90 days of that notice. A Board protest filed within 6 months of that notice (or the end of the appeal process) and before the chargeback stays offset or collection until the Board's final order, after which the franchisor has 90 days.</t>
         </is>
       </c>
       <c r="O6" s="6" t="inlineStr">
@@ -26317,7 +26317,7 @@
       </c>
       <c r="AM6" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="AN6" s="6" t="inlineStr">
@@ -26902,7 +26902,7 @@
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>after submission</t>
+          <t>after receipt of the claim</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr"/>
@@ -26932,7 +26932,7 @@
       </c>
       <c r="N10" s="6" t="inlineStr">
         <is>
-          <t>No more than one audit per calendar year (§ 320.696(2)). Only the portion proven false or fraudulent, or substantially noncompliant, may be charged back. Within 30 days after the audit, the licensee must meet with the dealer (in person, phone or video) and give a detailed explanation with documentation and the basis for selecting the dealer. The dealer gets at least 45 days to respond, and the chargeback basis cannot change without new information. The dealer may protest to DHSMV within 30 days of the final notice; recovery is stayed, and the licensee bears the burden.</t>
+          <t>No more than one warranty, retail customer repair or other service-related audit per calendar year (§ 320.696(2); the cap does not name incentive audits). A post-payment chargeback is allowed only as a result of a timely conducted audit, and only for the portion proven false or fraudulent or not in substantial compliance with reasonable, written, uniformly applied procedures. Within 30 days after the audit, the licensee must meet with the dealer (in person, phone or video) and give a detailed explanation with documentation for each claim, plus a written statement of why the dealer was selected. The dealer gets at least 45 days to respond. The chargeback basis cannot change unless new information is received within 30 days after the audit ends, and then the dealer gets the same meeting and response rights again. After any internal dispute process, the licensee gives written notice of the final amount; the dealer may protest to DHSMV within 30 days after receiving it. A timely protest stays recovery until the department's final, unappealable determination, and the licensee bears the burden.</t>
         </is>
       </c>
       <c r="O10" s="6" t="inlineStr">
@@ -27055,7 +27055,7 @@
       </c>
       <c r="AM10" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="AN10" s="6" t="inlineStr">
@@ -27971,7 +27971,7 @@
       </c>
       <c r="AM15" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="AN15" s="6" t="inlineStr">
@@ -37203,7 +37203,7 @@
       <c r="J4" s="6" t="inlineStr"/>
       <c r="K4" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="L4" s="6" t="inlineStr">
@@ -37301,7 +37301,7 @@
       <c r="J6" s="6" t="inlineStr"/>
       <c r="K6" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="L6" s="6" t="inlineStr">
@@ -37505,7 +37505,7 @@
       <c r="J10" s="6" t="inlineStr"/>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="L10" s="6" t="inlineStr">
@@ -37760,7 +37760,7 @@
       <c r="J15" s="6" t="inlineStr"/>
       <c r="K15" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="L15" s="6" t="inlineStr">
@@ -42083,7 +42083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:J36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -42153,12 +42153,12 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
+          <t>Audit brief added for Florida, California, Illinois and Arkansas: what to know before auditing paid factory-warranty claims, on the state page and as a one-page PDF; 10 matrix fields corrected</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
@@ -42201,12 +42201,12 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
+          <t>Audit brief added for Florida, California, Illinois and Arkansas: what to know before auditing paid factory-warranty claims, on the state page and as a one-page PDF; 10 matrix fields corrected</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -42249,12 +42249,12 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
+          <t>Audit brief added for Florida, California, Illinois and Arkansas: what to know before auditing paid factory-warranty claims, on the state page and as a one-page PDF; 10 matrix fields corrected</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -42297,7 +42297,7 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -42323,7 +42323,7 @@
       <c r="F5" s="6" t="inlineStr"/>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>Official page returned HTTP 503 this run; search found no new action. Prior status carried forward (House Commerce, last action 07/01/2026). Not law.</t>
+          <t>Official page returned HTTP 503 this run; search found no new action. Prior status carried forward. Not law.</t>
         </is>
       </c>
       <c r="H5" s="6" t="inlineStr">
@@ -42345,7 +42345,7 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -42371,7 +42371,7 @@
       <c r="F6" s="6" t="inlineStr"/>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Re-checked on nyassembly.gov 10/12/2026: passed Assembly 06/01/2026, referred to Senate Rules; no Senate action.</t>
+          <t>Re-checked on nyassembly.gov 10/19/2026: passed Assembly 06/01/2026, delivered to Senate, referred to Rules; no Senate action since.</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
@@ -42393,7 +42393,7 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
@@ -42419,7 +42419,7 @@
       <c r="F7" s="6" t="inlineStr"/>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>Official page returned HTTP 503 this run; search found no new action. Prior status carried forward (House Rules). Not law.</t>
+          <t>Official page returned HTTP 503 this run; search found no new action. Prior status carried forward. Not law.</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr">
@@ -42441,12 +42441,12 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Source review: all 50 states' agency rules checked; Tennessee limits added from Commission rules; Rhode Island 10/1 law moved into current data; 23 matrix fields updated</t>
+          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -42467,7 +42467,7 @@
       <c r="F8" s="6" t="inlineStr"/>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Pending in House Commerce (hearing listed 10/5/2026); not law.</t>
+          <t>Official page returned HTTP 503 this run; search found no new action. Prior status carried forward (House Commerce, last action 07/01/2026). Not law.</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
@@ -42489,12 +42489,12 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Source review: all 50 states' agency rules checked; Tennessee limits added from Commission rules; Rhode Island 10/1 law moved into current data; 23 matrix fields updated</t>
+          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -42515,7 +42515,7 @@
       <c r="F9" s="6" t="inlineStr"/>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Passed Assembly 06/01/2026; in Senate Rules. No Senate action (official record checked 10/6/2026).</t>
+          <t>Re-checked on nyassembly.gov 10/12/2026: passed Assembly 06/01/2026, referred to Senate Rules; no Senate action.</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
@@ -42537,12 +42537,12 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Source review: all 50 states' agency rules checked; Tennessee limits added from Commission rules; Rhode Island 10/1 law moved into current data; 23 matrix fields updated</t>
+          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -42563,7 +42563,7 @@
       <c r="F10" s="6" t="inlineStr"/>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>No new action found in search this run (not re-verified on the official site; prior status carried forward). Still pending as of 10/6/2026 (HB5197, introduced 2/10/2026, also in House Rules).</t>
+          <t>Official page returned HTTP 503 this run; search found no new action. Prior status carried forward (House Rules). Not law.</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
@@ -42585,156 +42585,144 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>0 enacted changes, 3 pending bills (1 moved earlier than logged), 0 law-data updates; 4 laws reached 10/1/2026 effective date</t>
+          <t>Source review: all 50 states' agency rules checked; Tennessee limits added from Commission rules; Rhode Island 10/1 law moved into current data; 23 matrix fields updated</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>enacted_recent</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>RI</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>2026 S 2347 Sub A (P.L. 2026, ch. 180) / H 8213 Sub A (P.L. 2026, ch. 179)</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>SB 1182 (2025-26), PN 1866</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr"/>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Effective 10/01/2026 reached; no lawsuit or injunction found in search.</t>
+          <t>Pending in House Commerce (hearing listed 10/5/2026); not law.</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>Actual-technician-time warranty labor rule; no change since baseline.</t>
+          <t>No committee action since referral; still pending.</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>Now in effect; site date selector applies it automatically. No data change.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>https://webserver.rilegislature.gov/PublicLaws/law26/law26180.htm</t>
+          <t>https://www.palegis.us/legislation/bills/2025/sb1182</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>0 enacted changes, 3 pending bills (1 moved earlier than logged), 0 law-data updates; 4 laws reached 10/1/2026 effective date</t>
+          <t>Source review: all 50 states' agency rules checked; Tennessee limits added from Commission rules; Rhode Island 10/1 law moved into current data; 23 matrix fields updated</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>enacted_recent</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>LB972 (2026), Sec. 70</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>A8773 (Magnarelli) / S8360 (Cooney), 2025-26</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr"/>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Effective 10/01/2026 reached; no lawsuit or injunction found in search.</t>
+          <t>Passed Assembly 06/01/2026; in Senate Rules. No Senate action (official record checked 10/6/2026).</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>RV scope carve-out; no change since baseline.</t>
+          <t>No Senate action since referral; still pending.</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>Now in effect; site date selector applies it automatically. No data change.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>https://nebraskalegislature.gov/FloorDocs/109/PDF/Slip/LB972.pdf</t>
+          <t>https://nyassembly.gov/leg/?default_fld=&amp;leg_video=&amp;bn=A08773&amp;term=2025&amp;Summary=Y&amp;Actions=Y</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>0 enacted changes, 3 pending bills (1 moved earlier than logged), 0 law-data updates; 4 laws reached 10/1/2026 effective date</t>
+          <t>Source review: all 50 states' agency rules checked; Tennessee limits added from Commission rules; Rhode Island 10/1 law moved into current data; 23 matrix fields updated</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>enacted_recent</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>CT</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Public Act 26-24 (sSB 413), §§ 20-25</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>SB1939 (104th GA), as amended by Senate Floor Amendments 1-2</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr"/>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Effective 10/01/2026 reached; no lawsuit or injunction found in search.</t>
+          <t>No new action found in search this run (not re-verified on the official site; prior status carried forward). Still pending as of 10/6/2026 (HB5197, introduced 2/10/2026, also in House Rules).</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>Stop-sale/recall inventory compensation; no change since baseline.</t>
+          <t>No House action since Rules re-assignment; still pending.</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>Now in effect; site date selector applies it automatically. No data change.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>https://www.cga.ct.gov/2026/ACT/PA/PDF/2026PA-00024-R00SB-00413-PA.PDF</t>
+          <t>https://www.ilga.gov/Legislation/BillStatus?DocNum=1939&amp;GAID=18&amp;DocTypeID=SB&amp;SessionID=114</t>
         </is>
       </c>
     </row>
@@ -42756,12 +42744,12 @@
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>RI</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>2026 SB 345 (Chapter 463; cross-filed HB 1214)</t>
+          <t>2026 S 2347 Sub A (P.L. 2026, ch. 180) / H 8213 Sub A (P.L. 2026, ch. 179)</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
@@ -42776,7 +42764,7 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>MVA hearing route for association disputes; no change since baseline.</t>
+          <t>Actual-technician-time warranty labor rule; no change since baseline.</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
@@ -42786,7 +42774,7 @@
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>https://mgaleg.maryland.gov/mgawebsite/Legislation/Details/sb0345?ys=2026RS</t>
+          <t>https://webserver.rilegislature.gov/PublicLaws/law26/law26180.htm</t>
         </is>
       </c>
     </row>
@@ -42803,38 +42791,42 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_recent</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>SB 1182 (2025-26), PN 1866</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="inlineStr"/>
+          <t>LB972 (2026), Sec. 70</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>No new action found in search this run (not re-verified on the official site; prior status carried forward).</t>
+          <t>Effective 10/01/2026 reached; no lawsuit or injunction found in search.</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>No committee action since referral; still pending.</t>
+          <t>RV scope carve-out; no change since baseline.</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>Watch only, unchanged.</t>
+          <t>Now in effect; site date selector applies it automatically. No data change.</t>
         </is>
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
-          <t>https://www.palegis.us/legislation/bills/2025/sb1182</t>
+          <t>https://nebraskalegislature.gov/FloorDocs/109/PDF/Slip/LB972.pdf</t>
         </is>
       </c>
     </row>
@@ -42851,38 +42843,42 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_recent</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>CT</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>A8773 (Magnarelli) / S8360 (Cooney), 2025-26</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr"/>
+          <t>Public Act 26-24 (sSB 413), §§ 20-25</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>Official record: passed Assembly 06/01/2026, delivered to Senate, referred to Rules. No Senate action since.</t>
+          <t>Effective 10/01/2026 reached; no lawsuit or injunction found in search.</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>No Senate action since referral; still pending.</t>
+          <t>Stop-sale/recall inventory compensation; no change since baseline.</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>Watch only, unchanged.</t>
+          <t>Now in effect; site date selector applies it automatically. No data change.</t>
         </is>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>https://nyassembly.gov/leg/?default_fld=&amp;leg_video=&amp;bn=A08773&amp;term=2025&amp;Summary=Y&amp;Actions=Y</t>
+          <t>https://www.cga.ct.gov/2026/ACT/PA/PDF/2026PA-00024-R00SB-00413-PA.PDF</t>
         </is>
       </c>
     </row>
@@ -42899,194 +42895,186 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_recent</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>MD</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>SB1939 (104th GA), as amended by Senate Floor Amendments 1-2</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="inlineStr"/>
+          <t>2026 SB 345 (Chapter 463; cross-filed HB 1214)</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>No new action found in search this run (not re-verified on the official site; prior status carried forward).</t>
+          <t>Effective 10/01/2026 reached; no lawsuit or injunction found in search.</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>No House action since Rules re-assignment; still pending.</t>
+          <t>MVA hearing route for association disputes; no change since baseline.</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>Watch only, unchanged.</t>
+          <t>Now in effect; site date selector applies it automatically. No data change.</t>
         </is>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
-          <t>https://www.ilga.gov/Legislation/BillStatus?DocNum=1939&amp;GAID=18&amp;DocTypeID=SB&amp;SessionID=114</t>
+          <t>https://mgaleg.maryland.gov/mgawebsite/Legislation/Details/sb0345?ys=2026RS</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
+          <t>0 enacted changes, 3 pending bills (1 moved earlier than logged), 0 law-data updates; 4 laws reached 10/1/2026 effective date</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>enacted_upcoming</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>RI</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>2026 S 2347 Sub A (P.L. 2026, ch. 180) / H 8213 Sub A (P.L. 2026, ch. 179)</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>SB 1182 (2025-26), PN 1866</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr"/>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>Confirmed unchanged: signed 06/22/2026, takes effect 10/01/2026. No lawsuit or injunction against the actual-time law found in a fresh search.</t>
+          <t>No new action found in search this run (not re-verified on the official site; prior status carried forward).</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>Actual-technician-time warranty labor rule; no change since baseline.</t>
+          <t>No committee action since referral; still pending.</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>No change from baseline.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t>https://webserver.rilegislature.gov/PublicLaws/law26/law26180.htm</t>
+          <t>https://www.palegis.us/legislation/bills/2025/sb1182</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
+          <t>0 enacted changes, 3 pending bills (1 moved earlier than logged), 0 law-data updates; 4 laws reached 10/1/2026 effective date</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>enacted_upcoming</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>LB972 (2026), Sec. 70</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>A8773 (Magnarelli) / S8360 (Cooney), 2025-26</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr"/>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>Confirmed unchanged: approved 04/14/2026, Sec. 70 operative 10/01/2026 per Sec. 84.</t>
+          <t>Official record: passed Assembly 06/01/2026, delivered to Senate, referred to Rules. No Senate action since.</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>RV scope carve-out; no change since baseline.</t>
+          <t>No Senate action since referral; still pending.</t>
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr">
         <is>
-          <t>No change from baseline.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t>https://nebraskalegislature.gov/FloorDocs/109/PDF/Slip/LB972.pdf</t>
+          <t>https://nyassembly.gov/leg/?default_fld=&amp;leg_video=&amp;bn=A08773&amp;term=2025&amp;Summary=Y&amp;Actions=Y</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
+          <t>0 enacted changes, 3 pending bills (1 moved earlier than logged), 0 law-data updates; 4 laws reached 10/1/2026 effective date</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>enacted_upcoming</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>CT</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>Public Act 26-24 (sSB 413), §§ 20-25</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>SB1939 (104th GA), as amended by Senate Floor Amendments 1-2</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr"/>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Confirmed unchanged: signed 05/27/2026, §§ 20-25 effective 10/01/2026.</t>
+          <t>No new action found in search this run (not re-verified on the official site; prior status carried forward).</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>Stop-sale/recall inventory compensation; no change since baseline.</t>
+          <t>No House action since Rules re-assignment; still pending.</t>
         </is>
       </c>
       <c r="I20" s="6" t="inlineStr">
         <is>
-          <t>No change from baseline.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
-          <t>https://www.cga.ct.gov/2026/ACT/PA/PDF/2026PA-00024-R00SB-00413-PA.PDF</t>
+          <t>https://www.ilga.gov/Legislation/BillStatus?DocNum=1939&amp;GAID=18&amp;DocTypeID=SB&amp;SessionID=114</t>
         </is>
       </c>
     </row>
@@ -43108,12 +43096,12 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>RI</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>2026 SB 345 (Chapter 463; cross-filed HB 1214)</t>
+          <t>2026 S 2347 Sub A (P.L. 2026, ch. 180) / H 8213 Sub A (P.L. 2026, ch. 179)</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
@@ -43123,12 +43111,12 @@
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>Confirmed unchanged: approved 05/12/2026, effective 10/01/2026.</t>
+          <t>Confirmed unchanged: signed 06/22/2026, takes effect 10/01/2026. No lawsuit or injunction against the actual-time law found in a fresh search.</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>MVA hearing route for association disputes; no change since baseline.</t>
+          <t>Actual-technician-time warranty labor rule; no change since baseline.</t>
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr">
@@ -43138,7 +43126,7 @@
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
-          <t>https://mgaleg.maryland.gov/mgawebsite/Legislation/Details/sb0345?ys=2026RS</t>
+          <t>https://webserver.rilegislature.gov/PublicLaws/law26/law26180.htm</t>
         </is>
       </c>
     </row>
@@ -43155,38 +43143,42 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_upcoming</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>SB 1182 (2025-26), PN 1866</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="inlineStr"/>
+          <t>LB972 (2026), Sec. 70</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>Re-checked via palegis.us (bill page returned a server error on two attempts; corroborated via a bill-tracking aggregator citing the official record) and web search. Still 'in committee': House Commerce Committee, last action 07/01/2026. No House floor action found.</t>
+          <t>Confirmed unchanged: approved 04/14/2026, Sec. 70 operative 10/01/2026 per Sec. 84.</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>No committee action since referral; still pending.</t>
+          <t>RV scope carve-out; no change since baseline.</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr">
         <is>
-          <t>Watch only, unchanged.</t>
+          <t>No change from baseline.</t>
         </is>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
-          <t>https://www.palegis.us/legislation/bills/2025/sb1182</t>
+          <t>https://nebraskalegislature.gov/FloorDocs/109/PDF/Slip/LB972.pdf</t>
         </is>
       </c>
     </row>
@@ -43203,38 +43195,42 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_upcoming</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>CT</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>A8773 (Magnarelli) / S8360 (Cooney), 2025-26</t>
-        </is>
-      </c>
-      <c r="F23" s="6" t="inlineStr"/>
+          <t>Public Act 26-24 (sSB 413), §§ 20-25</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>Re-checked on nyassembly.gov: A8773's last action is still 06/01/2026 (referred to Senate Rules); no further Senate action found.</t>
+          <t>Confirmed unchanged: signed 05/27/2026, §§ 20-25 effective 10/01/2026.</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>No Senate action since referral; still pending.</t>
+          <t>Stop-sale/recall inventory compensation; no change since baseline.</t>
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr">
         <is>
-          <t>Watch only, unchanged.</t>
+          <t>No change from baseline.</t>
         </is>
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
-          <t>https://nyassembly.gov/leg/?default_fld=&amp;leg_video=&amp;bn=A08773&amp;term=2025&amp;Summary=Y&amp;Actions=Y</t>
+          <t>https://www.cga.ct.gov/2026/ACT/PA/PDF/2026PA-00024-R00SB-00413-PA.PDF</t>
         </is>
       </c>
     </row>
@@ -43251,194 +43247,186 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_upcoming</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>MD</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>SB1939 (104th GA), as amended by Senate Floor Amendments 1-2</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr"/>
+          <t>2026 SB 345 (Chapter 463; cross-filed HB 1214)</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>Re-checked via web search (ilga.gov bill-status page returned a server error). Still pending in House Rules Committee since 03/20/2026; spring session adjourned 06/01/2026 with no further action.</t>
+          <t>Confirmed unchanged: approved 05/12/2026, effective 10/01/2026.</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>No House action since Rules re-assignment; still pending.</t>
+          <t>MVA hearing route for association disputes; no change since baseline.</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr">
         <is>
-          <t>Watch only, unchanged.</t>
+          <t>No change from baseline.</t>
         </is>
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
-          <t>https://www.ilga.gov/Legislation/BillStatus?DocNum=1939&amp;GAID=18&amp;DocTypeID=SB&amp;SessionID=114</t>
+          <t>https://mgaleg.maryland.gov/mgawebsite/Legislation/Details/sb0345?ys=2026RS</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Baseline: 4 enacted changes take effect Oct 1, 2026 (RI, NE, CT, MD); 3 bills still pending (PA, NY, IL)</t>
+          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>enacted_upcoming</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>RI</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>2026 S 2347 Sub A (P.L. 2026, ch. 180) / H 8213 Sub A (P.L. 2026, ch. 179)</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>SB 1182 (2025-26), PN 1866</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr"/>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>Signed by Governor 06/22/2026 (S 2347 Sub A = Chapter 180; H 8213 Sub A = Chapter 179); takes effect 10/01/2026</t>
+          <t>Re-checked via palegis.us (bill page returned a server error on two attempts; corroborated via a bill-tracking aggregator citing the official record) and web search. Still 'in committee': House Commerce Committee, last action 07/01/2026. No House floor action found.</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>Amends R.I. Gen. Laws § 31-5.1-6 and related sections. Warranty labor is paid at the dealer's non-warranty labor rate multiplied by the ACTUAL time the technician worked.</t>
+          <t>No committee action since referral; still pending.</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
         <is>
-          <t>Already reflected: date selector switches RI to actual technician time and CPO Required on 10/1/2026.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
-          <t>https://webserver.rilegislature.gov/PublicLaws/law26/law26180.htm</t>
+          <t>https://www.palegis.us/legislation/bills/2025/sb1182</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Baseline: 4 enacted changes take effect Oct 1, 2026 (RI, NE, CT, MD); 3 bills still pending (PA, NY, IL)</t>
+          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>enacted_upcoming</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>LB972 (2026), Sec. 70</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>A8773 (Magnarelli) / S8360 (Cooney), 2025-26</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr"/>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>Passed 48-1-0 on 04/10/2026; approved by Governor 04/14/2026. Sec. 84 makes Sec. 70 operative 10/01/2026.</t>
+          <t>Re-checked on nyassembly.gov: A8773's last action is still 06/01/2026 (referred to Senate Rules); no further Senate action found.</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>Sec. 70 adds § 60-1438(7): 'This section does not apply to recreational vehicles.' RVs move to the new Recreational Vehicle Industry Regulation Act. A word diff of Sec.</t>
+          <t>No Senate action since referral; still pending.</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
         <is>
-          <t>Scope only (RVs removed). No change to passenger-vehicle cells.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
-          <t>https://nebraskalegislature.gov/FloorDocs/109/PDF/Slip/LB972.pdf</t>
+          <t>https://nyassembly.gov/leg/?default_fld=&amp;leg_video=&amp;bn=A08773&amp;term=2025&amp;Summary=Y&amp;Actions=Y</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Baseline: 4 enacted changes take effect Oct 1, 2026 (RI, NE, CT, MD); 3 bills still pending (PA, NY, IL)</t>
+          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>enacted_upcoming</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>CT</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>Public Act 26-24 (sSB 413), §§ 20-25</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>SB1939 (104th GA), as amended by Senate Floor Amendments 1-2</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr"/>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>Signed by Governor 05/27/2026 (per the cga.ct.gov bill status page); §§ 20-25 effective 10/01/2026</t>
+          <t>Re-checked via web search (ilga.gov bill-status page returned a server error). Still pending in House Rules Committee since 03/20/2026; spring session adjourned 06/01/2026 with no further action.</t>
         </is>
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>New § 22 covers used vehicles in a dealer's inventory that are under a stop-sale or do-not-drive order for a federal safety or emissions recall.</t>
+          <t>No House action since Rules re-assignment; still pending.</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
         <is>
-          <t>Claim rules extend to stop-sale compensation claims. Labor rate and time cells unchanged.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
-          <t>https://www.cga.ct.gov/2026/ACT/PA/PDF/2026PA-00024-R00SB-00413-PA.PDF</t>
+          <t>https://www.ilga.gov/Legislation/BillStatus?DocNum=1939&amp;GAID=18&amp;DocTypeID=SB&amp;SessionID=114</t>
         </is>
       </c>
     </row>
@@ -43460,12 +43448,12 @@
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>RI</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>2026 SB 345 (Chapter 463; cross-filed HB 1214)</t>
+          <t>2026 S 2347 Sub A (P.L. 2026, ch. 180) / H 8213 Sub A (P.L. 2026, ch. 179)</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
@@ -43475,22 +43463,22 @@
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>Approved by Governor 05/12/2026 (Chapter 463); effective 10/01/2026</t>
+          <t>Signed by Governor 06/22/2026 (S 2347 Sub A = Chapter 180; H 8213 Sub A = Chapter 179); takes effect 10/01/2026</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>Procedural, with an indirect effect on warranty. A dealer association or manufacturer association may request an MVA administrative hearing to resolve a dispute or to get an interpretation of the franchise law, which includes the § 15-212 warranty rules.</t>
+          <t>Amends R.I. Gen. Laws § 31-5.1-6 and related sections. Warranty labor is paid at the dealer's non-warranty labor rate multiplied by the ACTUAL time the technician worked.</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr">
         <is>
-          <t>Procedural (association hearings). No change to § 15-212 cells.</t>
+          <t>Already reflected: date selector switches RI to actual technician time and CPO Required on 10/1/2026.</t>
         </is>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>https://mgaleg.maryland.gov/mgawebsite/Legislation/Details/sb0345?ys=2026RS</t>
+          <t>https://webserver.rilegislature.gov/PublicLaws/law26/law26180.htm</t>
         </is>
       </c>
     </row>
@@ -43507,42 +43495,42 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>enacted_recent</t>
+          <t>enacted_upcoming</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>2026 HB 648 (2026 Ky. Acts ch. 83), amending KRS 190.046</t>
+          <t>LB972 (2026), Sec. 70</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>Signed by Governor 04/10/2026 (Acts Ch. 83); the official KRS 190.046 page shows 'Effective: July 15, 2026'</t>
+          <t>Passed 48-1-0 on 04/10/2026; approved by Governor 04/14/2026. Sec. 84 makes Sec. 70 operative 10/01/2026.</t>
         </is>
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>Rewrites KRS 190.046(2)(d) for vehicles in Class 7 and above (49 C.F.R. 565.15, heavy trucks) and makes component manufacturers liable. Parts are paid at acquisition cost plus a 30% gross margin.</t>
+          <t>Sec. 70 adds § 60-1438(7): 'This section does not apply to recreational vehicles.' RVs move to the new Recreational Vehicle Industry Regulation Act. A word diff of Sec.</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
         <is>
-          <t>Class 7+ heavy trucks only; noted in KY record. Light-duty cells unchanged.</t>
+          <t>Scope only (RVs removed). No change to passenger-vehicle cells.</t>
         </is>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
-          <t>https://apps.legislature.ky.gov/record/26rs/hb648.html</t>
+          <t>https://nebraskalegislature.gov/FloorDocs/109/PDF/Slip/LB972.pdf</t>
         </is>
       </c>
     </row>
@@ -43559,38 +43547,42 @@
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_upcoming</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>CT</t>
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>SB 1182 (2025-26), PN 1866</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="inlineStr"/>
+          <t>Public Act 26-24 (sSB 413), §§ 20-25</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>Passed Senate 50-0 on 06/30/2026; referred to House COMMERCE Committee 07/01/2026; no House action since. The 2025-26 session ends 11/30/2026 and the bill dies if not enacted.</t>
+          <t>Signed by Governor 05/27/2026 (per the cga.ct.gov bill status page); §§ 20-25 effective 10/01/2026</t>
         </is>
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>Would amend Board of Vehicles Act § 307 to expressly cover extended warranty, CPO warranty, manufacturer-sponsored maintenance programs, parts-exchange programs and 'a service contract issued by a manufacturer or distributor or its common entity'.</t>
+          <t>New § 22 covers used vehicles in a dealer's inventory that are under a stop-sale or do-not-drive order for a federal safety or emissions recall.</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr">
         <is>
-          <t>Watch only. If enacted, PA service-contract and CPO cells would change.</t>
+          <t>Claim rules extend to stop-sale compensation claims. Labor rate and time cells unchanged.</t>
         </is>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>https://www.palegis.us/legislation/bills/2025/sb1182</t>
+          <t>https://www.cga.ct.gov/2026/ACT/PA/PDF/2026PA-00024-R00SB-00413-PA.PDF</t>
         </is>
       </c>
     </row>
@@ -43607,38 +43599,42 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_upcoming</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>MD</t>
         </is>
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>A8773 (Magnarelli) / S8360 (Cooney), 2025-26</t>
-        </is>
-      </c>
-      <c r="F31" s="6" t="inlineStr"/>
+          <t>2026 SB 345 (Chapter 463; cross-filed HB 1214)</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>A8773 passed the Assembly 06/01/2026, went to the Senate and was referred to Senate RULES the same day. S8360 has been in Senate TRANSPORTATION since 01/07/2026. The Senate has not acted; the bills die 12/31/2026.</t>
+          <t>Approved by Governor 05/12/2026 (Chapter 463); effective 10/01/2026</t>
         </is>
       </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t>Would amend VTL § 465 to cover affiliates and subsidiaries and to list 'extended service contract repairs', 'component part warranties' and 'any other franchisor compensated repairs'.</t>
+          <t>Procedural, with an indirect effect on warranty. A dealer association or manufacturer association may request an MVA administrative hearing to resolve a dispute or to get an interpretation of the franchise law, which includes the § 15-212 warranty rules.</t>
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr">
         <is>
-          <t>Watch only. If enacted, NY paid-hours rules would add 1.5× and actual-time fallbacks.</t>
+          <t>Procedural (association hearings). No change to § 15-212 cells.</t>
         </is>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
-          <t>https://nyassembly.gov/leg/?default_fld=&amp;leg_video=&amp;bn=A08773&amp;term=2025&amp;Summary=Y&amp;Actions=Y</t>
+          <t>https://mgaleg.maryland.gov/mgawebsite/Legislation/Details/sb0345?ys=2026RS</t>
         </is>
       </c>
     </row>
@@ -43655,38 +43651,42 @@
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_recent</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>KY</t>
         </is>
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>SB1939 (104th GA), as amended by Senate Floor Amendments 1-2</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="inlineStr"/>
+          <t>2026 HB 648 (2026 Ky. Acts ch. 83), amending KRS 190.046</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
-          <t>Passed Senate 55-0 on 04/10/2025. In the House it was re-assigned to the Rules Committee on 03/20/2026. It could move in the fall veto session (House session days Nov 17-19 and Dec 1-3, 2026) or the lame-duck session before the 104th GA ends in January 2027.</t>
+          <t>Signed by Governor 04/10/2026 (Acts Ch. 83); the official KRS 190.046 page shows 'Effective: July 15, 2026'</t>
         </is>
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>Mainly a direct-sales ban: an OEM not licensed to sell direct before 1/1/2022 may not own or operate a dealership or sell direct. It also amends 815 ILCS 710/6.</t>
+          <t>Rewrites KRS 190.046(2)(d) for vehicles in Class 7 and above (49 C.F.R. 565.15, heavy trucks) and makes component manufacturers liable. Parts are paid at acquisition cost plus a 30% gross margin.</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
         <is>
-          <t>Watch only. Mostly a direct-sales bill; parts-markup maintenance definition would change.</t>
+          <t>Class 7+ heavy trucks only; noted in KY record. Light-duty cells unchanged.</t>
         </is>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
-          <t>https://www.ilga.gov/Legislation/BillStatus?DocNum=1939&amp;GAID=18&amp;DocTypeID=SB&amp;SessionID=114</t>
+          <t>https://apps.legislature.ky.gov/record/26rs/hb648.html</t>
         </is>
       </c>
     </row>
@@ -43703,43 +43703,187 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>dead_or_stalled</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>H4019 (194th General Court), 'An Act to ensure fair compensation for warranty service labor'</t>
+          <t>SB 1182 (2025-26), PN 1866</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr"/>
       <c r="G33" s="6" t="inlineStr">
         <is>
+          <t>Passed Senate 50-0 on 06/30/2026; referred to House COMMERCE Committee 07/01/2026; no House action since. The 2025-26 session ends 11/30/2026 and the bill dies if not enacted.</t>
+        </is>
+      </c>
+      <c r="H33" s="6" t="inlineStr">
+        <is>
+          <t>Would amend Board of Vehicles Act § 307 to expressly cover extended warranty, CPO warranty, manufacturer-sponsored maintenance programs, parts-exchange programs and 'a service contract issued by a manufacturer or distributor or its common entity'.</t>
+        </is>
+      </c>
+      <c r="I33" s="6" t="inlineStr">
+        <is>
+          <t>Watch only. If enacted, PA service-contract and CPO cells would change.</t>
+        </is>
+      </c>
+      <c r="J33" s="6" t="inlineStr">
+        <is>
+          <t>https://www.palegis.us/legislation/bills/2025/sb1182</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>Baseline: 4 enacted changes take effect Oct 1, 2026 (RI, NE, CT, MD); 3 bills still pending (PA, NY, IL)</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>A8773 (Magnarelli) / S8360 (Cooney), 2025-26</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="inlineStr"/>
+      <c r="G34" s="6" t="inlineStr">
+        <is>
+          <t>A8773 passed the Assembly 06/01/2026, went to the Senate and was referred to Senate RULES the same day. S8360 has been in Senate TRANSPORTATION since 01/07/2026. The Senate has not acted; the bills die 12/31/2026.</t>
+        </is>
+      </c>
+      <c r="H34" s="6" t="inlineStr">
+        <is>
+          <t>Would amend VTL § 465 to cover affiliates and subsidiaries and to list 'extended service contract repairs', 'component part warranties' and 'any other franchisor compensated repairs'.</t>
+        </is>
+      </c>
+      <c r="I34" s="6" t="inlineStr">
+        <is>
+          <t>Watch only. If enacted, NY paid-hours rules would add 1.5× and actual-time fallbacks.</t>
+        </is>
+      </c>
+      <c r="J34" s="6" t="inlineStr">
+        <is>
+          <t>https://nyassembly.gov/leg/?default_fld=&amp;leg_video=&amp;bn=A08773&amp;term=2025&amp;Summary=Y&amp;Actions=Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>Baseline: 4 enacted changes take effect Oct 1, 2026 (RI, NE, CT, MD); 3 bills still pending (PA, NY, IL)</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t>SB1939 (104th GA), as amended by Senate Floor Amendments 1-2</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="inlineStr"/>
+      <c r="G35" s="6" t="inlineStr">
+        <is>
+          <t>Passed Senate 55-0 on 04/10/2025. In the House it was re-assigned to the Rules Committee on 03/20/2026. It could move in the fall veto session (House session days Nov 17-19 and Dec 1-3, 2026) or the lame-duck session before the 104th GA ends in January 2027.</t>
+        </is>
+      </c>
+      <c r="H35" s="6" t="inlineStr">
+        <is>
+          <t>Mainly a direct-sales ban: an OEM not licensed to sell direct before 1/1/2022 may not own or operate a dealership or sell direct. It also amends 815 ILCS 710/6.</t>
+        </is>
+      </c>
+      <c r="I35" s="6" t="inlineStr">
+        <is>
+          <t>Watch only. Mostly a direct-sales bill; parts-markup maintenance definition would change.</t>
+        </is>
+      </c>
+      <c r="J35" s="6" t="inlineStr">
+        <is>
+          <t>https://www.ilga.gov/Legislation/BillStatus?DocNum=1939&amp;GAID=18&amp;DocTypeID=SB&amp;SessionID=114</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>Baseline: 4 enacted changes take effect Oct 1, 2026 (RI, NE, CT, MD); 3 bills still pending (PA, NY, IL)</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>dead_or_stalled</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>H4019 (194th General Court), 'An Act to ensure fair compensation for warranty service labor'</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr"/>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
           <t>Accompanied a study order (see H5320) on 04/02/2026, which means it is effectively dead. Formal sessions ended 07/31/2026.</t>
         </is>
       </c>
-      <c r="H33" s="6" t="inlineStr">
+      <c r="H36" s="6" t="inlineStr">
         <is>
           <t>Would have let dealers base warranty labor time on aftermarket or retail time guides. Hearing held 02/04/2026 before the Joint Committee on Consumer Protection and Professional Licensure.</t>
         </is>
       </c>
-      <c r="I33" s="6" t="inlineStr">
+      <c r="I36" s="6" t="inlineStr">
         <is>
           <t>Effectively dead (study order). No action.</t>
         </is>
       </c>
-      <c r="J33" s="6" t="inlineStr">
+      <c r="J36" s="6" t="inlineStr">
         <is>
           <t>https://malegislature.gov/Bills/194/H4019/BillHistory</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J33"/>
+  <autoFilter ref="A1:J36"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Audit brief PDF: summary table on page 1, numbered notes on page 2
</commit_message>
<xml_diff>
--- a/docs/downloads/warranty-atlas.xlsx
+++ b/docs/downloads/warranty-atlas.xlsx
@@ -42158,7 +42158,7 @@
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>Audit brief added for Florida, California, Illinois and Arkansas: what to know before auditing paid factory-warranty claims, on the state page and as a one-page PDF; 10 matrix fields corrected</t>
+          <t>Audit brief added for Florida, California, Illinois and Arkansas: what to know before auditing paid factory-warranty claims, on the state page and as a PDF (summary table plus notes); 10 matrix fields corrected</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
@@ -42206,7 +42206,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Audit brief added for Florida, California, Illinois and Arkansas: what to know before auditing paid factory-warranty claims, on the state page and as a one-page PDF; 10 matrix fields corrected</t>
+          <t>Audit brief added for Florida, California, Illinois and Arkansas: what to know before auditing paid factory-warranty claims, on the state page and as a PDF (summary table plus notes); 10 matrix fields corrected</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -42254,7 +42254,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Audit brief added for Florida, California, Illinois and Arkansas: what to know before auditing paid factory-warranty claims, on the state page and as a one-page PDF; 10 matrix fields corrected</t>
+          <t>Audit brief added for Florida, California, Illinois and Arkansas: what to know before auditing paid factory-warranty claims, on the state page and as a PDF (summary table plus notes); 10 matrix fields corrected</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Four-state research review applied: practice lines, California protest clock, Illinois provisional score, narrowed readings
</commit_message>
<xml_diff>
--- a/docs/downloads/warranty-atlas.xlsx
+++ b/docs/downloads/warranty-atlas.xlsx
@@ -2266,7 +2266,7 @@
       </c>
       <c r="O15" s="6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Unresolved (conflict in statute)</t>
         </is>
       </c>
       <c r="P15" s="6" t="inlineStr">
@@ -9748,7 +9748,7 @@
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>Points = weight × level ÷ 3. Score = sum of points (0–100). Weights are a judgment call about how much each limit constrains audits and chargebacks, and are a draft that may change. Levels are read from the statute text and, where a state agency rule sets the limit, from that rule. The score measures how strict the law is, not how likely an audit dispute is.</t>
+          <t>Points = weight × level ÷ 3. Score = sum of points (0–100). Weights are a judgment call about how much each limit constrains audits and chargebacks, and are a draft that may change. Levels are read from the statute text and, where a state agency rule sets the limit, from that rule. A limit marked provisional rests on statute text that conflicts with itself (recorded as unresolved, with a reason); that state's score is shown with its range until the reading is settled. The score measures how strict the law is, not how likely an audit dispute is.</t>
         </is>
       </c>
     </row>
@@ -26194,7 +26194,7 @@
       </c>
       <c r="N6" s="6" t="inlineStr">
         <is>
-          <t>Audits on a reasonable basis, never punitive, retaliatory or unfairly discriminatory, and no more than one random audit per 9 months (any additional audit needs written disclosure of its basis). Chargeback grounds are the same four as the denial grounds. No extrapolation unless the sample is random and the method statistically valid. Written notice of specific grounds within 30 days after the audit, then at least 30 days (scaled to claim volume) to rebut or cure. No chargeback until 45 days after the later of the disapproval or Final Denial notice, and it must be taken within 90 days of that notice. A Board protest filed within 6 months of that notice (or the end of the appeal process) and before the chargeback stays offset or collection until the Board's final order, after which the franchisor has 90 days.</t>
+          <t>Audits on a reasonable basis, never punitive, retaliatory or unfairly discriminatory, and no more than one random audit per 9 months (any additional audit needs written disclosure of its basis). Chargeback grounds are the same four as the denial grounds. No extrapolation unless the sample is random and the method statistically valid. Written notice of specific grounds within 30 days after the audit, then at least 30 days (scaled to claim volume) to rebut or cure. No chargeback until 45 days after the later of the disapproval or Final Denial notice, and it must be taken within 90 days of that notice. A Board protest filed within 6 months after the later of the disapproval notice or the end of the appeal process, and before the chargeback, stays offset or collection until the Board's final order, after which the franchisor has 90 days.</t>
         </is>
       </c>
       <c r="O6" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Weekly check 2026-10-26: 0 enacted changes, 3 pending bills unchanged, 0 law-data updates
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0184G451sX47VFdw2BDCwr2Q
</commit_message>
<xml_diff>
--- a/docs/downloads/warranty-atlas.xlsx
+++ b/docs/downloads/warranty-atlas.xlsx
@@ -26,7 +26,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Rate sample rules'!$A$1:$L$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Law dates'!$A$1:$M$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Governing bodies'!$A$1:$J$51</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Weekly log'!$A$1:$J$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Weekly log'!$A$1:$J$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'News'!$A$1:$J$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Audit procedures'!$A$1:$X$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Audit climate'!$A$1:$V$51</definedName>
@@ -497,7 +497,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Built 2026-10-23 from the live Atlas data files.</t>
+          <t>Built 2026-10-26 from the live Atlas data files.</t>
         </is>
       </c>
     </row>
@@ -42083,7 +42083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J36"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -42153,12 +42153,12 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>Audit brief added for Florida, California, Illinois and Arkansas: what to know before auditing paid factory-warranty claims, on the state page and as a PDF (summary table plus notes); 10 matrix fields corrected</t>
+          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
@@ -42179,12 +42179,12 @@
       <c r="F2" s="6" t="inlineStr"/>
       <c r="G2" s="6" t="inlineStr">
         <is>
-          <t>Official page returned HTTP 503 this run; search found no new action. Prior status carried forward. Not law.</t>
+          <t>Re-checked on palegis.us 2026-10-26: passed Senate 50-0 on 06/30/2026, referred to House Commerce 07/01/2026. A Commerce Committee voting meeting is listed for 10/05/2026 but the page records no outcome. Not law.</t>
         </is>
       </c>
       <c r="H2" s="6" t="inlineStr">
         <is>
-          <t>No committee action since referral; still pending.</t>
+          <t>In House Commerce; listed for a 10/5 committee vote with no recorded outcome.</t>
         </is>
       </c>
       <c r="I2" s="6" t="inlineStr">
@@ -42201,12 +42201,12 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Audit brief added for Florida, California, Illinois and Arkansas: what to know before auditing paid factory-warranty claims, on the state page and as a PDF (summary table plus notes); 10 matrix fields corrected</t>
+          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -42227,7 +42227,7 @@
       <c r="F3" s="6" t="inlineStr"/>
       <c r="G3" s="6" t="inlineStr">
         <is>
-          <t>Re-checked on nyassembly.gov 10/19/2026: passed Assembly 06/01/2026, delivered to Senate, referred to Rules; no Senate action since.</t>
+          <t>Re-checked on nyassembly.gov 10/26/2026: passed Assembly 06/01/2026, delivered to Senate, referred to Rules; no Senate action since.</t>
         </is>
       </c>
       <c r="H3" s="6" t="inlineStr">
@@ -42249,12 +42249,12 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Audit brief added for Florida, California, Illinois and Arkansas: what to know before auditing paid factory-warranty claims, on the state page and as a PDF (summary table plus notes); 10 matrix fields corrected</t>
+          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -42275,7 +42275,7 @@
       <c r="F4" s="6" t="inlineStr"/>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>Official page returned HTTP 503 this run; search found no new action. Prior status carried forward. Not law.</t>
+          <t>Official page returned HTTP 503 again this run; no new action found by search. Prior status carried forward. Not law.</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
@@ -42297,12 +42297,12 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
+          <t>Audit brief added for Florida, California, Illinois and Arkansas: what to know before auditing paid factory-warranty claims, on the state page and as a PDF (summary table plus notes); 10 matrix fields corrected</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -42345,12 +42345,12 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
+          <t>Audit brief added for Florida, California, Illinois and Arkansas: what to know before auditing paid factory-warranty claims, on the state page and as a PDF (summary table plus notes); 10 matrix fields corrected</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -42393,12 +42393,12 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
+          <t>Audit brief added for Florida, California, Illinois and Arkansas: what to know before auditing paid factory-warranty claims, on the state page and as a PDF (summary table plus notes); 10 matrix fields corrected</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -42441,7 +42441,7 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
@@ -42467,7 +42467,7 @@
       <c r="F8" s="6" t="inlineStr"/>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Official page returned HTTP 503 this run; search found no new action. Prior status carried forward (House Commerce, last action 07/01/2026). Not law.</t>
+          <t>Official page returned HTTP 503 this run; search found no new action. Prior status carried forward. Not law.</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
@@ -42489,7 +42489,7 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
@@ -42515,7 +42515,7 @@
       <c r="F9" s="6" t="inlineStr"/>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Re-checked on nyassembly.gov 10/12/2026: passed Assembly 06/01/2026, referred to Senate Rules; no Senate action.</t>
+          <t>Re-checked on nyassembly.gov 10/19/2026: passed Assembly 06/01/2026, delivered to Senate, referred to Rules; no Senate action since.</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
@@ -42537,7 +42537,7 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -42563,7 +42563,7 @@
       <c r="F10" s="6" t="inlineStr"/>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Official page returned HTTP 503 this run; search found no new action. Prior status carried forward (House Rules). Not law.</t>
+          <t>Official page returned HTTP 503 this run; search found no new action. Prior status carried forward. Not law.</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
@@ -42585,12 +42585,12 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Source review: all 50 states' agency rules checked; Tennessee limits added from Commission rules; Rhode Island 10/1 law moved into current data; 23 matrix fields updated</t>
+          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -42611,7 +42611,7 @@
       <c r="F11" s="6" t="inlineStr"/>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Pending in House Commerce (hearing listed 10/5/2026); not law.</t>
+          <t>Official page returned HTTP 503 this run; search found no new action. Prior status carried forward (House Commerce, last action 07/01/2026). Not law.</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
@@ -42633,12 +42633,12 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Source review: all 50 states' agency rules checked; Tennessee limits added from Commission rules; Rhode Island 10/1 law moved into current data; 23 matrix fields updated</t>
+          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -42659,7 +42659,7 @@
       <c r="F12" s="6" t="inlineStr"/>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Passed Assembly 06/01/2026; in Senate Rules. No Senate action (official record checked 10/6/2026).</t>
+          <t>Re-checked on nyassembly.gov 10/12/2026: passed Assembly 06/01/2026, referred to Senate Rules; no Senate action.</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
@@ -42681,12 +42681,12 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Source review: all 50 states' agency rules checked; Tennessee limits added from Commission rules; Rhode Island 10/1 law moved into current data; 23 matrix fields updated</t>
+          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -42707,7 +42707,7 @@
       <c r="F13" s="6" t="inlineStr"/>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>No new action found in search this run (not re-verified on the official site; prior status carried forward). Still pending as of 10/6/2026 (HB5197, introduced 2/10/2026, also in House Rules).</t>
+          <t>Official page returned HTTP 503 this run; search found no new action. Prior status carried forward (House Rules). Not law.</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
@@ -42729,156 +42729,144 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>0 enacted changes, 3 pending bills (1 moved earlier than logged), 0 law-data updates; 4 laws reached 10/1/2026 effective date</t>
+          <t>Source review: all 50 states' agency rules checked; Tennessee limits added from Commission rules; Rhode Island 10/1 law moved into current data; 23 matrix fields updated</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>enacted_recent</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>RI</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>2026 S 2347 Sub A (P.L. 2026, ch. 180) / H 8213 Sub A (P.L. 2026, ch. 179)</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>SB 1182 (2025-26), PN 1866</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr"/>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>Effective 10/01/2026 reached; no lawsuit or injunction found in search.</t>
+          <t>Pending in House Commerce (hearing listed 10/5/2026); not law.</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>Actual-technician-time warranty labor rule; no change since baseline.</t>
+          <t>No committee action since referral; still pending.</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>Now in effect; site date selector applies it automatically. No data change.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>https://webserver.rilegislature.gov/PublicLaws/law26/law26180.htm</t>
+          <t>https://www.palegis.us/legislation/bills/2025/sb1182</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>0 enacted changes, 3 pending bills (1 moved earlier than logged), 0 law-data updates; 4 laws reached 10/1/2026 effective date</t>
+          <t>Source review: all 50 states' agency rules checked; Tennessee limits added from Commission rules; Rhode Island 10/1 law moved into current data; 23 matrix fields updated</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>enacted_recent</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>LB972 (2026), Sec. 70</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>A8773 (Magnarelli) / S8360 (Cooney), 2025-26</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr"/>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Effective 10/01/2026 reached; no lawsuit or injunction found in search.</t>
+          <t>Passed Assembly 06/01/2026; in Senate Rules. No Senate action (official record checked 10/6/2026).</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>RV scope carve-out; no change since baseline.</t>
+          <t>No Senate action since referral; still pending.</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>Now in effect; site date selector applies it automatically. No data change.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
-          <t>https://nebraskalegislature.gov/FloorDocs/109/PDF/Slip/LB972.pdf</t>
+          <t>https://nyassembly.gov/leg/?default_fld=&amp;leg_video=&amp;bn=A08773&amp;term=2025&amp;Summary=Y&amp;Actions=Y</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>0 enacted changes, 3 pending bills (1 moved earlier than logged), 0 law-data updates; 4 laws reached 10/1/2026 effective date</t>
+          <t>Source review: all 50 states' agency rules checked; Tennessee limits added from Commission rules; Rhode Island 10/1 law moved into current data; 23 matrix fields updated</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>enacted_recent</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>CT</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>Public Act 26-24 (sSB 413), §§ 20-25</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>SB1939 (104th GA), as amended by Senate Floor Amendments 1-2</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr"/>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>Effective 10/01/2026 reached; no lawsuit or injunction found in search.</t>
+          <t>No new action found in search this run (not re-verified on the official site; prior status carried forward). Still pending as of 10/6/2026 (HB5197, introduced 2/10/2026, also in House Rules).</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>Stop-sale/recall inventory compensation; no change since baseline.</t>
+          <t>No House action since Rules re-assignment; still pending.</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>Now in effect; site date selector applies it automatically. No data change.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>https://www.cga.ct.gov/2026/ACT/PA/PDF/2026PA-00024-R00SB-00413-PA.PDF</t>
+          <t>https://www.ilga.gov/Legislation/BillStatus?DocNum=1939&amp;GAID=18&amp;DocTypeID=SB&amp;SessionID=114</t>
         </is>
       </c>
     </row>
@@ -42900,12 +42888,12 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>RI</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>2026 SB 345 (Chapter 463; cross-filed HB 1214)</t>
+          <t>2026 S 2347 Sub A (P.L. 2026, ch. 180) / H 8213 Sub A (P.L. 2026, ch. 179)</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -42920,7 +42908,7 @@
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>MVA hearing route for association disputes; no change since baseline.</t>
+          <t>Actual-technician-time warranty labor rule; no change since baseline.</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
@@ -42930,7 +42918,7 @@
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
-          <t>https://mgaleg.maryland.gov/mgawebsite/Legislation/Details/sb0345?ys=2026RS</t>
+          <t>https://webserver.rilegislature.gov/PublicLaws/law26/law26180.htm</t>
         </is>
       </c>
     </row>
@@ -42947,38 +42935,42 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_recent</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>SB 1182 (2025-26), PN 1866</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="inlineStr"/>
+          <t>LB972 (2026), Sec. 70</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>No new action found in search this run (not re-verified on the official site; prior status carried forward).</t>
+          <t>Effective 10/01/2026 reached; no lawsuit or injunction found in search.</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>No committee action since referral; still pending.</t>
+          <t>RV scope carve-out; no change since baseline.</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>Watch only, unchanged.</t>
+          <t>Now in effect; site date selector applies it automatically. No data change.</t>
         </is>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t>https://www.palegis.us/legislation/bills/2025/sb1182</t>
+          <t>https://nebraskalegislature.gov/FloorDocs/109/PDF/Slip/LB972.pdf</t>
         </is>
       </c>
     </row>
@@ -42995,38 +42987,42 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_recent</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>CT</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>A8773 (Magnarelli) / S8360 (Cooney), 2025-26</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr"/>
+          <t>Public Act 26-24 (sSB 413), §§ 20-25</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>Official record: passed Assembly 06/01/2026, delivered to Senate, referred to Rules. No Senate action since.</t>
+          <t>Effective 10/01/2026 reached; no lawsuit or injunction found in search.</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>No Senate action since referral; still pending.</t>
+          <t>Stop-sale/recall inventory compensation; no change since baseline.</t>
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr">
         <is>
-          <t>Watch only, unchanged.</t>
+          <t>Now in effect; site date selector applies it automatically. No data change.</t>
         </is>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t>https://nyassembly.gov/leg/?default_fld=&amp;leg_video=&amp;bn=A08773&amp;term=2025&amp;Summary=Y&amp;Actions=Y</t>
+          <t>https://www.cga.ct.gov/2026/ACT/PA/PDF/2026PA-00024-R00SB-00413-PA.PDF</t>
         </is>
       </c>
     </row>
@@ -43043,194 +43039,186 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_recent</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>MD</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>SB1939 (104th GA), as amended by Senate Floor Amendments 1-2</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr"/>
+          <t>2026 SB 345 (Chapter 463; cross-filed HB 1214)</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>No new action found in search this run (not re-verified on the official site; prior status carried forward).</t>
+          <t>Effective 10/01/2026 reached; no lawsuit or injunction found in search.</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>No House action since Rules re-assignment; still pending.</t>
+          <t>MVA hearing route for association disputes; no change since baseline.</t>
         </is>
       </c>
       <c r="I20" s="6" t="inlineStr">
         <is>
-          <t>Watch only, unchanged.</t>
+          <t>Now in effect; site date selector applies it automatically. No data change.</t>
         </is>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
-          <t>https://www.ilga.gov/Legislation/BillStatus?DocNum=1939&amp;GAID=18&amp;DocTypeID=SB&amp;SessionID=114</t>
+          <t>https://mgaleg.maryland.gov/mgawebsite/Legislation/Details/sb0345?ys=2026RS</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
+          <t>0 enacted changes, 3 pending bills (1 moved earlier than logged), 0 law-data updates; 4 laws reached 10/1/2026 effective date</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>enacted_upcoming</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>RI</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>2026 S 2347 Sub A (P.L. 2026, ch. 180) / H 8213 Sub A (P.L. 2026, ch. 179)</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>SB 1182 (2025-26), PN 1866</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr"/>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>Confirmed unchanged: signed 06/22/2026, takes effect 10/01/2026. No lawsuit or injunction against the actual-time law found in a fresh search.</t>
+          <t>No new action found in search this run (not re-verified on the official site; prior status carried forward).</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>Actual-technician-time warranty labor rule; no change since baseline.</t>
+          <t>No committee action since referral; still pending.</t>
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr">
         <is>
-          <t>No change from baseline.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
-          <t>https://webserver.rilegislature.gov/PublicLaws/law26/law26180.htm</t>
+          <t>https://www.palegis.us/legislation/bills/2025/sb1182</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
+          <t>0 enacted changes, 3 pending bills (1 moved earlier than logged), 0 law-data updates; 4 laws reached 10/1/2026 effective date</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>enacted_upcoming</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>LB972 (2026), Sec. 70</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>A8773 (Magnarelli) / S8360 (Cooney), 2025-26</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr"/>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>Confirmed unchanged: approved 04/14/2026, Sec. 70 operative 10/01/2026 per Sec. 84.</t>
+          <t>Official record: passed Assembly 06/01/2026, delivered to Senate, referred to Rules. No Senate action since.</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>RV scope carve-out; no change since baseline.</t>
+          <t>No Senate action since referral; still pending.</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr">
         <is>
-          <t>No change from baseline.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
-          <t>https://nebraskalegislature.gov/FloorDocs/109/PDF/Slip/LB972.pdf</t>
+          <t>https://nyassembly.gov/leg/?default_fld=&amp;leg_video=&amp;bn=A08773&amp;term=2025&amp;Summary=Y&amp;Actions=Y</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
+          <t>0 enacted changes, 3 pending bills (1 moved earlier than logged), 0 law-data updates; 4 laws reached 10/1/2026 effective date</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>enacted_upcoming</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>CT</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>Public Act 26-24 (sSB 413), §§ 20-25</t>
-        </is>
-      </c>
-      <c r="F23" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>SB1939 (104th GA), as amended by Senate Floor Amendments 1-2</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr"/>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>Confirmed unchanged: signed 05/27/2026, §§ 20-25 effective 10/01/2026.</t>
+          <t>No new action found in search this run (not re-verified on the official site; prior status carried forward).</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>Stop-sale/recall inventory compensation; no change since baseline.</t>
+          <t>No House action since Rules re-assignment; still pending.</t>
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr">
         <is>
-          <t>No change from baseline.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
-          <t>https://www.cga.ct.gov/2026/ACT/PA/PDF/2026PA-00024-R00SB-00413-PA.PDF</t>
+          <t>https://www.ilga.gov/Legislation/BillStatus?DocNum=1939&amp;GAID=18&amp;DocTypeID=SB&amp;SessionID=114</t>
         </is>
       </c>
     </row>
@@ -43252,12 +43240,12 @@
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>RI</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>2026 SB 345 (Chapter 463; cross-filed HB 1214)</t>
+          <t>2026 S 2347 Sub A (P.L. 2026, ch. 180) / H 8213 Sub A (P.L. 2026, ch. 179)</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
@@ -43267,12 +43255,12 @@
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>Confirmed unchanged: approved 05/12/2026, effective 10/01/2026.</t>
+          <t>Confirmed unchanged: signed 06/22/2026, takes effect 10/01/2026. No lawsuit or injunction against the actual-time law found in a fresh search.</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>MVA hearing route for association disputes; no change since baseline.</t>
+          <t>Actual-technician-time warranty labor rule; no change since baseline.</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr">
@@ -43282,7 +43270,7 @@
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
-          <t>https://mgaleg.maryland.gov/mgawebsite/Legislation/Details/sb0345?ys=2026RS</t>
+          <t>https://webserver.rilegislature.gov/PublicLaws/law26/law26180.htm</t>
         </is>
       </c>
     </row>
@@ -43299,38 +43287,42 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_upcoming</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>SB 1182 (2025-26), PN 1866</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr"/>
+          <t>LB972 (2026), Sec. 70</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>Re-checked via palegis.us (bill page returned a server error on two attempts; corroborated via a bill-tracking aggregator citing the official record) and web search. Still 'in committee': House Commerce Committee, last action 07/01/2026. No House floor action found.</t>
+          <t>Confirmed unchanged: approved 04/14/2026, Sec. 70 operative 10/01/2026 per Sec. 84.</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>No committee action since referral; still pending.</t>
+          <t>RV scope carve-out; no change since baseline.</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
         <is>
-          <t>Watch only, unchanged.</t>
+          <t>No change from baseline.</t>
         </is>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
-          <t>https://www.palegis.us/legislation/bills/2025/sb1182</t>
+          <t>https://nebraskalegislature.gov/FloorDocs/109/PDF/Slip/LB972.pdf</t>
         </is>
       </c>
     </row>
@@ -43347,38 +43339,42 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_upcoming</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>CT</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>A8773 (Magnarelli) / S8360 (Cooney), 2025-26</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr"/>
+          <t>Public Act 26-24 (sSB 413), §§ 20-25</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>Re-checked on nyassembly.gov: A8773's last action is still 06/01/2026 (referred to Senate Rules); no further Senate action found.</t>
+          <t>Confirmed unchanged: signed 05/27/2026, §§ 20-25 effective 10/01/2026.</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>No Senate action since referral; still pending.</t>
+          <t>Stop-sale/recall inventory compensation; no change since baseline.</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
         <is>
-          <t>Watch only, unchanged.</t>
+          <t>No change from baseline.</t>
         </is>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
-          <t>https://nyassembly.gov/leg/?default_fld=&amp;leg_video=&amp;bn=A08773&amp;term=2025&amp;Summary=Y&amp;Actions=Y</t>
+          <t>https://www.cga.ct.gov/2026/ACT/PA/PDF/2026PA-00024-R00SB-00413-PA.PDF</t>
         </is>
       </c>
     </row>
@@ -43395,194 +43391,186 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_upcoming</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>MD</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>SB1939 (104th GA), as amended by Senate Floor Amendments 1-2</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr"/>
+          <t>2026 SB 345 (Chapter 463; cross-filed HB 1214)</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>Re-checked via web search (ilga.gov bill-status page returned a server error). Still pending in House Rules Committee since 03/20/2026; spring session adjourned 06/01/2026 with no further action.</t>
+          <t>Confirmed unchanged: approved 05/12/2026, effective 10/01/2026.</t>
         </is>
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>No House action since Rules re-assignment; still pending.</t>
+          <t>MVA hearing route for association disputes; no change since baseline.</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
         <is>
-          <t>Watch only, unchanged.</t>
+          <t>No change from baseline.</t>
         </is>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
-          <t>https://www.ilga.gov/Legislation/BillStatus?DocNum=1939&amp;GAID=18&amp;DocTypeID=SB&amp;SessionID=114</t>
+          <t>https://mgaleg.maryland.gov/mgawebsite/Legislation/Details/sb0345?ys=2026RS</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Baseline: 4 enacted changes take effect Oct 1, 2026 (RI, NE, CT, MD); 3 bills still pending (PA, NY, IL)</t>
+          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>enacted_upcoming</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>RI</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>2026 S 2347 Sub A (P.L. 2026, ch. 180) / H 8213 Sub A (P.L. 2026, ch. 179)</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>SB 1182 (2025-26), PN 1866</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr"/>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>Signed by Governor 06/22/2026 (S 2347 Sub A = Chapter 180; H 8213 Sub A = Chapter 179); takes effect 10/01/2026</t>
+          <t>Re-checked via palegis.us (bill page returned a server error on two attempts; corroborated via a bill-tracking aggregator citing the official record) and web search. Still 'in committee': House Commerce Committee, last action 07/01/2026. No House floor action found.</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>Amends R.I. Gen. Laws § 31-5.1-6 and related sections. Warranty labor is paid at the dealer's non-warranty labor rate multiplied by the ACTUAL time the technician worked.</t>
+          <t>No committee action since referral; still pending.</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr">
         <is>
-          <t>Already reflected: date selector switches RI to actual technician time and CPO Required on 10/1/2026.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>https://webserver.rilegislature.gov/PublicLaws/law26/law26180.htm</t>
+          <t>https://www.palegis.us/legislation/bills/2025/sb1182</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Baseline: 4 enacted changes take effect Oct 1, 2026 (RI, NE, CT, MD); 3 bills still pending (PA, NY, IL)</t>
+          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>enacted_upcoming</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>LB972 (2026), Sec. 70</t>
-        </is>
-      </c>
-      <c r="F29" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>A8773 (Magnarelli) / S8360 (Cooney), 2025-26</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr"/>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>Passed 48-1-0 on 04/10/2026; approved by Governor 04/14/2026. Sec. 84 makes Sec. 70 operative 10/01/2026.</t>
+          <t>Re-checked on nyassembly.gov: A8773's last action is still 06/01/2026 (referred to Senate Rules); no further Senate action found.</t>
         </is>
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>Sec. 70 adds § 60-1438(7): 'This section does not apply to recreational vehicles.' RVs move to the new Recreational Vehicle Industry Regulation Act. A word diff of Sec.</t>
+          <t>No Senate action since referral; still pending.</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
         <is>
-          <t>Scope only (RVs removed). No change to passenger-vehicle cells.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
-          <t>https://nebraskalegislature.gov/FloorDocs/109/PDF/Slip/LB972.pdf</t>
+          <t>https://nyassembly.gov/leg/?default_fld=&amp;leg_video=&amp;bn=A08773&amp;term=2025&amp;Summary=Y&amp;Actions=Y</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Baseline: 4 enacted changes take effect Oct 1, 2026 (RI, NE, CT, MD); 3 bills still pending (PA, NY, IL)</t>
+          <t>0 enacted changes, 3 pending bills unchanged, 0 law-data updates</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>enacted_upcoming</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>CT</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>Public Act 26-24 (sSB 413), §§ 20-25</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>SB1939 (104th GA), as amended by Senate Floor Amendments 1-2</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr"/>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>Signed by Governor 05/27/2026 (per the cga.ct.gov bill status page); §§ 20-25 effective 10/01/2026</t>
+          <t>Re-checked via web search (ilga.gov bill-status page returned a server error). Still pending in House Rules Committee since 03/20/2026; spring session adjourned 06/01/2026 with no further action.</t>
         </is>
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>New § 22 covers used vehicles in a dealer's inventory that are under a stop-sale or do-not-drive order for a federal safety or emissions recall.</t>
+          <t>No House action since Rules re-assignment; still pending.</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr">
         <is>
-          <t>Claim rules extend to stop-sale compensation claims. Labor rate and time cells unchanged.</t>
+          <t>Watch only, unchanged.</t>
         </is>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>https://www.cga.ct.gov/2026/ACT/PA/PDF/2026PA-00024-R00SB-00413-PA.PDF</t>
+          <t>https://www.ilga.gov/Legislation/BillStatus?DocNum=1939&amp;GAID=18&amp;DocTypeID=SB&amp;SessionID=114</t>
         </is>
       </c>
     </row>
@@ -43604,12 +43592,12 @@
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>RI</t>
         </is>
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>2026 SB 345 (Chapter 463; cross-filed HB 1214)</t>
+          <t>2026 S 2347 Sub A (P.L. 2026, ch. 180) / H 8213 Sub A (P.L. 2026, ch. 179)</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
@@ -43619,22 +43607,22 @@
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>Approved by Governor 05/12/2026 (Chapter 463); effective 10/01/2026</t>
+          <t>Signed by Governor 06/22/2026 (S 2347 Sub A = Chapter 180; H 8213 Sub A = Chapter 179); takes effect 10/01/2026</t>
         </is>
       </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t>Procedural, with an indirect effect on warranty. A dealer association or manufacturer association may request an MVA administrative hearing to resolve a dispute or to get an interpretation of the franchise law, which includes the § 15-212 warranty rules.</t>
+          <t>Amends R.I. Gen. Laws § 31-5.1-6 and related sections. Warranty labor is paid at the dealer's non-warranty labor rate multiplied by the ACTUAL time the technician worked.</t>
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr">
         <is>
-          <t>Procedural (association hearings). No change to § 15-212 cells.</t>
+          <t>Already reflected: date selector switches RI to actual technician time and CPO Required on 10/1/2026.</t>
         </is>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
-          <t>https://mgaleg.maryland.gov/mgawebsite/Legislation/Details/sb0345?ys=2026RS</t>
+          <t>https://webserver.rilegislature.gov/PublicLaws/law26/law26180.htm</t>
         </is>
       </c>
     </row>
@@ -43651,42 +43639,42 @@
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>enacted_recent</t>
+          <t>enacted_upcoming</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>2026 HB 648 (2026 Ky. Acts ch. 83), amending KRS 190.046</t>
+          <t>LB972 (2026), Sec. 70</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
-          <t>Signed by Governor 04/10/2026 (Acts Ch. 83); the official KRS 190.046 page shows 'Effective: July 15, 2026'</t>
+          <t>Passed 48-1-0 on 04/10/2026; approved by Governor 04/14/2026. Sec. 84 makes Sec. 70 operative 10/01/2026.</t>
         </is>
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>Rewrites KRS 190.046(2)(d) for vehicles in Class 7 and above (49 C.F.R. 565.15, heavy trucks) and makes component manufacturers liable. Parts are paid at acquisition cost plus a 30% gross margin.</t>
+          <t>Sec. 70 adds § 60-1438(7): 'This section does not apply to recreational vehicles.' RVs move to the new Recreational Vehicle Industry Regulation Act. A word diff of Sec.</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
         <is>
-          <t>Class 7+ heavy trucks only; noted in KY record. Light-duty cells unchanged.</t>
+          <t>Scope only (RVs removed). No change to passenger-vehicle cells.</t>
         </is>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
-          <t>https://apps.legislature.ky.gov/record/26rs/hb648.html</t>
+          <t>https://nebraskalegislature.gov/FloorDocs/109/PDF/Slip/LB972.pdf</t>
         </is>
       </c>
     </row>
@@ -43703,38 +43691,42 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_upcoming</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>CT</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>SB 1182 (2025-26), PN 1866</t>
-        </is>
-      </c>
-      <c r="F33" s="6" t="inlineStr"/>
+          <t>Public Act 26-24 (sSB 413), §§ 20-25</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
-          <t>Passed Senate 50-0 on 06/30/2026; referred to House COMMERCE Committee 07/01/2026; no House action since. The 2025-26 session ends 11/30/2026 and the bill dies if not enacted.</t>
+          <t>Signed by Governor 05/27/2026 (per the cga.ct.gov bill status page); §§ 20-25 effective 10/01/2026</t>
         </is>
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>Would amend Board of Vehicles Act § 307 to expressly cover extended warranty, CPO warranty, manufacturer-sponsored maintenance programs, parts-exchange programs and 'a service contract issued by a manufacturer or distributor or its common entity'.</t>
+          <t>New § 22 covers used vehicles in a dealer's inventory that are under a stop-sale or do-not-drive order for a federal safety or emissions recall.</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
         <is>
-          <t>Watch only. If enacted, PA service-contract and CPO cells would change.</t>
+          <t>Claim rules extend to stop-sale compensation claims. Labor rate and time cells unchanged.</t>
         </is>
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
-          <t>https://www.palegis.us/legislation/bills/2025/sb1182</t>
+          <t>https://www.cga.ct.gov/2026/ACT/PA/PDF/2026PA-00024-R00SB-00413-PA.PDF</t>
         </is>
       </c>
     </row>
@@ -43751,38 +43743,42 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_upcoming</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>MD</t>
         </is>
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>A8773 (Magnarelli) / S8360 (Cooney), 2025-26</t>
-        </is>
-      </c>
-      <c r="F34" s="6" t="inlineStr"/>
+          <t>2026 SB 345 (Chapter 463; cross-filed HB 1214)</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
-          <t>A8773 passed the Assembly 06/01/2026, went to the Senate and was referred to Senate RULES the same day. S8360 has been in Senate TRANSPORTATION since 01/07/2026. The Senate has not acted; the bills die 12/31/2026.</t>
+          <t>Approved by Governor 05/12/2026 (Chapter 463); effective 10/01/2026</t>
         </is>
       </c>
       <c r="H34" s="6" t="inlineStr">
         <is>
-          <t>Would amend VTL § 465 to cover affiliates and subsidiaries and to list 'extended service contract repairs', 'component part warranties' and 'any other franchisor compensated repairs'.</t>
+          <t>Procedural, with an indirect effect on warranty. A dealer association or manufacturer association may request an MVA administrative hearing to resolve a dispute or to get an interpretation of the franchise law, which includes the § 15-212 warranty rules.</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr">
         <is>
-          <t>Watch only. If enacted, NY paid-hours rules would add 1.5× and actual-time fallbacks.</t>
+          <t>Procedural (association hearings). No change to § 15-212 cells.</t>
         </is>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
-          <t>https://nyassembly.gov/leg/?default_fld=&amp;leg_video=&amp;bn=A08773&amp;term=2025&amp;Summary=Y&amp;Actions=Y</t>
+          <t>https://mgaleg.maryland.gov/mgawebsite/Legislation/Details/sb0345?ys=2026RS</t>
         </is>
       </c>
     </row>
@@ -43799,38 +43795,42 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>enacted_recent</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>KY</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>SB1939 (104th GA), as amended by Senate Floor Amendments 1-2</t>
-        </is>
-      </c>
-      <c r="F35" s="6" t="inlineStr"/>
+          <t>2026 HB 648 (2026 Ky. Acts ch. 83), amending KRS 190.046</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
-          <t>Passed Senate 55-0 on 04/10/2025. In the House it was re-assigned to the Rules Committee on 03/20/2026. It could move in the fall veto session (House session days Nov 17-19 and Dec 1-3, 2026) or the lame-duck session before the 104th GA ends in January 2027.</t>
+          <t>Signed by Governor 04/10/2026 (Acts Ch. 83); the official KRS 190.046 page shows 'Effective: July 15, 2026'</t>
         </is>
       </c>
       <c r="H35" s="6" t="inlineStr">
         <is>
-          <t>Mainly a direct-sales ban: an OEM not licensed to sell direct before 1/1/2022 may not own or operate a dealership or sell direct. It also amends 815 ILCS 710/6.</t>
+          <t>Rewrites KRS 190.046(2)(d) for vehicles in Class 7 and above (49 C.F.R. 565.15, heavy trucks) and makes component manufacturers liable. Parts are paid at acquisition cost plus a 30% gross margin.</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr">
         <is>
-          <t>Watch only. Mostly a direct-sales bill; parts-markup maintenance definition would change.</t>
+          <t>Class 7+ heavy trucks only; noted in KY record. Light-duty cells unchanged.</t>
         </is>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
-          <t>https://www.ilga.gov/Legislation/BillStatus?DocNum=1939&amp;GAID=18&amp;DocTypeID=SB&amp;SessionID=114</t>
+          <t>https://apps.legislature.ky.gov/record/26rs/hb648.html</t>
         </is>
       </c>
     </row>
@@ -43847,43 +43847,187 @@
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>dead_or_stalled</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>H4019 (194th General Court), 'An Act to ensure fair compensation for warranty service labor'</t>
+          <t>SB 1182 (2025-26), PN 1866</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr"/>
       <c r="G36" s="6" t="inlineStr">
         <is>
+          <t>Passed Senate 50-0 on 06/30/2026; referred to House COMMERCE Committee 07/01/2026; no House action since. The 2025-26 session ends 11/30/2026 and the bill dies if not enacted.</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr">
+        <is>
+          <t>Would amend Board of Vehicles Act § 307 to expressly cover extended warranty, CPO warranty, manufacturer-sponsored maintenance programs, parts-exchange programs and 'a service contract issued by a manufacturer or distributor or its common entity'.</t>
+        </is>
+      </c>
+      <c r="I36" s="6" t="inlineStr">
+        <is>
+          <t>Watch only. If enacted, PA service-contract and CPO cells would change.</t>
+        </is>
+      </c>
+      <c r="J36" s="6" t="inlineStr">
+        <is>
+          <t>https://www.palegis.us/legislation/bills/2025/sb1182</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>Baseline: 4 enacted changes take effect Oct 1, 2026 (RI, NE, CT, MD); 3 bills still pending (PA, NY, IL)</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="E37" s="6" t="inlineStr">
+        <is>
+          <t>A8773 (Magnarelli) / S8360 (Cooney), 2025-26</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="inlineStr"/>
+      <c r="G37" s="6" t="inlineStr">
+        <is>
+          <t>A8773 passed the Assembly 06/01/2026, went to the Senate and was referred to Senate RULES the same day. S8360 has been in Senate TRANSPORTATION since 01/07/2026. The Senate has not acted; the bills die 12/31/2026.</t>
+        </is>
+      </c>
+      <c r="H37" s="6" t="inlineStr">
+        <is>
+          <t>Would amend VTL § 465 to cover affiliates and subsidiaries and to list 'extended service contract repairs', 'component part warranties' and 'any other franchisor compensated repairs'.</t>
+        </is>
+      </c>
+      <c r="I37" s="6" t="inlineStr">
+        <is>
+          <t>Watch only. If enacted, NY paid-hours rules would add 1.5× and actual-time fallbacks.</t>
+        </is>
+      </c>
+      <c r="J37" s="6" t="inlineStr">
+        <is>
+          <t>https://nyassembly.gov/leg/?default_fld=&amp;leg_video=&amp;bn=A08773&amp;term=2025&amp;Summary=Y&amp;Actions=Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>Baseline: 4 enacted changes take effect Oct 1, 2026 (RI, NE, CT, MD); 3 bills still pending (PA, NY, IL)</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
+        <is>
+          <t>SB1939 (104th GA), as amended by Senate Floor Amendments 1-2</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="inlineStr"/>
+      <c r="G38" s="6" t="inlineStr">
+        <is>
+          <t>Passed Senate 55-0 on 04/10/2025. In the House it was re-assigned to the Rules Committee on 03/20/2026. It could move in the fall veto session (House session days Nov 17-19 and Dec 1-3, 2026) or the lame-duck session before the 104th GA ends in January 2027.</t>
+        </is>
+      </c>
+      <c r="H38" s="6" t="inlineStr">
+        <is>
+          <t>Mainly a direct-sales ban: an OEM not licensed to sell direct before 1/1/2022 may not own or operate a dealership or sell direct. It also amends 815 ILCS 710/6.</t>
+        </is>
+      </c>
+      <c r="I38" s="6" t="inlineStr">
+        <is>
+          <t>Watch only. Mostly a direct-sales bill; parts-markup maintenance definition would change.</t>
+        </is>
+      </c>
+      <c r="J38" s="6" t="inlineStr">
+        <is>
+          <t>https://www.ilga.gov/Legislation/BillStatus?DocNum=1939&amp;GAID=18&amp;DocTypeID=SB&amp;SessionID=114</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>Baseline: 4 enacted changes take effect Oct 1, 2026 (RI, NE, CT, MD); 3 bills still pending (PA, NY, IL)</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>dead_or_stalled</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="inlineStr">
+        <is>
+          <t>H4019 (194th General Court), 'An Act to ensure fair compensation for warranty service labor'</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="inlineStr"/>
+      <c r="G39" s="6" t="inlineStr">
+        <is>
           <t>Accompanied a study order (see H5320) on 04/02/2026, which means it is effectively dead. Formal sessions ended 07/31/2026.</t>
         </is>
       </c>
-      <c r="H36" s="6" t="inlineStr">
+      <c r="H39" s="6" t="inlineStr">
         <is>
           <t>Would have let dealers base warranty labor time on aftermarket or retail time guides. Hearing held 02/04/2026 before the Joint Committee on Consumer Protection and Professional Licensure.</t>
         </is>
       </c>
-      <c r="I36" s="6" t="inlineStr">
+      <c r="I39" s="6" t="inlineStr">
         <is>
           <t>Effectively dead (study order). No action.</t>
         </is>
       </c>
-      <c r="J36" s="6" t="inlineStr">
+      <c r="J39" s="6" t="inlineStr">
         <is>
           <t>https://malegislature.gov/Bills/194/H4019/BillHistory</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J36"/>
+  <autoFilter ref="A1:J39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>